<commit_message>
Finance : frais généraux divisés en ressources humaines et frais matériels (28/10/2026)
Budget mensuel : deux blocs avec sous-totaux. Nouvel onglet « Frais généraux
3 ans » : postes RH (effectif, salaire brut, mois payés, charges patronales)
et frais matériels pour les années 2 et 3, reliés au plan financier.
Besoin de financement à 3 ans : 309 726 € en hypothèses centrales.
Fiche des données manquantes mise à jour.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/2 FINANCE/PREVISIONS/2026 1027 Modèle - Budget, plan financier, prix et marges.xlsx
+++ b/2 FINANCE/PREVISIONS/2026 1027 Modèle - Budget, plan financier, prix et marges.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vians\Documents\Claude\Projects\HEC-GEMM-Groupe-7\2 FINANCE\PREVISIONS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A8DBC3A-486E-40A6-BFAF-35066D0D0378}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A68D3D2-8882-46A6-9CD1-8C34C95E3736}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{09426CC5-4BCC-48B7-8854-C5C8E2CE30D1}"/>
   </bookViews>
@@ -18,6 +18,7 @@
     <sheet name="Budget mensuel" sheetId="3" r:id="rId3"/>
     <sheet name="Prévu et réel" sheetId="4" r:id="rId4"/>
     <sheet name="Plan financier 3 ans" sheetId="5" r:id="rId5"/>
+    <sheet name="Frais généraux 3 ans" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="384" uniqueCount="228">
   <si>
     <t>Prévisions — budget, plan financier, prix et marges</t>
   </si>
@@ -429,12 +430,6 @@
     <t>Coûts directs</t>
   </si>
   <si>
-    <t>Charges fixes</t>
-  </si>
-  <si>
-    <t>Salaires et charges sociales</t>
-  </si>
-  <si>
     <t>Locaux et bureaux</t>
   </si>
   <si>
@@ -459,9 +454,6 @@
     <t>Autres charges (création de la société)</t>
   </si>
   <si>
-    <t>Total des charges fixes</t>
-  </si>
-  <si>
     <t>Résultat</t>
   </si>
   <si>
@@ -594,10 +586,148 @@
     <t>Année 1 : budget mensuel. H : 2 soirées A par mois en année 2, 3 en année 3 ; privatisations et contrats cadres de 2 à 4 soirées par an et par client (5 PRODUIT, offre ; 3 MARKETING, personas)</t>
   </si>
   <si>
-    <t>Année 1 : budget mensuel. H année 2 : un coordinateur au SMIC (F 1 867,02 € brut par mois au 01/06/2026, Éditions Tissot), marketing et honoraires. H année 3 : deux fondateurs rémunérés et un commercial</t>
-  </si>
-  <si>
     <t>H : site et identité visuelle, coffrets cadeaux numérotés, petit matériel de service</t>
+  </si>
+  <si>
+    <t>Frais généraux : 1. Ressources humaines</t>
+  </si>
+  <si>
+    <t>Rémunération des fondateurs (brut)</t>
+  </si>
+  <si>
+    <t>Salaires des employés (brut)</t>
+  </si>
+  <si>
+    <t>H : aucun salarié la première année</t>
+  </si>
+  <si>
+    <t>Charges sociales patronales</t>
+  </si>
+  <si>
+    <t>H : aucune rémunération versée, donc aucune charge</t>
+  </si>
+  <si>
+    <t>Stagiaires et indépendants</t>
+  </si>
+  <si>
+    <t>H : aucun la première année</t>
+  </si>
+  <si>
+    <t>Total ressources humaines</t>
+  </si>
+  <si>
+    <t>Frais généraux : 2. Frais matériels et de fonctionnement</t>
+  </si>
+  <si>
+    <t>Total frais matériels et de fonctionnement</t>
+  </si>
+  <si>
+    <t>Total des frais généraux</t>
+  </si>
+  <si>
+    <t>Frais généraux des années 2 et 3</t>
+  </si>
+  <si>
+    <t>Ressources humaines poste par poste, puis frais matériels et de fonctionnement. L'année 1 est détaillée mois par mois dans le budget mensuel.</t>
+  </si>
+  <si>
+    <t>Taux de charges sociales patronales</t>
+  </si>
+  <si>
+    <t>H : ordre de grandeur hors allègements (la réduction générale abaisse fortement ce taux près du SMIC) ; à faire confirmer par l'expert-comptable</t>
+  </si>
+  <si>
+    <t>1. Ressources humaines</t>
+  </si>
+  <si>
+    <t>Effectif</t>
+  </si>
+  <si>
+    <t>Salaire brut mensuel par personne (€)</t>
+  </si>
+  <si>
+    <t>Mois payés en année 2</t>
+  </si>
+  <si>
+    <t>Mois payés en année 3</t>
+  </si>
+  <si>
+    <t>Coût chargé année 2 (€)</t>
+  </si>
+  <si>
+    <t>Coût chargé année 3 (€)</t>
+  </si>
+  <si>
+    <t>Fondateurs (rémunération)</t>
+  </si>
+  <si>
+    <t>H : deux fondateurs rémunérés à partir de l'année 3 ; montant à décider par la Direction</t>
+  </si>
+  <si>
+    <t>Coordinateur ou coordinatrice d'événements</t>
+  </si>
+  <si>
+    <t>F SMIC brut de 1 867,02 € par mois au 01/06/2026 (Éditions Tissot, 26/05/2026) ; H : poste à temps plein dès l'année 2</t>
+  </si>
+  <si>
+    <t>Commercial ou commerciale entreprises</t>
+  </si>
+  <si>
+    <t>H : recrutement en année 3 pour les privatisations et les contrats cadres ; salaire à vérifier (grille de rémunération)</t>
+  </si>
+  <si>
+    <t>2. Frais matériels et de fonctionnement</t>
+  </si>
+  <si>
+    <t>Année 2 (€)</t>
+  </si>
+  <si>
+    <t>Année 3 (€)</t>
+  </si>
+  <si>
+    <t>H : travail à distance en année 2 ; coworking pour 3 postes à 300 € par mois en année 3</t>
+  </si>
+  <si>
+    <t>Logiciels et outils (site, billetterie, fichier clients)</t>
+  </si>
+  <si>
+    <t>H : montée en charge des outils</t>
+  </si>
+  <si>
+    <t>H : contenus, dîners de concierges, coffrets, relations presse</t>
+  </si>
+  <si>
+    <t>F 1 000 à 1 500 € par an au-delà de 1 M€ de chiffre d'affaires (Coover 2026) ; H : devis à obtenir</t>
+  </si>
+  <si>
+    <t>H : comptabilité, paie dès le premier salarié, contrats</t>
+  </si>
+  <si>
+    <t>H : repérage de lieux, rencontres de chefs</t>
+  </si>
+  <si>
+    <t>Autres frais</t>
+  </si>
+  <si>
+    <t>Frais de ressources humaines</t>
+  </si>
+  <si>
+    <t>Frais matériels et de fonctionnement</t>
+  </si>
+  <si>
+    <t>Année 1 : budget mensuel (ligne 21). Années 2 et 3 : onglet Frais généraux 3 ans, poste par poste</t>
+  </si>
+  <si>
+    <t>Année 1 : budget mensuel (ligne 31). Années 2 et 3 : onglet Frais généraux 3 ans</t>
+  </si>
+  <si>
+    <t>Somme des deux lignes précédentes</t>
+  </si>
+  <si>
+    <t>Frais généraux</t>
+  </si>
+  <si>
+    <t>Mis à jour le 28/10/2026 : frais généraux divisés en ressources humaines (fondateurs, salariés, charges sociales, stagiaires et indépendants) et frais matériels et de fonctionnement (locaux, outils, marketing, assurance, honoraires, banque, déplacements, autres). Année 1 : budget mensuel. Années 2 et 3 : onglet « Frais généraux 3 ans ».</t>
   </si>
 </sst>
 </file>
@@ -612,7 +742,7 @@
     <numFmt numFmtId="168" formatCode="mmm\ yyyy"/>
     <numFmt numFmtId="169" formatCode="#,##0.0;\-#,##0.0;&quot;-&quot;"/>
   </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -686,8 +816,38 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF008000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -715,6 +875,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9D9D9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -746,7 +912,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -828,11 +994,27 @@
     <xf numFmtId="167" fontId="9" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="167" fontId="10" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="8" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="169" fontId="8" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="12" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="13" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="167" fontId="8" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="7" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="14" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1168,7 +1350,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FBA644DB-8C71-4A8A-A457-0A27A3813ADD}">
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.6328125" style="1" customWidth="1"/>
@@ -1288,6 +1470,14 @@
       </c>
       <c r="B16" s="9" t="s">
         <v>27</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A17" s="8" t="s">
+        <v>226</v>
+      </c>
+      <c r="B17" s="9" t="s">
+        <v>227</v>
       </c>
     </row>
   </sheetData>
@@ -2391,7 +2581,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62A8117B-BF63-41C1-92C8-4FEDF95C8C14}">
-  <dimension ref="A1:P29"/>
+  <dimension ref="A1:P35"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="44.6328125" style="1" customWidth="1"/>
@@ -2553,7 +2743,7 @@
         <v>90</v>
       </c>
       <c r="P7" s="11" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
     </row>
     <row r="8" spans="1:16" ht="13" x14ac:dyDescent="0.3">
@@ -2604,7 +2794,7 @@
         <v>90</v>
       </c>
       <c r="P8" s="11" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
     </row>
     <row r="9" spans="1:16" ht="13" x14ac:dyDescent="0.3">
@@ -2655,7 +2845,7 @@
         <v>90</v>
       </c>
       <c r="P9" s="11" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
     </row>
     <row r="10" spans="1:16" ht="13" x14ac:dyDescent="0.3">
@@ -2706,7 +2896,7 @@
         <v>90</v>
       </c>
       <c r="P10" s="11" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
     </row>
     <row r="11" spans="1:16" ht="13" x14ac:dyDescent="0.3">
@@ -2959,7 +3149,7 @@
     </row>
     <row r="16" spans="1:16" ht="13" x14ac:dyDescent="0.3">
       <c r="A16" s="10" t="s">
-        <v>128</v>
+        <v>181</v>
       </c>
       <c r="B16" s="10"/>
       <c r="C16" s="10"/>
@@ -2979,10 +3169,10 @@
     </row>
     <row r="17" spans="1:16" ht="13" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
-        <v>129</v>
+        <v>182</v>
       </c>
       <c r="B17" s="17">
-        <f t="shared" ref="B17:B26" si="3">SUM(C17:N17)</f>
+        <f t="shared" ref="B17:B32" si="3">SUM(C17:N17)</f>
         <v>0</v>
       </c>
       <c r="C17" s="15">
@@ -3025,611 +3215,898 @@
         <v>90</v>
       </c>
       <c r="P17" s="11" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="18" spans="1:16" ht="13" x14ac:dyDescent="0.3">
-      <c r="A18" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="B18" s="17">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>183</v>
+      </c>
+      <c r="B18" s="42">
+        <f>SUM(C18:N18)</f>
+        <v>0</v>
+      </c>
+      <c r="C18" s="41">
+        <v>0</v>
+      </c>
+      <c r="D18" s="41">
+        <v>0</v>
+      </c>
+      <c r="E18" s="41">
+        <v>0</v>
+      </c>
+      <c r="F18" s="41">
+        <v>0</v>
+      </c>
+      <c r="G18" s="41">
+        <v>0</v>
+      </c>
+      <c r="H18" s="41">
+        <v>0</v>
+      </c>
+      <c r="I18" s="41">
+        <v>0</v>
+      </c>
+      <c r="J18" s="41">
+        <v>0</v>
+      </c>
+      <c r="K18" s="41">
+        <v>0</v>
+      </c>
+      <c r="L18" s="41">
+        <v>0</v>
+      </c>
+      <c r="M18" s="41">
+        <v>0</v>
+      </c>
+      <c r="N18" s="41">
+        <v>0</v>
+      </c>
+      <c r="O18" s="40" t="s">
+        <v>90</v>
+      </c>
+      <c r="P18" s="40" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="19" spans="1:16" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>185</v>
+      </c>
+      <c r="B19" s="42">
+        <f>SUM(C19:N19)</f>
+        <v>0</v>
+      </c>
+      <c r="C19" s="41">
+        <v>0</v>
+      </c>
+      <c r="D19" s="41">
+        <v>0</v>
+      </c>
+      <c r="E19" s="41">
+        <v>0</v>
+      </c>
+      <c r="F19" s="41">
+        <v>0</v>
+      </c>
+      <c r="G19" s="41">
+        <v>0</v>
+      </c>
+      <c r="H19" s="41">
+        <v>0</v>
+      </c>
+      <c r="I19" s="41">
+        <v>0</v>
+      </c>
+      <c r="J19" s="41">
+        <v>0</v>
+      </c>
+      <c r="K19" s="41">
+        <v>0</v>
+      </c>
+      <c r="L19" s="41">
+        <v>0</v>
+      </c>
+      <c r="M19" s="41">
+        <v>0</v>
+      </c>
+      <c r="N19" s="41">
+        <v>0</v>
+      </c>
+      <c r="O19" s="40" t="s">
+        <v>90</v>
+      </c>
+      <c r="P19" s="40" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>187</v>
+      </c>
+      <c r="B20" s="42">
+        <f>SUM(C20:N20)</f>
+        <v>0</v>
+      </c>
+      <c r="C20" s="41">
+        <v>0</v>
+      </c>
+      <c r="D20" s="41">
+        <v>0</v>
+      </c>
+      <c r="E20" s="41">
+        <v>0</v>
+      </c>
+      <c r="F20" s="41">
+        <v>0</v>
+      </c>
+      <c r="G20" s="41">
+        <v>0</v>
+      </c>
+      <c r="H20" s="41">
+        <v>0</v>
+      </c>
+      <c r="I20" s="41">
+        <v>0</v>
+      </c>
+      <c r="J20" s="41">
+        <v>0</v>
+      </c>
+      <c r="K20" s="41">
+        <v>0</v>
+      </c>
+      <c r="L20" s="41">
+        <v>0</v>
+      </c>
+      <c r="M20" s="41">
+        <v>0</v>
+      </c>
+      <c r="N20" s="41">
+        <v>0</v>
+      </c>
+      <c r="O20" s="40" t="s">
+        <v>90</v>
+      </c>
+      <c r="P20" s="40" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A21" s="44" t="s">
+        <v>189</v>
+      </c>
+      <c r="B21" s="42">
+        <f>SUM(C21:N21)</f>
+        <v>0</v>
+      </c>
+      <c r="C21" s="42">
+        <f t="shared" ref="C21:N21" si="4">SUM(C17:C20)</f>
+        <v>0</v>
+      </c>
+      <c r="D21" s="42">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="E21" s="42">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="F21" s="42">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="G21" s="42">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="H21" s="42">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="I21" s="42">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="J21" s="42">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="K21" s="42">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="L21" s="42">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="M21" s="42">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="N21" s="42">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A22" s="43" t="s">
+        <v>190</v>
+      </c>
+      <c r="B22" s="43"/>
+      <c r="C22" s="43"/>
+      <c r="D22" s="43"/>
+      <c r="E22" s="43"/>
+      <c r="F22" s="43"/>
+      <c r="G22" s="43"/>
+      <c r="H22" s="43"/>
+      <c r="I22" s="43"/>
+      <c r="J22" s="43"/>
+      <c r="K22" s="43"/>
+      <c r="L22" s="43"/>
+      <c r="M22" s="43"/>
+      <c r="N22" s="43"/>
+      <c r="O22" s="43"/>
+      <c r="P22" s="43"/>
+    </row>
+    <row r="23" spans="1:16" ht="13" x14ac:dyDescent="0.3">
+      <c r="A23" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="B23" s="17">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="C18" s="15">
-        <v>0</v>
-      </c>
-      <c r="D18" s="15">
-        <v>0</v>
-      </c>
-      <c r="E18" s="15">
-        <v>0</v>
-      </c>
-      <c r="F18" s="15">
-        <v>0</v>
-      </c>
-      <c r="G18" s="15">
-        <v>0</v>
-      </c>
-      <c r="H18" s="15">
-        <v>0</v>
-      </c>
-      <c r="I18" s="15">
-        <v>0</v>
-      </c>
-      <c r="J18" s="15">
-        <v>0</v>
-      </c>
-      <c r="K18" s="15">
-        <v>0</v>
-      </c>
-      <c r="L18" s="15">
-        <v>0</v>
-      </c>
-      <c r="M18" s="15">
-        <v>0</v>
-      </c>
-      <c r="N18" s="15">
-        <v>0</v>
-      </c>
-      <c r="O18" s="11" t="s">
+      <c r="C23" s="15">
+        <v>0</v>
+      </c>
+      <c r="D23" s="15">
+        <v>0</v>
+      </c>
+      <c r="E23" s="15">
+        <v>0</v>
+      </c>
+      <c r="F23" s="15">
+        <v>0</v>
+      </c>
+      <c r="G23" s="15">
+        <v>0</v>
+      </c>
+      <c r="H23" s="15">
+        <v>0</v>
+      </c>
+      <c r="I23" s="15">
+        <v>0</v>
+      </c>
+      <c r="J23" s="15">
+        <v>0</v>
+      </c>
+      <c r="K23" s="15">
+        <v>0</v>
+      </c>
+      <c r="L23" s="15">
+        <v>0</v>
+      </c>
+      <c r="M23" s="15">
+        <v>0</v>
+      </c>
+      <c r="N23" s="15">
+        <v>0</v>
+      </c>
+      <c r="O23" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="P18" s="11" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="19" spans="1:16" ht="13" x14ac:dyDescent="0.3">
-      <c r="A19" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="B19" s="17">
+      <c r="P23" s="11" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16" ht="13" x14ac:dyDescent="0.3">
+      <c r="A24" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="B24" s="17">
         <f t="shared" si="3"/>
         <v>960</v>
       </c>
-      <c r="C19" s="15">
+      <c r="C24" s="15">
         <v>80</v>
       </c>
-      <c r="D19" s="15">
+      <c r="D24" s="15">
         <v>80</v>
       </c>
-      <c r="E19" s="15">
+      <c r="E24" s="15">
         <v>80</v>
       </c>
-      <c r="F19" s="15">
+      <c r="F24" s="15">
         <v>80</v>
       </c>
-      <c r="G19" s="15">
+      <c r="G24" s="15">
         <v>80</v>
       </c>
-      <c r="H19" s="15">
+      <c r="H24" s="15">
         <v>80</v>
       </c>
-      <c r="I19" s="15">
+      <c r="I24" s="15">
         <v>80</v>
       </c>
-      <c r="J19" s="15">
+      <c r="J24" s="15">
         <v>80</v>
       </c>
-      <c r="K19" s="15">
+      <c r="K24" s="15">
         <v>80</v>
       </c>
-      <c r="L19" s="15">
+      <c r="L24" s="15">
         <v>80</v>
       </c>
-      <c r="M19" s="15">
+      <c r="M24" s="15">
         <v>80</v>
       </c>
-      <c r="N19" s="15">
+      <c r="N24" s="15">
         <v>80</v>
       </c>
-      <c r="O19" s="11" t="s">
+      <c r="O24" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="P19" s="11" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="20" spans="1:16" ht="13" x14ac:dyDescent="0.3">
-      <c r="A20" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="B20" s="17">
+      <c r="P24" s="11" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="25" spans="1:16" ht="13" x14ac:dyDescent="0.3">
+      <c r="A25" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="B25" s="17">
         <f t="shared" si="3"/>
         <v>7200</v>
       </c>
-      <c r="C20" s="15">
+      <c r="C25" s="15">
         <v>300</v>
       </c>
-      <c r="D20" s="15">
+      <c r="D25" s="15">
         <v>1500</v>
       </c>
-      <c r="E20" s="15">
+      <c r="E25" s="15">
         <v>1500</v>
       </c>
-      <c r="F20" s="15">
+      <c r="F25" s="15">
         <v>1500</v>
       </c>
-      <c r="G20" s="15">
+      <c r="G25" s="15">
         <v>300</v>
       </c>
-      <c r="H20" s="15">
+      <c r="H25" s="15">
         <v>300</v>
       </c>
-      <c r="I20" s="15">
+      <c r="I25" s="15">
         <v>300</v>
       </c>
-      <c r="J20" s="15">
+      <c r="J25" s="15">
         <v>300</v>
       </c>
-      <c r="K20" s="15">
+      <c r="K25" s="15">
         <v>300</v>
       </c>
-      <c r="L20" s="15">
+      <c r="L25" s="15">
         <v>300</v>
       </c>
-      <c r="M20" s="15">
+      <c r="M25" s="15">
         <v>300</v>
       </c>
-      <c r="N20" s="15">
+      <c r="N25" s="15">
         <v>300</v>
       </c>
-      <c r="O20" s="11" t="s">
+      <c r="O25" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="P20" s="11" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="21" spans="1:16" ht="13" x14ac:dyDescent="0.3">
-      <c r="A21" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B21" s="17">
+      <c r="P25" s="11" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="26" spans="1:16" ht="13" x14ac:dyDescent="0.3">
+      <c r="A26" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="B26" s="17">
         <f t="shared" si="3"/>
         <v>600</v>
       </c>
-      <c r="C21" s="15">
+      <c r="C26" s="15">
         <v>50</v>
       </c>
-      <c r="D21" s="15">
+      <c r="D26" s="15">
         <v>50</v>
       </c>
-      <c r="E21" s="15">
+      <c r="E26" s="15">
         <v>50</v>
       </c>
-      <c r="F21" s="15">
+      <c r="F26" s="15">
         <v>50</v>
       </c>
-      <c r="G21" s="15">
+      <c r="G26" s="15">
         <v>50</v>
       </c>
-      <c r="H21" s="15">
+      <c r="H26" s="15">
         <v>50</v>
       </c>
-      <c r="I21" s="15">
+      <c r="I26" s="15">
         <v>50</v>
       </c>
-      <c r="J21" s="15">
+      <c r="J26" s="15">
         <v>50</v>
       </c>
-      <c r="K21" s="15">
+      <c r="K26" s="15">
         <v>50</v>
       </c>
-      <c r="L21" s="15">
+      <c r="L26" s="15">
         <v>50</v>
       </c>
-      <c r="M21" s="15">
+      <c r="M26" s="15">
         <v>50</v>
       </c>
-      <c r="N21" s="15">
+      <c r="N26" s="15">
         <v>50</v>
       </c>
-      <c r="O21" s="11" t="s">
+      <c r="O26" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="P21" s="11" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="22" spans="1:16" ht="13" x14ac:dyDescent="0.3">
-      <c r="A22" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="B22" s="17">
+      <c r="P26" s="11" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="27" spans="1:16" ht="13" x14ac:dyDescent="0.3">
+      <c r="A27" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="B27" s="17">
         <f t="shared" si="3"/>
         <v>2700</v>
       </c>
-      <c r="C22" s="15">
+      <c r="C27" s="15">
         <v>1600</v>
       </c>
-      <c r="D22" s="15">
+      <c r="D27" s="15">
         <v>100</v>
       </c>
-      <c r="E22" s="15">
+      <c r="E27" s="15">
         <v>100</v>
       </c>
-      <c r="F22" s="15">
+      <c r="F27" s="15">
         <v>100</v>
       </c>
-      <c r="G22" s="15">
+      <c r="G27" s="15">
         <v>100</v>
       </c>
-      <c r="H22" s="15">
+      <c r="H27" s="15">
         <v>100</v>
       </c>
-      <c r="I22" s="15">
+      <c r="I27" s="15">
         <v>100</v>
       </c>
-      <c r="J22" s="15">
+      <c r="J27" s="15">
         <v>100</v>
       </c>
-      <c r="K22" s="15">
+      <c r="K27" s="15">
         <v>100</v>
       </c>
-      <c r="L22" s="15">
+      <c r="L27" s="15">
         <v>100</v>
       </c>
-      <c r="M22" s="15">
+      <c r="M27" s="15">
         <v>100</v>
       </c>
-      <c r="N22" s="15">
+      <c r="N27" s="15">
         <v>100</v>
       </c>
-      <c r="O22" s="11" t="s">
+      <c r="O27" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="P22" s="11" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="23" spans="1:16" ht="13" x14ac:dyDescent="0.3">
-      <c r="A23" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="B23" s="17">
+      <c r="P27" s="11" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="28" spans="1:16" ht="13" x14ac:dyDescent="0.3">
+      <c r="A28" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B28" s="17">
         <f t="shared" si="3"/>
         <v>360</v>
       </c>
-      <c r="C23" s="15">
+      <c r="C28" s="15">
         <v>30</v>
       </c>
-      <c r="D23" s="15">
+      <c r="D28" s="15">
         <v>30</v>
       </c>
-      <c r="E23" s="15">
+      <c r="E28" s="15">
         <v>30</v>
       </c>
-      <c r="F23" s="15">
+      <c r="F28" s="15">
         <v>30</v>
       </c>
-      <c r="G23" s="15">
+      <c r="G28" s="15">
         <v>30</v>
       </c>
-      <c r="H23" s="15">
+      <c r="H28" s="15">
         <v>30</v>
       </c>
-      <c r="I23" s="15">
+      <c r="I28" s="15">
         <v>30</v>
       </c>
-      <c r="J23" s="15">
+      <c r="J28" s="15">
         <v>30</v>
       </c>
-      <c r="K23" s="15">
+      <c r="K28" s="15">
         <v>30</v>
       </c>
-      <c r="L23" s="15">
+      <c r="L28" s="15">
         <v>30</v>
       </c>
-      <c r="M23" s="15">
+      <c r="M28" s="15">
         <v>30</v>
       </c>
-      <c r="N23" s="15">
+      <c r="N28" s="15">
         <v>30</v>
       </c>
-      <c r="O23" s="11" t="s">
+      <c r="O28" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="P23" s="11" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="24" spans="1:16" ht="13" x14ac:dyDescent="0.3">
-      <c r="A24" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="B24" s="17">
+      <c r="P28" s="11" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="29" spans="1:16" ht="13" x14ac:dyDescent="0.3">
+      <c r="A29" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="B29" s="17">
         <f t="shared" si="3"/>
         <v>600</v>
       </c>
-      <c r="C24" s="15">
+      <c r="C29" s="15">
         <v>50</v>
       </c>
-      <c r="D24" s="15">
+      <c r="D29" s="15">
         <v>50</v>
       </c>
-      <c r="E24" s="15">
+      <c r="E29" s="15">
         <v>50</v>
       </c>
-      <c r="F24" s="15">
+      <c r="F29" s="15">
         <v>50</v>
       </c>
-      <c r="G24" s="15">
+      <c r="G29" s="15">
         <v>50</v>
       </c>
-      <c r="H24" s="15">
+      <c r="H29" s="15">
         <v>50</v>
       </c>
-      <c r="I24" s="15">
+      <c r="I29" s="15">
         <v>50</v>
       </c>
-      <c r="J24" s="15">
+      <c r="J29" s="15">
         <v>50</v>
       </c>
-      <c r="K24" s="15">
+      <c r="K29" s="15">
         <v>50</v>
       </c>
-      <c r="L24" s="15">
+      <c r="L29" s="15">
         <v>50</v>
       </c>
-      <c r="M24" s="15">
+      <c r="M29" s="15">
         <v>50</v>
       </c>
-      <c r="N24" s="15">
+      <c r="N29" s="15">
         <v>50</v>
       </c>
-      <c r="O24" s="11" t="s">
+      <c r="O29" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="P24" s="11" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="25" spans="1:16" ht="13" x14ac:dyDescent="0.3">
-      <c r="A25" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="B25" s="17">
+      <c r="P29" s="11" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="30" spans="1:16" ht="13" x14ac:dyDescent="0.3">
+      <c r="A30" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="B30" s="17">
         <f t="shared" si="3"/>
         <v>252</v>
       </c>
-      <c r="C25" s="15">
+      <c r="C30" s="15">
         <v>252</v>
       </c>
-      <c r="D25" s="15">
-        <v>0</v>
-      </c>
-      <c r="E25" s="15">
-        <v>0</v>
-      </c>
-      <c r="F25" s="15">
-        <v>0</v>
-      </c>
-      <c r="G25" s="15">
-        <v>0</v>
-      </c>
-      <c r="H25" s="15">
-        <v>0</v>
-      </c>
-      <c r="I25" s="15">
-        <v>0</v>
-      </c>
-      <c r="J25" s="15">
-        <v>0</v>
-      </c>
-      <c r="K25" s="15">
-        <v>0</v>
-      </c>
-      <c r="L25" s="15">
-        <v>0</v>
-      </c>
-      <c r="M25" s="15">
-        <v>0</v>
-      </c>
-      <c r="N25" s="15">
-        <v>0</v>
-      </c>
-      <c r="O25" s="11" t="s">
-        <v>152</v>
-      </c>
-      <c r="P25" s="11" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="26" spans="1:16" ht="13" x14ac:dyDescent="0.3">
-      <c r="A26" s="2" t="s">
+      <c r="D30" s="15">
+        <v>0</v>
+      </c>
+      <c r="E30" s="15">
+        <v>0</v>
+      </c>
+      <c r="F30" s="15">
+        <v>0</v>
+      </c>
+      <c r="G30" s="15">
+        <v>0</v>
+      </c>
+      <c r="H30" s="15">
+        <v>0</v>
+      </c>
+      <c r="I30" s="15">
+        <v>0</v>
+      </c>
+      <c r="J30" s="15">
+        <v>0</v>
+      </c>
+      <c r="K30" s="15">
+        <v>0</v>
+      </c>
+      <c r="L30" s="15">
+        <v>0</v>
+      </c>
+      <c r="M30" s="15">
+        <v>0</v>
+      </c>
+      <c r="N30" s="15">
+        <v>0</v>
+      </c>
+      <c r="O30" s="11" t="s">
+        <v>149</v>
+      </c>
+      <c r="P30" s="11" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="31" spans="1:16" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A31" s="44" t="s">
+        <v>191</v>
+      </c>
+      <c r="B31" s="42">
+        <f>SUM(C31:N31)</f>
+        <v>12672</v>
+      </c>
+      <c r="C31" s="42">
+        <f t="shared" ref="C31:N31" si="5">SUM(C23:C30)</f>
+        <v>2362</v>
+      </c>
+      <c r="D31" s="42">
+        <f t="shared" si="5"/>
+        <v>1810</v>
+      </c>
+      <c r="E31" s="42">
+        <f t="shared" si="5"/>
+        <v>1810</v>
+      </c>
+      <c r="F31" s="42">
+        <f t="shared" si="5"/>
+        <v>1810</v>
+      </c>
+      <c r="G31" s="42">
+        <f t="shared" si="5"/>
+        <v>610</v>
+      </c>
+      <c r="H31" s="42">
+        <f t="shared" si="5"/>
+        <v>610</v>
+      </c>
+      <c r="I31" s="42">
+        <f t="shared" si="5"/>
+        <v>610</v>
+      </c>
+      <c r="J31" s="42">
+        <f t="shared" si="5"/>
+        <v>610</v>
+      </c>
+      <c r="K31" s="42">
+        <f t="shared" si="5"/>
+        <v>610</v>
+      </c>
+      <c r="L31" s="42">
+        <f t="shared" si="5"/>
+        <v>610</v>
+      </c>
+      <c r="M31" s="42">
+        <f t="shared" si="5"/>
+        <v>610</v>
+      </c>
+      <c r="N31" s="42">
+        <f t="shared" si="5"/>
+        <v>610</v>
+      </c>
+    </row>
+    <row r="32" spans="1:16" ht="13" x14ac:dyDescent="0.3">
+      <c r="A32" s="45" t="s">
+        <v>192</v>
+      </c>
+      <c r="B32" s="46">
+        <f>SUM(C32:N32)</f>
+        <v>12672</v>
+      </c>
+      <c r="C32" s="46">
+        <f t="shared" ref="C32:N32" si="6">C21+C31</f>
+        <v>2362</v>
+      </c>
+      <c r="D32" s="46">
+        <f t="shared" si="6"/>
+        <v>1810</v>
+      </c>
+      <c r="E32" s="46">
+        <f t="shared" si="6"/>
+        <v>1810</v>
+      </c>
+      <c r="F32" s="46">
+        <f t="shared" si="6"/>
+        <v>1810</v>
+      </c>
+      <c r="G32" s="46">
+        <f t="shared" si="6"/>
+        <v>610</v>
+      </c>
+      <c r="H32" s="46">
+        <f t="shared" si="6"/>
+        <v>610</v>
+      </c>
+      <c r="I32" s="46">
+        <f t="shared" si="6"/>
+        <v>610</v>
+      </c>
+      <c r="J32" s="46">
+        <f t="shared" si="6"/>
+        <v>610</v>
+      </c>
+      <c r="K32" s="46">
+        <f t="shared" si="6"/>
+        <v>610</v>
+      </c>
+      <c r="L32" s="46">
+        <f t="shared" si="6"/>
+        <v>610</v>
+      </c>
+      <c r="M32" s="46">
+        <f t="shared" si="6"/>
+        <v>610</v>
+      </c>
+      <c r="N32" s="46">
+        <f t="shared" si="6"/>
+        <v>610</v>
+      </c>
+    </row>
+    <row r="33" spans="1:16" ht="13" x14ac:dyDescent="0.3">
+      <c r="A33" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="B33" s="10"/>
+      <c r="C33" s="10"/>
+      <c r="D33" s="10"/>
+      <c r="E33" s="10"/>
+      <c r="F33" s="10"/>
+      <c r="G33" s="10"/>
+      <c r="H33" s="10"/>
+      <c r="I33" s="10"/>
+      <c r="J33" s="10"/>
+      <c r="K33" s="10"/>
+      <c r="L33" s="10"/>
+      <c r="M33" s="10"/>
+      <c r="N33" s="10"/>
+      <c r="O33" s="10"/>
+      <c r="P33" s="10"/>
+    </row>
+    <row r="34" spans="1:16" ht="13" x14ac:dyDescent="0.3">
+      <c r="A34" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B34" s="17">
+        <f>SUM(C34:N34)</f>
+        <v>-16255.821428571435</v>
+      </c>
+      <c r="C34" s="17">
+        <f t="shared" ref="C34:N34" si="7">C15-C32</f>
+        <v>-2362</v>
+      </c>
+      <c r="D34" s="17">
+        <f t="shared" si="7"/>
+        <v>-1810</v>
+      </c>
+      <c r="E34" s="17">
+        <f t="shared" si="7"/>
+        <v>-2664.0714285714294</v>
+      </c>
+      <c r="F34" s="17">
+        <f t="shared" si="7"/>
+        <v>-4162.2857142857156</v>
+      </c>
+      <c r="G34" s="17">
+        <f t="shared" si="7"/>
+        <v>-1473.2500000000009</v>
+      </c>
+      <c r="H34" s="17">
+        <f t="shared" si="7"/>
+        <v>-231.92857142857247</v>
+      </c>
+      <c r="I34" s="17">
+        <f t="shared" si="7"/>
+        <v>-1730.1428571428587</v>
+      </c>
+      <c r="J34" s="17">
+        <f t="shared" si="7"/>
+        <v>-241.10714285714312</v>
+      </c>
+      <c r="K34" s="17">
+        <f t="shared" si="7"/>
+        <v>-1464.0714285714294</v>
+      </c>
+      <c r="L34" s="17">
+        <f t="shared" si="7"/>
+        <v>-610</v>
+      </c>
+      <c r="M34" s="17">
+        <f t="shared" si="7"/>
+        <v>-498</v>
+      </c>
+      <c r="N34" s="17">
+        <f t="shared" si="7"/>
+        <v>991.03571428571377</v>
+      </c>
+    </row>
+    <row r="35" spans="1:16" ht="13" x14ac:dyDescent="0.3">
+      <c r="A35" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="B26" s="17">
-        <f t="shared" si="3"/>
-        <v>12672</v>
-      </c>
-      <c r="C26" s="17">
-        <f t="shared" ref="C26:N26" si="4">SUM(C17:C25)</f>
-        <v>2362</v>
-      </c>
-      <c r="D26" s="17">
-        <f t="shared" si="4"/>
-        <v>1810</v>
-      </c>
-      <c r="E26" s="17">
-        <f t="shared" si="4"/>
-        <v>1810</v>
-      </c>
-      <c r="F26" s="17">
-        <f t="shared" si="4"/>
-        <v>1810</v>
-      </c>
-      <c r="G26" s="17">
-        <f t="shared" si="4"/>
-        <v>610</v>
-      </c>
-      <c r="H26" s="17">
-        <f t="shared" si="4"/>
-        <v>610</v>
-      </c>
-      <c r="I26" s="17">
-        <f t="shared" si="4"/>
-        <v>610</v>
-      </c>
-      <c r="J26" s="17">
-        <f t="shared" si="4"/>
-        <v>610</v>
-      </c>
-      <c r="K26" s="17">
-        <f t="shared" si="4"/>
-        <v>610</v>
-      </c>
-      <c r="L26" s="17">
-        <f t="shared" si="4"/>
-        <v>610</v>
-      </c>
-      <c r="M26" s="17">
-        <f t="shared" si="4"/>
-        <v>610</v>
-      </c>
-      <c r="N26" s="17">
-        <f t="shared" si="4"/>
-        <v>610</v>
-      </c>
-    </row>
-    <row r="27" spans="1:16" ht="13" x14ac:dyDescent="0.3">
-      <c r="A27" s="10" t="s">
-        <v>139</v>
-      </c>
-      <c r="B27" s="10"/>
-      <c r="C27" s="10"/>
-      <c r="D27" s="10"/>
-      <c r="E27" s="10"/>
-      <c r="F27" s="10"/>
-      <c r="G27" s="10"/>
-      <c r="H27" s="10"/>
-      <c r="I27" s="10"/>
-      <c r="J27" s="10"/>
-      <c r="K27" s="10"/>
-      <c r="L27" s="10"/>
-      <c r="M27" s="10"/>
-      <c r="N27" s="10"/>
-      <c r="O27" s="10"/>
-      <c r="P27" s="10"/>
-    </row>
-    <row r="28" spans="1:16" ht="13" x14ac:dyDescent="0.3">
-      <c r="A28" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="B28" s="17">
-        <f>SUM(C28:N28)</f>
+      <c r="B35" s="17">
+        <f>N35</f>
         <v>-16255.821428571435</v>
       </c>
-      <c r="C28" s="17">
-        <f t="shared" ref="C28:N28" si="5">C15-C26</f>
+      <c r="C35" s="17">
+        <f>C34</f>
         <v>-2362</v>
       </c>
-      <c r="D28" s="17">
-        <f t="shared" si="5"/>
-        <v>-1810</v>
-      </c>
-      <c r="E28" s="17">
-        <f t="shared" si="5"/>
-        <v>-2664.0714285714294</v>
-      </c>
-      <c r="F28" s="17">
-        <f t="shared" si="5"/>
-        <v>-4162.2857142857156</v>
-      </c>
-      <c r="G28" s="17">
-        <f t="shared" si="5"/>
-        <v>-1473.2500000000009</v>
-      </c>
-      <c r="H28" s="17">
-        <f t="shared" si="5"/>
-        <v>-231.92857142857247</v>
-      </c>
-      <c r="I28" s="17">
-        <f t="shared" si="5"/>
-        <v>-1730.1428571428587</v>
-      </c>
-      <c r="J28" s="17">
-        <f t="shared" si="5"/>
-        <v>-241.10714285714312</v>
-      </c>
-      <c r="K28" s="17">
-        <f t="shared" si="5"/>
-        <v>-1464.0714285714294</v>
-      </c>
-      <c r="L28" s="17">
-        <f t="shared" si="5"/>
-        <v>-610</v>
-      </c>
-      <c r="M28" s="17">
-        <f t="shared" si="5"/>
-        <v>-498</v>
-      </c>
-      <c r="N28" s="17">
-        <f t="shared" si="5"/>
-        <v>991.03571428571377</v>
-      </c>
-    </row>
-    <row r="29" spans="1:16" ht="13" x14ac:dyDescent="0.3">
-      <c r="A29" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="B29" s="17">
-        <f>N29</f>
-        <v>-16255.821428571435</v>
-      </c>
-      <c r="C29" s="17">
-        <f>C28</f>
-        <v>-2362</v>
-      </c>
-      <c r="D29" s="17">
-        <f t="shared" ref="D29:N29" si="6">C29+D28</f>
+      <c r="D35" s="17">
+        <f t="shared" ref="D35:N35" si="8">C35+D34</f>
         <v>-4172</v>
       </c>
-      <c r="E29" s="17">
-        <f t="shared" si="6"/>
+      <c r="E35" s="17">
+        <f t="shared" si="8"/>
         <v>-6836.0714285714294</v>
       </c>
-      <c r="F29" s="17">
-        <f t="shared" si="6"/>
+      <c r="F35" s="17">
+        <f t="shared" si="8"/>
         <v>-10998.357142857145</v>
       </c>
-      <c r="G29" s="17">
-        <f t="shared" si="6"/>
+      <c r="G35" s="17">
+        <f t="shared" si="8"/>
         <v>-12471.607142857145</v>
       </c>
-      <c r="H29" s="17">
-        <f t="shared" si="6"/>
+      <c r="H35" s="17">
+        <f t="shared" si="8"/>
         <v>-12703.535714285717</v>
       </c>
-      <c r="I29" s="17">
-        <f t="shared" si="6"/>
+      <c r="I35" s="17">
+        <f t="shared" si="8"/>
         <v>-14433.678571428576</v>
       </c>
-      <c r="J29" s="17">
-        <f t="shared" si="6"/>
+      <c r="J35" s="17">
+        <f t="shared" si="8"/>
         <v>-14674.785714285719</v>
       </c>
-      <c r="K29" s="17">
-        <f t="shared" si="6"/>
+      <c r="K35" s="17">
+        <f t="shared" si="8"/>
         <v>-16138.857142857149</v>
       </c>
-      <c r="L29" s="17">
-        <f t="shared" si="6"/>
+      <c r="L35" s="17">
+        <f t="shared" si="8"/>
         <v>-16748.857142857149</v>
       </c>
-      <c r="M29" s="17">
-        <f t="shared" si="6"/>
+      <c r="M35" s="17">
+        <f t="shared" si="8"/>
         <v>-17246.857142857149</v>
       </c>
-      <c r="N29" s="17">
-        <f t="shared" si="6"/>
+      <c r="N35" s="17">
+        <f t="shared" si="8"/>
         <v>-16255.821428571435</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O7:O25" xr:uid="{31226B02-E24A-4164-8201-A9757FEFEA83}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O7:O16 O31 O17:O30" xr:uid="{31226B02-E24A-4164-8201-A9757FEFEA83}">
       <formula1>"F,I,P,H"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3650,17 +4127,17 @@
   <sheetData>
     <row r="1" spans="1:14" ht="18" x14ac:dyDescent="0.4">
       <c r="A1" s="3" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
     </row>
     <row r="2" spans="1:14" ht="13" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
     </row>
     <row r="5" spans="1:14" ht="13" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>118</v>
@@ -3716,7 +4193,7 @@
     </row>
     <row r="6" spans="1:14" ht="13" x14ac:dyDescent="0.3">
       <c r="A6" s="10" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="B6" s="10"/>
       <c r="C6" s="10"/>
@@ -3734,7 +4211,7 @@
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="B7" s="13">
         <f>SUM(C7:N7)</f>
@@ -3791,7 +4268,7 @@
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="B8" s="13">
         <f>SUM(C8:N8)</f>
@@ -3812,7 +4289,7 @@
     </row>
     <row r="9" spans="1:14" ht="13" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="B9" s="14">
         <f>SUM(C9:N9)</f>
@@ -3887,7 +4364,7 @@
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="B12" s="16">
         <f>SUM(C12:N12)</f>
@@ -3944,7 +4421,7 @@
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="B13" s="16">
         <f>SUM(C13:N13)</f>
@@ -3965,7 +4442,7 @@
     </row>
     <row r="14" spans="1:14" ht="13" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="B14" s="17">
         <f>SUM(C14:N14)</f>
@@ -4022,7 +4499,7 @@
     </row>
     <row r="16" spans="1:14" ht="13" x14ac:dyDescent="0.3">
       <c r="A16" s="10" t="s">
-        <v>138</v>
+        <v>192</v>
       </c>
       <c r="B16" s="10"/>
       <c r="C16" s="10"/>
@@ -4040,64 +4517,64 @@
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="B17" s="16">
         <f>SUM(C17:N17)</f>
         <v>12672</v>
       </c>
       <c r="C17" s="36">
-        <f>'Budget mensuel'!C26</f>
+        <f>'Budget mensuel'!C32</f>
         <v>2362</v>
       </c>
       <c r="D17" s="36">
-        <f>'Budget mensuel'!D26</f>
+        <f>'Budget mensuel'!D32</f>
         <v>1810</v>
       </c>
       <c r="E17" s="36">
-        <f>'Budget mensuel'!E26</f>
+        <f>'Budget mensuel'!E32</f>
         <v>1810</v>
       </c>
       <c r="F17" s="36">
-        <f>'Budget mensuel'!F26</f>
+        <f>'Budget mensuel'!F32</f>
         <v>1810</v>
       </c>
       <c r="G17" s="36">
-        <f>'Budget mensuel'!G26</f>
+        <f>'Budget mensuel'!G32</f>
         <v>610</v>
       </c>
       <c r="H17" s="36">
-        <f>'Budget mensuel'!H26</f>
+        <f>'Budget mensuel'!H32</f>
         <v>610</v>
       </c>
       <c r="I17" s="36">
-        <f>'Budget mensuel'!I26</f>
+        <f>'Budget mensuel'!I32</f>
         <v>610</v>
       </c>
       <c r="J17" s="36">
-        <f>'Budget mensuel'!J26</f>
+        <f>'Budget mensuel'!J32</f>
         <v>610</v>
       </c>
       <c r="K17" s="36">
-        <f>'Budget mensuel'!K26</f>
+        <f>'Budget mensuel'!K32</f>
         <v>610</v>
       </c>
       <c r="L17" s="36">
-        <f>'Budget mensuel'!L26</f>
+        <f>'Budget mensuel'!L32</f>
         <v>610</v>
       </c>
       <c r="M17" s="36">
-        <f>'Budget mensuel'!M26</f>
+        <f>'Budget mensuel'!M32</f>
         <v>610</v>
       </c>
       <c r="N17" s="36">
-        <f>'Budget mensuel'!N26</f>
+        <f>'Budget mensuel'!N32</f>
         <v>610</v>
       </c>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="B18" s="16">
         <f>SUM(C18:N18)</f>
@@ -4118,7 +4595,7 @@
     </row>
     <row r="19" spans="1:14" ht="13" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="B19" s="17">
         <f>SUM(C19:N19)</f>
@@ -4175,7 +4652,7 @@
     </row>
     <row r="21" spans="1:14" ht="13" x14ac:dyDescent="0.3">
       <c r="A21" s="10" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="B21" s="10"/>
       <c r="C21" s="10"/>
@@ -4193,64 +4670,64 @@
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="B22" s="16">
         <f>SUM(C22:N22)</f>
         <v>-16255.821428571435</v>
       </c>
       <c r="C22" s="36">
-        <f>'Budget mensuel'!C28</f>
+        <f>'Budget mensuel'!C34</f>
         <v>-2362</v>
       </c>
       <c r="D22" s="36">
-        <f>'Budget mensuel'!D28</f>
+        <f>'Budget mensuel'!D34</f>
         <v>-1810</v>
       </c>
       <c r="E22" s="36">
-        <f>'Budget mensuel'!E28</f>
+        <f>'Budget mensuel'!E34</f>
         <v>-2664.0714285714294</v>
       </c>
       <c r="F22" s="36">
-        <f>'Budget mensuel'!F28</f>
+        <f>'Budget mensuel'!F34</f>
         <v>-4162.2857142857156</v>
       </c>
       <c r="G22" s="36">
-        <f>'Budget mensuel'!G28</f>
+        <f>'Budget mensuel'!G34</f>
         <v>-1473.2500000000009</v>
       </c>
       <c r="H22" s="36">
-        <f>'Budget mensuel'!H28</f>
+        <f>'Budget mensuel'!H34</f>
         <v>-231.92857142857247</v>
       </c>
       <c r="I22" s="36">
-        <f>'Budget mensuel'!I28</f>
+        <f>'Budget mensuel'!I34</f>
         <v>-1730.1428571428587</v>
       </c>
       <c r="J22" s="36">
-        <f>'Budget mensuel'!J28</f>
+        <f>'Budget mensuel'!J34</f>
         <v>-241.10714285714312</v>
       </c>
       <c r="K22" s="36">
-        <f>'Budget mensuel'!K28</f>
+        <f>'Budget mensuel'!K34</f>
         <v>-1464.0714285714294</v>
       </c>
       <c r="L22" s="36">
-        <f>'Budget mensuel'!L28</f>
+        <f>'Budget mensuel'!L34</f>
         <v>-610</v>
       </c>
       <c r="M22" s="36">
-        <f>'Budget mensuel'!M28</f>
+        <f>'Budget mensuel'!M34</f>
         <v>-498</v>
       </c>
       <c r="N22" s="36">
-        <f>'Budget mensuel'!N28</f>
+        <f>'Budget mensuel'!N34</f>
         <v>991.03571428571377</v>
       </c>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="B23" s="16">
         <f>SUM(C23:N23)</f>
@@ -4271,7 +4748,7 @@
     </row>
     <row r="24" spans="1:14" ht="13" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="B24" s="17">
         <f>SUM(C24:N24)</f>
@@ -4328,7 +4805,7 @@
     </row>
     <row r="26" spans="1:14" ht="13" x14ac:dyDescent="0.3">
       <c r="A26" s="10" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="B26" s="10"/>
       <c r="C26" s="10"/>
@@ -4346,7 +4823,7 @@
     </row>
     <row r="27" spans="1:14" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="7" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="C27" s="18"/>
       <c r="D27" s="18"/>
@@ -4368,7 +4845,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42FB26B6-A531-4D48-8F04-B3463A220999}">
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="46.6328125" style="1" customWidth="1"/>
@@ -4381,12 +4858,12 @@
   <sheetData>
     <row r="1" spans="1:7" ht="18" x14ac:dyDescent="0.4">
       <c r="A1" s="3" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="13" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="13" x14ac:dyDescent="0.25">
@@ -4397,13 +4874,13 @@
         <v>32</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="F5" s="6" t="s">
         <v>37</v>
@@ -4414,7 +4891,7 @@
     </row>
     <row r="6" spans="1:7" ht="13" x14ac:dyDescent="0.3">
       <c r="A6" s="10" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="B6" s="10"/>
       <c r="C6" s="10"/>
@@ -4428,7 +4905,7 @@
         <v>120</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="C7" s="37">
         <f>'Budget mensuel'!$B$7</f>
@@ -4444,7 +4921,7 @@
         <v>90</v>
       </c>
       <c r="G7" s="22" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="37.5" x14ac:dyDescent="0.25">
@@ -4452,7 +4929,7 @@
         <v>121</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="C8" s="37">
         <f>'Budget mensuel'!$B$8</f>
@@ -4468,7 +4945,7 @@
         <v>90</v>
       </c>
       <c r="G8" s="22" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="37.5" x14ac:dyDescent="0.25">
@@ -4476,7 +4953,7 @@
         <v>122</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="C9" s="37">
         <f>'Budget mensuel'!$B$9</f>
@@ -4492,15 +4969,15 @@
         <v>90</v>
       </c>
       <c r="G9" s="22" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A10" s="19" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="B10" s="19" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="C10" s="37">
         <f>'Budget mensuel'!$B$10</f>
@@ -4516,7 +4993,7 @@
         <v>90</v>
       </c>
       <c r="G10" s="22" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="13" x14ac:dyDescent="0.25">
@@ -4524,7 +5001,7 @@
         <v>124</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="C11" s="24">
         <f t="shared" ref="C11:E11" si="0">SUM(C7:C10)</f>
@@ -4543,7 +5020,7 @@
     </row>
     <row r="12" spans="1:7" ht="13" x14ac:dyDescent="0.25">
       <c r="A12" s="29" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="B12" s="29"/>
       <c r="C12" s="29"/>
@@ -4640,172 +5117,708 @@
       <c r="F16" s="21"/>
       <c r="G16" s="22"/>
     </row>
-    <row r="17" spans="1:7" ht="37.5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" customFormat="1" ht="29" x14ac:dyDescent="0.35">
+      <c r="A17" s="51" t="s">
+        <v>221</v>
+      </c>
+      <c r="B17" s="51" t="s">
+        <v>170</v>
+      </c>
+      <c r="C17" s="50">
+        <f>'Budget mensuel'!$B$21</f>
+        <v>0</v>
+      </c>
+      <c r="D17" s="50">
+        <f>'Frais généraux 3 ans'!$F$13</f>
+        <v>32486.147999999997</v>
+      </c>
+      <c r="E17" s="50">
+        <f>'Frais généraux 3 ans'!$G$13</f>
+        <v>168206.14799999999</v>
+      </c>
+      <c r="F17" s="40" t="s">
+        <v>90</v>
+      </c>
+      <c r="G17" s="52" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A18" s="51" t="s">
+        <v>222</v>
+      </c>
+      <c r="B18" s="51" t="s">
+        <v>170</v>
+      </c>
+      <c r="C18" s="50">
+        <f>'Budget mensuel'!$B$31</f>
+        <v>12672</v>
+      </c>
+      <c r="D18" s="50">
+        <f>'Frais généraux 3 ans'!$F$25</f>
+        <v>24300</v>
+      </c>
+      <c r="E18" s="50">
+        <f>'Frais généraux 3 ans'!$G$25</f>
+        <v>57800</v>
+      </c>
+      <c r="F18" s="40" t="s">
+        <v>90</v>
+      </c>
+      <c r="G18" s="52" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="13" x14ac:dyDescent="0.25">
+      <c r="A19" s="8" t="s">
+        <v>192</v>
+      </c>
+      <c r="B19" s="8" t="s">
+        <v>170</v>
+      </c>
+      <c r="C19" s="28">
+        <f t="shared" ref="C19:E19" si="3">C17+C18</f>
+        <v>12672</v>
+      </c>
+      <c r="D19" s="28">
+        <f t="shared" si="3"/>
+        <v>56786.148000000001</v>
+      </c>
+      <c r="E19" s="28">
+        <f t="shared" si="3"/>
+        <v>226006.14799999999</v>
+      </c>
+      <c r="F19" s="21"/>
+      <c r="G19" s="22" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="13" x14ac:dyDescent="0.25">
+      <c r="A20" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="B20" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="C20" s="28">
+        <f t="shared" ref="C20:E20" si="4">C15-C19</f>
+        <v>-16255.821428571449</v>
+      </c>
+      <c r="D20" s="28">
+        <f t="shared" si="4"/>
+        <v>-59771.576571428639</v>
+      </c>
+      <c r="E20" s="28">
+        <f t="shared" si="4"/>
+        <v>-215698.57657142874</v>
+      </c>
+      <c r="F20" s="21"/>
+      <c r="G20" s="22"/>
+    </row>
+    <row r="21" spans="1:7" ht="13" x14ac:dyDescent="0.25">
+      <c r="A21" s="29" t="s">
+        <v>171</v>
+      </c>
+      <c r="B21" s="29"/>
+      <c r="C21" s="29"/>
+      <c r="D21" s="29"/>
+      <c r="E21" s="29"/>
+      <c r="F21" s="29"/>
+      <c r="G21" s="30"/>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" s="19" t="s">
+        <v>172</v>
+      </c>
+      <c r="B22" s="19" t="s">
+        <v>56</v>
+      </c>
+      <c r="C22" s="26">
+        <v>3000</v>
+      </c>
+      <c r="D22" s="26">
+        <v>5000</v>
+      </c>
+      <c r="E22" s="26">
+        <v>10000</v>
+      </c>
+      <c r="F22" s="21" t="s">
+        <v>90</v>
+      </c>
+      <c r="G22" s="22" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="13" x14ac:dyDescent="0.25">
+      <c r="A23" s="8" t="s">
+        <v>173</v>
+      </c>
+      <c r="B23" s="8" t="s">
+        <v>174</v>
+      </c>
+      <c r="C23" s="28">
+        <f t="shared" ref="C23:E23" si="5">C20-C22</f>
+        <v>-19255.821428571449</v>
+      </c>
+      <c r="D23" s="28">
+        <f t="shared" si="5"/>
+        <v>-64771.576571428639</v>
+      </c>
+      <c r="E23" s="28">
+        <f t="shared" si="5"/>
+        <v>-225698.57657142874</v>
+      </c>
+      <c r="F23" s="21"/>
+      <c r="G23" s="22"/>
+    </row>
+    <row r="24" spans="1:7" ht="13" x14ac:dyDescent="0.25">
+      <c r="A24" s="8" t="s">
+        <v>175</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>174</v>
+      </c>
+      <c r="C24" s="28">
+        <f>C23</f>
+        <v>-19255.821428571449</v>
+      </c>
+      <c r="D24" s="28">
+        <f t="shared" ref="D24:E24" si="6">C24+D23</f>
+        <v>-84027.398000000088</v>
+      </c>
+      <c r="E24" s="28">
+        <f t="shared" si="6"/>
+        <v>-309725.97457142884</v>
+      </c>
+      <c r="F24" s="21"/>
+      <c r="G24" s="22"/>
+    </row>
+    <row r="25" spans="1:7" ht="13" x14ac:dyDescent="0.25">
+      <c r="A25" s="8" t="s">
+        <v>176</v>
+      </c>
+      <c r="B25" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="C25" s="39">
+        <f t="shared" ref="C25:E25" si="7">IF(C11&gt;0,IF(C15&gt;0,C19/(C15/C11),0),0)</f>
+        <v>0</v>
+      </c>
+      <c r="D25" s="39">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="E25" s="39">
+        <f t="shared" si="7"/>
+        <v>1841.8030438651526</v>
+      </c>
+      <c r="F25" s="21"/>
+      <c r="G25" s="22"/>
+    </row>
+    <row r="27" spans="1:7" ht="13" x14ac:dyDescent="0.3">
+      <c r="A27" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="C27" s="17">
+        <f>MAX(0,-MIN(C24:E24))</f>
+        <v>309725.97457142884</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="13" x14ac:dyDescent="0.3">
+      <c r="A29" s="4" t="s">
+        <v>178</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F7:F25" xr:uid="{CE6E7BBF-D2B8-4903-BD10-C829B0A39B99}">
+      <formula1>"F,I,P,H"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C299EF4-2BFD-4A30-9CB8-0FD18304D49C}">
+  <dimension ref="A1:I27"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="46.6328125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="10.6328125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="16.6328125" style="1" customWidth="1"/>
+    <col min="4" max="5" width="13.6328125" style="1" customWidth="1"/>
+    <col min="6" max="7" width="16.6328125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="8.6328125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="70.6328125" style="1" customWidth="1"/>
+    <col min="10" max="16384" width="10.90625" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="18" x14ac:dyDescent="0.4">
+      <c r="A1" s="3" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="13" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="13" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="C4" s="47">
+        <v>0.45</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="13" x14ac:dyDescent="0.3">
+      <c r="A6" s="10" t="s">
+        <v>197</v>
+      </c>
+      <c r="B6" s="10"/>
+      <c r="C6" s="10"/>
+      <c r="D6" s="10"/>
+      <c r="E6" s="10"/>
+      <c r="F6" s="10"/>
+      <c r="G6" s="10"/>
+      <c r="H6" s="10"/>
+      <c r="I6" s="10"/>
+    </row>
+    <row r="7" spans="1:9" ht="42" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>199</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>203</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="I7" s="6" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="25" x14ac:dyDescent="0.25">
+      <c r="A8" s="21" t="s">
+        <v>204</v>
+      </c>
+      <c r="B8" s="20">
+        <v>2</v>
+      </c>
+      <c r="C8" s="25">
+        <v>2500</v>
+      </c>
+      <c r="D8" s="20">
+        <v>0</v>
+      </c>
+      <c r="E8" s="20">
+        <v>12</v>
+      </c>
+      <c r="F8" s="48">
+        <f t="shared" ref="F8:F12" si="0">B8*C8*D8*(1+$C$4)</f>
+        <v>0</v>
+      </c>
+      <c r="G8" s="48">
+        <f t="shared" ref="G8:G12" si="1">B8*C8*E8*(1+$C$4)</f>
+        <v>87000</v>
+      </c>
+      <c r="H8" s="21" t="s">
+        <v>90</v>
+      </c>
+      <c r="I8" s="22" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="25" x14ac:dyDescent="0.25">
+      <c r="A9" s="21" t="s">
+        <v>206</v>
+      </c>
+      <c r="B9" s="20">
+        <v>1</v>
+      </c>
+      <c r="C9" s="25">
+        <v>1867.02</v>
+      </c>
+      <c r="D9" s="20">
+        <v>12</v>
+      </c>
+      <c r="E9" s="20">
+        <v>12</v>
+      </c>
+      <c r="F9" s="48">
+        <f t="shared" si="0"/>
+        <v>32486.147999999997</v>
+      </c>
+      <c r="G9" s="48">
+        <f t="shared" si="1"/>
+        <v>32486.147999999997</v>
+      </c>
+      <c r="H9" s="21" t="s">
+        <v>90</v>
+      </c>
+      <c r="I9" s="22" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="25" x14ac:dyDescent="0.25">
+      <c r="A10" s="21" t="s">
+        <v>208</v>
+      </c>
+      <c r="B10" s="20">
+        <v>1</v>
+      </c>
+      <c r="C10" s="25">
+        <v>2800</v>
+      </c>
+      <c r="D10" s="20">
+        <v>0</v>
+      </c>
+      <c r="E10" s="20">
+        <v>12</v>
+      </c>
+      <c r="F10" s="48">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G10" s="48">
+        <f t="shared" si="1"/>
+        <v>48720</v>
+      </c>
+      <c r="H10" s="21" t="s">
+        <v>90</v>
+      </c>
+      <c r="I10" s="22" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" s="21"/>
+      <c r="B11" s="20"/>
+      <c r="C11" s="25"/>
+      <c r="D11" s="20"/>
+      <c r="E11" s="20"/>
+      <c r="F11" s="48">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G11" s="48">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="H11" s="21"/>
+      <c r="I11" s="22"/>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" s="21"/>
+      <c r="B12" s="20"/>
+      <c r="C12" s="25"/>
+      <c r="D12" s="20"/>
+      <c r="E12" s="20"/>
+      <c r="F12" s="48">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G12" s="48">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="H12" s="21"/>
+      <c r="I12" s="22"/>
+    </row>
+    <row r="13" spans="1:9" ht="13" x14ac:dyDescent="0.25">
+      <c r="A13" s="8" t="s">
+        <v>189</v>
+      </c>
+      <c r="B13" s="24">
+        <f>SUM(B8:B12)</f>
+        <v>4</v>
+      </c>
+      <c r="C13" s="8"/>
+      <c r="D13" s="8"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="28">
+        <f>SUM(F8:F12)</f>
+        <v>32486.147999999997</v>
+      </c>
+      <c r="G13" s="28">
+        <f>SUM(G8:G12)</f>
+        <v>168206.14799999999</v>
+      </c>
+      <c r="H13" s="19"/>
+      <c r="I13" s="9"/>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" s="19"/>
+      <c r="B14" s="19"/>
+      <c r="C14" s="19"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="19"/>
+      <c r="G14" s="19"/>
+      <c r="H14" s="19"/>
+      <c r="I14" s="9"/>
+    </row>
+    <row r="15" spans="1:9" ht="13" x14ac:dyDescent="0.25">
+      <c r="A15" s="29" t="s">
+        <v>210</v>
+      </c>
+      <c r="B15" s="29"/>
+      <c r="C15" s="29"/>
+      <c r="D15" s="29"/>
+      <c r="E15" s="29"/>
+      <c r="F15" s="29"/>
+      <c r="G15" s="29"/>
+      <c r="H15" s="29"/>
+      <c r="I15" s="30"/>
+    </row>
+    <row r="16" spans="1:9" ht="13" x14ac:dyDescent="0.25">
+      <c r="A16" s="49" t="s">
+        <v>31</v>
+      </c>
+      <c r="B16" s="49"/>
+      <c r="C16" s="49"/>
+      <c r="D16" s="49"/>
+      <c r="E16" s="49"/>
+      <c r="F16" s="49" t="s">
+        <v>211</v>
+      </c>
+      <c r="G16" s="49" t="s">
+        <v>212</v>
+      </c>
+      <c r="H16" s="49" t="s">
+        <v>37</v>
+      </c>
+      <c r="I16" s="49" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" ht="25" x14ac:dyDescent="0.25">
       <c r="A17" s="19" t="s">
         <v>128</v>
       </c>
-      <c r="B17" s="19" t="s">
-        <v>173</v>
-      </c>
-      <c r="C17" s="39">
-        <f>'Budget mensuel'!$B$26</f>
-        <v>12672</v>
-      </c>
-      <c r="D17" s="26">
-        <v>60000</v>
-      </c>
-      <c r="E17" s="26">
-        <v>150000</v>
-      </c>
-      <c r="F17" s="21" t="s">
+      <c r="B17" s="19"/>
+      <c r="C17" s="19"/>
+      <c r="D17" s="19"/>
+      <c r="E17" s="19"/>
+      <c r="F17" s="26">
+        <v>0</v>
+      </c>
+      <c r="G17" s="26">
+        <v>10800</v>
+      </c>
+      <c r="H17" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="G17" s="22" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" ht="13" x14ac:dyDescent="0.25">
-      <c r="A18" s="8" t="s">
-        <v>161</v>
-      </c>
-      <c r="B18" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="C18" s="28">
-        <f t="shared" ref="C18:E18" si="3">C15-C17</f>
-        <v>-16255.821428571449</v>
-      </c>
-      <c r="D18" s="28">
-        <f t="shared" si="3"/>
-        <v>-62985.428571428638</v>
-      </c>
-      <c r="E18" s="28">
-        <f t="shared" si="3"/>
-        <v>-139692.42857142875</v>
-      </c>
-      <c r="F18" s="21"/>
-      <c r="G18" s="22"/>
-    </row>
-    <row r="19" spans="1:7" ht="13" x14ac:dyDescent="0.25">
-      <c r="A19" s="29" t="s">
-        <v>174</v>
-      </c>
-      <c r="B19" s="29"/>
-      <c r="C19" s="29"/>
-      <c r="D19" s="29"/>
-      <c r="E19" s="29"/>
-      <c r="F19" s="29"/>
-      <c r="G19" s="30"/>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I17" s="22" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" s="19" t="s">
+        <v>214</v>
+      </c>
+      <c r="B18" s="19"/>
+      <c r="C18" s="19"/>
+      <c r="D18" s="19"/>
+      <c r="E18" s="19"/>
+      <c r="F18" s="26">
+        <v>1500</v>
+      </c>
+      <c r="G18" s="26">
+        <v>3000</v>
+      </c>
+      <c r="H18" s="21" t="s">
+        <v>90</v>
+      </c>
+      <c r="I18" s="22" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" s="19" t="s">
+        <v>130</v>
+      </c>
+      <c r="B19" s="19"/>
+      <c r="C19" s="19"/>
+      <c r="D19" s="19"/>
+      <c r="E19" s="19"/>
+      <c r="F19" s="26">
+        <v>15000</v>
+      </c>
+      <c r="G19" s="26">
+        <v>30000</v>
+      </c>
+      <c r="H19" s="21" t="s">
+        <v>90</v>
+      </c>
+      <c r="I19" s="22" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" ht="25" x14ac:dyDescent="0.25">
       <c r="A20" s="19" t="s">
-        <v>175</v>
-      </c>
-      <c r="B20" s="19" t="s">
-        <v>56</v>
-      </c>
-      <c r="C20" s="26">
-        <v>3000</v>
-      </c>
-      <c r="D20" s="26">
-        <v>5000</v>
-      </c>
-      <c r="E20" s="26">
-        <v>10000</v>
-      </c>
-      <c r="F20" s="21" t="s">
+        <v>131</v>
+      </c>
+      <c r="B20" s="19"/>
+      <c r="C20" s="19"/>
+      <c r="D20" s="19"/>
+      <c r="E20" s="19"/>
+      <c r="F20" s="26">
+        <v>1200</v>
+      </c>
+      <c r="G20" s="26">
+        <v>2000</v>
+      </c>
+      <c r="H20" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="G20" s="22" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" ht="13" x14ac:dyDescent="0.25">
-      <c r="A21" s="8" t="s">
-        <v>176</v>
-      </c>
-      <c r="B21" s="8" t="s">
-        <v>177</v>
-      </c>
-      <c r="C21" s="28">
-        <f t="shared" ref="C21:E21" si="4">C18-C20</f>
-        <v>-19255.821428571449</v>
-      </c>
-      <c r="D21" s="28">
-        <f t="shared" si="4"/>
-        <v>-67985.428571428638</v>
-      </c>
-      <c r="E21" s="28">
-        <f t="shared" si="4"/>
-        <v>-149692.42857142875</v>
-      </c>
-      <c r="F21" s="21"/>
-      <c r="G21" s="22"/>
-    </row>
-    <row r="22" spans="1:7" ht="13" x14ac:dyDescent="0.25">
-      <c r="A22" s="8" t="s">
-        <v>178</v>
-      </c>
-      <c r="B22" s="8" t="s">
-        <v>177</v>
-      </c>
-      <c r="C22" s="28">
-        <f>C21</f>
-        <v>-19255.821428571449</v>
-      </c>
-      <c r="D22" s="28">
-        <f t="shared" ref="D22:E22" si="5">C22+D21</f>
-        <v>-87241.250000000087</v>
-      </c>
-      <c r="E22" s="28">
-        <f t="shared" si="5"/>
-        <v>-236933.67857142884</v>
-      </c>
-      <c r="F22" s="21"/>
-      <c r="G22" s="22"/>
-    </row>
-    <row r="23" spans="1:7" ht="13" x14ac:dyDescent="0.25">
-      <c r="A23" s="8" t="s">
-        <v>179</v>
-      </c>
-      <c r="B23" s="8" t="s">
-        <v>170</v>
-      </c>
-      <c r="C23" s="40">
-        <f t="shared" ref="C23:E23" si="6">IF(C11&gt;0,IF(C15&gt;0,C17/(C15/C11),0),0)</f>
-        <v>0</v>
-      </c>
-      <c r="D23" s="40">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="E23" s="40">
-        <f t="shared" si="6"/>
-        <v>1222.4023949108362</v>
-      </c>
-      <c r="F23" s="21"/>
-      <c r="G23" s="22"/>
-    </row>
-    <row r="25" spans="1:7" ht="13" x14ac:dyDescent="0.3">
+      <c r="I20" s="22" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" s="19" t="s">
+        <v>132</v>
+      </c>
+      <c r="B21" s="19"/>
+      <c r="C21" s="19"/>
+      <c r="D21" s="19"/>
+      <c r="E21" s="19"/>
+      <c r="F21" s="26">
+        <v>4000</v>
+      </c>
+      <c r="G21" s="26">
+        <v>6000</v>
+      </c>
+      <c r="H21" s="21" t="s">
+        <v>90</v>
+      </c>
+      <c r="I21" s="22" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22" s="19" t="s">
+        <v>133</v>
+      </c>
+      <c r="B22" s="19"/>
+      <c r="C22" s="19"/>
+      <c r="D22" s="19"/>
+      <c r="E22" s="19"/>
+      <c r="F22" s="26">
+        <v>600</v>
+      </c>
+      <c r="G22" s="26">
+        <v>1000</v>
+      </c>
+      <c r="H22" s="21" t="s">
+        <v>90</v>
+      </c>
+      <c r="I22" s="22" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A23" s="19" t="s">
+        <v>134</v>
+      </c>
+      <c r="B23" s="19"/>
+      <c r="C23" s="19"/>
+      <c r="D23" s="19"/>
+      <c r="E23" s="19"/>
+      <c r="F23" s="26">
+        <v>2000</v>
+      </c>
+      <c r="G23" s="26">
+        <v>4000</v>
+      </c>
+      <c r="H23" s="21" t="s">
+        <v>90</v>
+      </c>
+      <c r="I23" s="22" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A24" s="19" t="s">
+        <v>220</v>
+      </c>
+      <c r="B24" s="19"/>
+      <c r="C24" s="19"/>
+      <c r="D24" s="19"/>
+      <c r="E24" s="19"/>
+      <c r="F24" s="26">
+        <v>0</v>
+      </c>
+      <c r="G24" s="26">
+        <v>1000</v>
+      </c>
+      <c r="H24" s="21" t="s">
+        <v>90</v>
+      </c>
+      <c r="I24" s="22" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" ht="13" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
-        <v>180</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="C25" s="17">
-        <f>MAX(0,-MIN(C22:E22))</f>
-        <v>236933.67857142884</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" ht="13" x14ac:dyDescent="0.3">
-      <c r="A27" s="4" t="s">
-        <v>181</v>
+        <v>191</v>
+      </c>
+      <c r="B25" s="2"/>
+      <c r="C25" s="2"/>
+      <c r="D25" s="2"/>
+      <c r="E25" s="2"/>
+      <c r="F25" s="17">
+        <f>SUM(F17:F24)</f>
+        <v>24300</v>
+      </c>
+      <c r="G25" s="17">
+        <f>SUM(G17:G24)</f>
+        <v>57800</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" ht="13" x14ac:dyDescent="0.3">
+      <c r="A27" s="45" t="s">
+        <v>192</v>
+      </c>
+      <c r="B27" s="45"/>
+      <c r="C27" s="45"/>
+      <c r="D27" s="45"/>
+      <c r="E27" s="45"/>
+      <c r="F27" s="46">
+        <f>F13+F25</f>
+        <v>56786.148000000001</v>
+      </c>
+      <c r="G27" s="46">
+        <f>G13+G25</f>
+        <v>226006.14799999999</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F7:F23" xr:uid="{CE6E7BBF-D2B8-4903-BD10-C829B0A39B99}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H8:H24" xr:uid="{17BF4D97-1CC3-431D-AE47-E54A12C319AD}">
       <formula1>"F,I,P,H"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Finance : intégration du staffing des Opérations (28/10/2026)
Nouvel onglet Staffing dans le modèle Prévisions : effectifs proposés par
les Opérations × heures et coûts horaires (hypothèses), relié au coût de
l'équipe de chaque soirée. Trésorerie recalculée (investissements de l'année 1
inclus), tableau de bord régénéré, fiche des données manquantes mise à jour.
Besoin de financement à 3 ans : 557 940 € en hypothèses centrales.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/2 FINANCE/PREVISIONS/2026 1027 Modèle - Budget, plan financier, prix et marges.xlsx
+++ b/2 FINANCE/PREVISIONS/2026 1027 Modèle - Budget, plan financier, prix et marges.xlsx
@@ -8,17 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vians\Documents\Claude\Projects\HEC-GEMM-Groupe-7\2 FINANCE\PREVISIONS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A68D3D2-8882-46A6-9CD1-8C34C95E3736}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CCD5C6A-B0F7-4AAD-B84C-98FD8DDC5033}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{09426CC5-4BCC-48B7-8854-C5C8E2CE30D1}"/>
   </bookViews>
   <sheets>
     <sheet name="Mode d'emploi" sheetId="1" r:id="rId1"/>
     <sheet name="Prix et marges" sheetId="2" r:id="rId2"/>
-    <sheet name="Budget mensuel" sheetId="3" r:id="rId3"/>
-    <sheet name="Prévu et réel" sheetId="4" r:id="rId4"/>
-    <sheet name="Plan financier 3 ans" sheetId="5" r:id="rId5"/>
-    <sheet name="Frais généraux 3 ans" sheetId="6" r:id="rId6"/>
+    <sheet name="Staffing" sheetId="7" r:id="rId3"/>
+    <sheet name="Budget mensuel" sheetId="3" r:id="rId4"/>
+    <sheet name="Prévu et réel" sheetId="4" r:id="rId5"/>
+    <sheet name="Plan financier 3 ans" sheetId="5" r:id="rId6"/>
+    <sheet name="Frais généraux 3 ans" sheetId="6" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -44,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="384" uniqueCount="228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="428" uniqueCount="266">
   <si>
     <t>Prévisions — budget, plan financier, prix et marges</t>
   </si>
@@ -253,9 +254,6 @@
     <t>Matières et boissons</t>
   </si>
   <si>
-    <t>Équipe de service et sommelier</t>
-  </si>
-  <si>
     <t>Ménage et remise en état du lieu</t>
   </si>
   <si>
@@ -361,9 +359,6 @@
     <t>Même source ; accord mets-jus au même coût que l'accord mets-vins (pricing : « coût réel reste à chiffrer »)</t>
   </si>
   <si>
-    <t>Calé sur la cible du Produit (équipe de service et sommelier 14 / 12 / 11 % du prix HT). Qui assure le service (restaurant ou nous) reste à décider (pricing, point 3)</t>
-  </si>
-  <si>
     <t>Hypothèse temporaire ; cible « frais » du Produit 8 / 6 / 5 % du prix HT</t>
   </si>
   <si>
@@ -728,6 +723,126 @@
   </si>
   <si>
     <t>Mis à jour le 28/10/2026 : frais généraux divisés en ressources humaines (fondateurs, salariés, charges sociales, stagiaires et indépendants) et frais matériels et de fonctionnement (locaux, outils, marketing, assurance, honoraires, banque, déplacements, autres). Année 1 : budget mensuel. Années 2 et 3 : onglet « Frais généraux 3 ans ».</t>
+  </si>
+  <si>
+    <t>Staffing d'une soirée : effectifs des Opérations × heures × coût horaire</t>
+  </si>
+  <si>
+    <t>Effectifs repris du calculateur des Opérations (propositions, catégorie C2). Heures et coûts horaires : hypothèses temporaires, aucun devis à ce jour.</t>
+  </si>
+  <si>
+    <t>Service de salle fourni par :</t>
+  </si>
+  <si>
+    <t>Nous</t>
+  </si>
+  <si>
+    <t>Question non tranchée (Produit, pricing point 3 ; Opérations, note § 3.4). « Restaurant » sort les postes de salle du coût ; la part du restaurateur (Prix et marges, ligne 19) devrait alors augmenter.</t>
+  </si>
+  <si>
+    <t>Rôle</t>
+  </si>
+  <si>
+    <t>Heures par personne</t>
+  </si>
+  <si>
+    <t>Coût horaire chargé (€)</t>
+  </si>
+  <si>
+    <t>Privatisation (table de 10)</t>
+  </si>
+  <si>
+    <t>Poste de salle (1 = oui)</t>
+  </si>
+  <si>
+    <t>Source et nature</t>
+  </si>
+  <si>
+    <t>Brigade (second, commis)</t>
+  </si>
+  <si>
+    <t>Effectifs P (Opérations). H : 9 h (mise en place et service) à 35 €/h, coût d'un extra retenu dans le descriptif du projet 3 (H), à confirmer par devis</t>
+  </si>
+  <si>
+    <t>Maître d'hôtel</t>
+  </si>
+  <si>
+    <t>Effectifs P (Opérations). H : 8 h à 45 €/h</t>
+  </si>
+  <si>
+    <t>Serveurs (base)</t>
+  </si>
+  <si>
+    <t>Effectifs P (Opérations : 1 serveur pour 7 couverts). H : 7 h à 35 €/h</t>
+  </si>
+  <si>
+    <t>Serveur de réserve</t>
+  </si>
+  <si>
+    <t>Effectifs P (Opérations : 1 en criticité C2 et C3). H : 7 h à 35 €/h</t>
+  </si>
+  <si>
+    <t>Sommelier invité</t>
+  </si>
+  <si>
+    <t>Effectifs P (Opérations). H : 7 h à 60 €/h, cachet à négocier</t>
+  </si>
+  <si>
+    <t>Aide sommelier</t>
+  </si>
+  <si>
+    <t>Effectifs P (Opérations : à partir de 20 couverts). H : 7 h à 38 €/h</t>
+  </si>
+  <si>
+    <t>Plongeurs</t>
+  </si>
+  <si>
+    <t>Effectifs P (Opérations). H : 7 h à 30 €/h</t>
+  </si>
+  <si>
+    <t>Responsable de production (nous)</t>
+  </si>
+  <si>
+    <t>Effectifs P (Opérations). H : assuré par un fondateur, non rémunéré la première année (coût dans les frais généraux)</t>
+  </si>
+  <si>
+    <t>Interlocuteur client (Ventes)</t>
+  </si>
+  <si>
+    <t>Effectifs P (Opérations : en C2 et C3). H : assuré par un fondateur, non rémunéré la première année</t>
+  </si>
+  <si>
+    <t>Chef invité : 1 par soirée, compté à part (cachet, Prix et marges ligne 20)</t>
+  </si>
+  <si>
+    <t>Personnes mobilisées, hors chef</t>
+  </si>
+  <si>
+    <t>dont postes de salle</t>
+  </si>
+  <si>
+    <t>Heures de travail payées</t>
+  </si>
+  <si>
+    <t>Coût de l'équipe de la soirée (€ HT)</t>
+  </si>
+  <si>
+    <t>Source des effectifs : 6 OPERATIONS/PRODUCTION/2026 1028 Calculateur de staffing par événement.xlsx et 2026 1028 Typologie des événements, process et staffing.md (Opérations, 28/10/2026 ; colonnes Pilote 1, Le Voyage, Pilote 2 et Table d'affaires). Pour une soirée récurrente en criticité C1, le serveur de réserve et l'interlocuteur client ne sont pas nécessaires.</t>
+  </si>
+  <si>
+    <t>P / H</t>
+  </si>
+  <si>
+    <t>Onglet Staffing : effectifs des Opérations (P, 6 OPERATIONS/PRODUCTION/2026 1028 Calculateur de staffing par événement.xlsx et 2026 1028 Typologie des événements, process et staffing.md) × heures et coûts horaires (H). Remplace la cible du Produit (14 / 12 / 11 % du prix HT) utilisée le 27/10/2026</t>
+  </si>
+  <si>
+    <t>Équipe de service, brigade, sommelier et plonge</t>
+  </si>
+  <si>
+    <t>Staffing</t>
+  </si>
+  <si>
+    <t>Mis à jour le 28/10/2026 : le coût de l'équipe de chaque soirée (Prix et marges, ligne 26) est calculé dans l'onglet « Staffing » à partir des effectifs proposés par les Opérations (6 OPERATIONS/PRODUCTION/2026 1028 Calculateur de staffing par événement.xlsx et 2026 1028 Typologie des événements, process et staffing.md), multipliés par des heures et des coûts horaires en hypothèse (H). Le choix « service de salle fourni par le restaurant » y est modifiable.</t>
   </si>
 </sst>
 </file>
@@ -912,7 +1027,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1012,9 +1127,17 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="167" fontId="14" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="167" fontId="10" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1350,7 +1473,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FBA644DB-8C71-4A8A-A457-0A27A3813ADD}">
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.6328125" style="1" customWidth="1"/>
@@ -1474,10 +1597,18 @@
     </row>
     <row r="17" spans="1:2" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>227</v>
+        <v>225</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="50" x14ac:dyDescent="0.25">
+      <c r="A18" s="8" t="s">
+        <v>264</v>
+      </c>
+      <c r="B18" s="9" t="s">
+        <v>265</v>
       </c>
     </row>
   </sheetData>
@@ -1577,13 +1708,13 @@
         <v>10</v>
       </c>
       <c r="G7" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="H7" s="22" t="s">
         <v>87</v>
       </c>
-      <c r="H7" s="22" t="s">
+      <c r="I7" s="21" t="s">
         <v>88</v>
-      </c>
-      <c r="I7" s="21" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="37.5" x14ac:dyDescent="0.25">
@@ -1606,13 +1737,13 @@
         <v>1</v>
       </c>
       <c r="G8" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="H8" s="22" t="s">
         <v>90</v>
       </c>
-      <c r="H8" s="22" t="s">
+      <c r="I8" s="21" t="s">
         <v>91</v>
-      </c>
-      <c r="I8" s="21" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="13" x14ac:dyDescent="0.25">
@@ -1662,13 +1793,13 @@
         <v>300</v>
       </c>
       <c r="G10" s="21" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H10" s="22" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="I10" s="21" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="37.5" x14ac:dyDescent="0.25">
@@ -1691,13 +1822,13 @@
         <v>6000</v>
       </c>
       <c r="G11" s="21" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H11" s="22" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I11" s="21" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="50" x14ac:dyDescent="0.25">
@@ -1720,13 +1851,13 @@
         <v>0.12</v>
       </c>
       <c r="G12" s="21" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="H12" s="22" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="I12" s="21" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="13" x14ac:dyDescent="0.25">
@@ -1803,13 +1934,13 @@
         <v>0</v>
       </c>
       <c r="G15" s="21" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="H15" s="22" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I15" s="21" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="25" x14ac:dyDescent="0.25">
@@ -1832,13 +1963,13 @@
         <v>0</v>
       </c>
       <c r="G16" s="21" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="H16" s="22" t="s">
+        <v>96</v>
+      </c>
+      <c r="I16" s="21" t="s">
         <v>97</v>
-      </c>
-      <c r="I16" s="21" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="13" x14ac:dyDescent="0.25">
@@ -1901,13 +2032,13 @@
         <v>2000</v>
       </c>
       <c r="G19" s="21" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="H19" s="22" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="I19" s="21" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="50" x14ac:dyDescent="0.25">
@@ -1930,13 +2061,13 @@
         <v>1800</v>
       </c>
       <c r="G20" s="21" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="H20" s="22" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I20" s="21" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="21" spans="1:9" ht="25" x14ac:dyDescent="0.25">
@@ -1959,13 +2090,13 @@
         <v>0</v>
       </c>
       <c r="G21" s="21" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="H21" s="22" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="I21" s="21" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="22" spans="1:9" ht="13" x14ac:dyDescent="0.25">
@@ -2015,13 +2146,13 @@
         <v>50</v>
       </c>
       <c r="G23" s="21" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="H23" s="22" t="s">
+        <v>101</v>
+      </c>
+      <c r="I23" s="21" t="s">
         <v>102</v>
-      </c>
-      <c r="I23" s="21" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="24" spans="1:9" ht="25" x14ac:dyDescent="0.25">
@@ -2044,13 +2175,13 @@
         <v>30</v>
       </c>
       <c r="G24" s="21" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="H24" s="22" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="I24" s="21" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="25" spans="1:9" ht="13" x14ac:dyDescent="0.25">
@@ -2080,38 +2211,42 @@
       <c r="H25" s="22"/>
       <c r="I25" s="21"/>
     </row>
-    <row r="26" spans="1:9" ht="37.5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" ht="62.5" x14ac:dyDescent="0.25">
       <c r="A26" s="19" t="s">
-        <v>69</v>
+        <v>263</v>
       </c>
       <c r="B26" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="C26" s="26">
-        <v>870</v>
-      </c>
-      <c r="D26" s="26">
-        <v>1080</v>
-      </c>
-      <c r="E26" s="26">
-        <v>1350</v>
-      </c>
-      <c r="F26" s="26">
-        <v>950</v>
+      <c r="C26" s="54">
+        <f>Staffing!D21</f>
+        <v>3636</v>
+      </c>
+      <c r="D26" s="54">
+        <f>Staffing!E21</f>
+        <v>3636</v>
+      </c>
+      <c r="E26" s="54">
+        <f>Staffing!F21</f>
+        <v>3076</v>
+      </c>
+      <c r="F26" s="54">
+        <f>Staffing!G21</f>
+        <v>2040</v>
       </c>
       <c r="G26" s="21" t="s">
-        <v>90</v>
+        <v>261</v>
       </c>
       <c r="H26" s="22" t="s">
-        <v>105</v>
+        <v>262</v>
       </c>
       <c r="I26" s="21" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="19" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B27" s="19" t="s">
         <v>56</v>
@@ -2129,18 +2264,18 @@
         <v>150</v>
       </c>
       <c r="G27" s="21" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="H27" s="22" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="I27" s="21" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="19" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B28" s="19" t="s">
         <v>56</v>
@@ -2158,18 +2293,18 @@
         <v>150</v>
       </c>
       <c r="G28" s="21" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="H28" s="22" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="I28" s="21" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="19" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B29" s="19" t="s">
         <v>56</v>
@@ -2187,18 +2322,18 @@
         <v>150</v>
       </c>
       <c r="G29" s="21" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="H29" s="22" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="I29" s="21" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="30" spans="1:9" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A30" s="19" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B30" s="19" t="s">
         <v>64</v>
@@ -2216,18 +2351,18 @@
         <v>0</v>
       </c>
       <c r="G30" s="21" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="H30" s="22" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="I30" s="21" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="31" spans="1:9" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A31" s="19" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B31" s="19" t="s">
         <v>64</v>
@@ -2245,18 +2380,18 @@
         <v>0.1</v>
       </c>
       <c r="G31" s="21" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="H31" s="22" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="I31" s="21" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="32" spans="1:9" ht="13" x14ac:dyDescent="0.25">
       <c r="A32" s="8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B32" s="8" t="s">
         <v>56</v>
@@ -2283,7 +2418,7 @@
     </row>
     <row r="33" spans="1:9" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A33" s="19" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B33" s="19" t="s">
         <v>56</v>
@@ -2301,37 +2436,37 @@
         <v>0</v>
       </c>
       <c r="G33" s="21" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="H33" s="22" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="I33" s="21" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="34" spans="1:9" ht="13" x14ac:dyDescent="0.25">
       <c r="A34" s="8" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B34" s="8" t="s">
         <v>56</v>
       </c>
       <c r="C34" s="28">
         <f t="shared" ref="C34:F34" si="7">C19+C22+C25+C26+C27+C28+C29+C32+C33</f>
-        <v>5773.7142857142853</v>
+        <v>8539.7142857142862</v>
       </c>
       <c r="D34" s="28">
         <f t="shared" si="7"/>
-        <v>7988.25</v>
+        <v>10544.25</v>
       </c>
       <c r="E34" s="28">
         <f t="shared" si="7"/>
-        <v>12209.428571428572</v>
+        <v>13935.428571428572</v>
       </c>
       <c r="F34" s="28">
         <f t="shared" si="7"/>
-        <v>6803.5714285714284</v>
+        <v>7893.5714285714284</v>
       </c>
       <c r="G34" s="21"/>
       <c r="H34" s="22"/>
@@ -2339,7 +2474,7 @@
     </row>
     <row r="35" spans="1:9" ht="13" x14ac:dyDescent="0.25">
       <c r="A35" s="29" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B35" s="29"/>
       <c r="C35" s="29"/>
@@ -2352,26 +2487,26 @@
     </row>
     <row r="36" spans="1:9" ht="13" x14ac:dyDescent="0.25">
       <c r="A36" s="8" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B36" s="8" t="s">
         <v>56</v>
       </c>
       <c r="C36" s="28">
         <f t="shared" ref="C36:F36" si="8">C17-C34</f>
-        <v>-854.07142857142935</v>
+        <v>-3620.0714285714303</v>
       </c>
       <c r="D36" s="28">
         <f t="shared" si="8"/>
-        <v>-863.25000000000091</v>
+        <v>-3419.2500000000009</v>
       </c>
       <c r="E36" s="28">
         <f t="shared" si="8"/>
-        <v>-2352.2857142857156</v>
+        <v>-4078.2857142857156</v>
       </c>
       <c r="F36" s="28">
         <f t="shared" si="8"/>
-        <v>1232.1428571428569</v>
+        <v>142.14285714285688</v>
       </c>
       <c r="G36" s="21"/>
       <c r="H36" s="22"/>
@@ -2379,26 +2514,26 @@
     </row>
     <row r="37" spans="1:9" ht="13" x14ac:dyDescent="0.25">
       <c r="A37" s="8" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B37" s="8" t="s">
         <v>64</v>
       </c>
       <c r="C37" s="31">
         <f t="shared" ref="C37:F37" si="9">IF(C17&gt;0,C36/C17,0)</f>
-        <v>-0.1736043557168786</v>
+        <v>-0.73584029038112575</v>
       </c>
       <c r="D37" s="31">
         <f t="shared" si="9"/>
-        <v>-0.12115789473684224</v>
+        <v>-0.47989473684210543</v>
       </c>
       <c r="E37" s="31">
         <f t="shared" si="9"/>
-        <v>-0.23863768115942044</v>
+        <v>-0.41373913043478278</v>
       </c>
       <c r="F37" s="31">
         <f t="shared" si="9"/>
-        <v>0.15333333333333332</v>
+        <v>1.7688888888888858E-2</v>
       </c>
       <c r="G37" s="21"/>
       <c r="H37" s="22"/>
@@ -2406,26 +2541,26 @@
     </row>
     <row r="38" spans="1:9" ht="13" x14ac:dyDescent="0.25">
       <c r="A38" s="8" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B38" s="8" t="s">
         <v>54</v>
       </c>
       <c r="C38" s="27">
         <f t="shared" ref="C38:F38" si="10">IF(C9&gt;0,C36/C9,0)</f>
-        <v>-44.951127819548915</v>
+        <v>-190.53007518797003</v>
       </c>
       <c r="D38" s="27">
         <f t="shared" si="10"/>
-        <v>-45.434210526315837</v>
+        <v>-179.96052631578951</v>
       </c>
       <c r="E38" s="27">
         <f t="shared" si="10"/>
-        <v>-147.01785714285722</v>
+        <v>-254.89285714285722</v>
       </c>
       <c r="F38" s="27">
         <f t="shared" si="10"/>
-        <v>123.21428571428569</v>
+        <v>14.214285714285689</v>
       </c>
       <c r="G38" s="21"/>
       <c r="H38" s="22"/>
@@ -2433,7 +2568,7 @@
     </row>
     <row r="39" spans="1:9" ht="13" x14ac:dyDescent="0.25">
       <c r="A39" s="8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B39" s="8" t="s">
         <v>64</v>
@@ -2460,7 +2595,7 @@
     </row>
     <row r="40" spans="1:9" ht="13" x14ac:dyDescent="0.25">
       <c r="A40" s="8" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B40" s="8" t="s">
         <v>64</v>
@@ -2487,26 +2622,26 @@
     </row>
     <row r="41" spans="1:9" ht="13" x14ac:dyDescent="0.25">
       <c r="A41" s="8" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B41" s="8" t="s">
         <v>64</v>
       </c>
       <c r="C41" s="31">
         <f t="shared" ref="C41:F41" si="13">C37</f>
-        <v>-0.1736043557168786</v>
+        <v>-0.73584029038112575</v>
       </c>
       <c r="D41" s="31">
         <f t="shared" si="13"/>
-        <v>-0.12115789473684224</v>
+        <v>-0.47989473684210543</v>
       </c>
       <c r="E41" s="31">
         <f t="shared" si="13"/>
-        <v>-0.23863768115942044</v>
+        <v>-0.41373913043478278</v>
       </c>
       <c r="F41" s="31">
         <f t="shared" si="13"/>
-        <v>0.15333333333333332</v>
+        <v>1.7688888888888858E-2</v>
       </c>
       <c r="G41" s="21"/>
       <c r="H41" s="22"/>
@@ -2514,26 +2649,26 @@
     </row>
     <row r="42" spans="1:9" ht="13" x14ac:dyDescent="0.25">
       <c r="A42" s="8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B42" s="8" t="s">
         <v>48</v>
       </c>
       <c r="C42" s="27">
         <f t="shared" ref="C42:F42" si="14">IF(AND(C9&gt;0,1-C21-C30-C31&gt;0),((C19+C20+C26+C27+C28+C29+C33+C9*(C23+C24))/(1-C21-C30-C31)-C14-C16)/C9*(1+C12),0)</f>
-        <v>341.16388532306382</v>
+        <v>506.86350021394958</v>
       </c>
       <c r="D42" s="27">
         <f t="shared" si="14"/>
-        <v>474.48213681956508</v>
+        <v>635.7984898005185</v>
       </c>
       <c r="E42" s="27">
         <f t="shared" si="14"/>
-        <v>876.26696832579194</v>
+        <v>1012.9411764705883</v>
       </c>
       <c r="F42" s="27">
         <f t="shared" si="14"/>
-        <v>146.66666666666663</v>
+        <v>282.31111111111113</v>
       </c>
       <c r="G42" s="21"/>
       <c r="H42" s="22"/>
@@ -2541,26 +2676,26 @@
     </row>
     <row r="43" spans="1:9" ht="13" x14ac:dyDescent="0.25">
       <c r="A43" s="8" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B43" s="8" t="s">
         <v>44</v>
       </c>
       <c r="C43" s="31">
         <f t="shared" ref="C43:F43" si="15">IF(AND(C7&gt;0,C13*(1-C21-C30-C31)-(C23+C24)&gt;0),MAX(0,(C19+C20+C26+C27+C28+C29+C33-(C14+C16)*(1-C21-C30-C31))/(C13*(1-C21-C30-C31)-(C23+C24)))/C7,0)</f>
-        <v>1.0012620950778295</v>
+        <v>1.680058897770299</v>
       </c>
       <c r="D43" s="31">
         <f t="shared" si="15"/>
-        <v>0.94263728576425343</v>
+        <v>1.3896467296257435</v>
       </c>
       <c r="E43" s="31">
         <f t="shared" si="15"/>
-        <v>1.1106499386850297</v>
+        <v>1.3385906989906613</v>
       </c>
       <c r="F43" s="31">
         <f t="shared" si="15"/>
-        <v>0.23503325942350325</v>
+        <v>0.91175166297117516</v>
       </c>
       <c r="G43" s="21"/>
       <c r="H43" s="22"/>
@@ -2580,6 +2715,456 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{838C2CEE-3AA8-4CB7-9962-F225A7B6E75A}">
+  <dimension ref="A1:I23"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="36.6328125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="11.6328125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="13.6328125" style="1" customWidth="1"/>
+    <col min="4" max="6" width="12.6328125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="14.6328125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="10.6328125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="80.6328125" style="1" customWidth="1"/>
+    <col min="10" max="16384" width="10.90625" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="18" x14ac:dyDescent="0.4">
+      <c r="A1" s="3" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="13" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="250.5" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>229</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>229</v>
+      </c>
+      <c r="F4" s="11" t="s">
+        <v>229</v>
+      </c>
+      <c r="G4" s="11" t="s">
+        <v>229</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="42" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="6" t="s">
+        <v>231</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>232</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>233</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>234</v>
+      </c>
+      <c r="H6" s="6" t="s">
+        <v>235</v>
+      </c>
+      <c r="I6" s="6" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="25" x14ac:dyDescent="0.25">
+      <c r="A7" s="19" t="s">
+        <v>237</v>
+      </c>
+      <c r="B7" s="52">
+        <v>9</v>
+      </c>
+      <c r="C7" s="25">
+        <v>35</v>
+      </c>
+      <c r="D7" s="20">
+        <v>3</v>
+      </c>
+      <c r="E7" s="20">
+        <v>3</v>
+      </c>
+      <c r="F7" s="20">
+        <v>2</v>
+      </c>
+      <c r="G7" s="20">
+        <v>1</v>
+      </c>
+      <c r="H7" s="53">
+        <v>0</v>
+      </c>
+      <c r="I7" s="22" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" s="19" t="s">
+        <v>239</v>
+      </c>
+      <c r="B8" s="52">
+        <v>8</v>
+      </c>
+      <c r="C8" s="25">
+        <v>45</v>
+      </c>
+      <c r="D8" s="20">
+        <v>1</v>
+      </c>
+      <c r="E8" s="20">
+        <v>1</v>
+      </c>
+      <c r="F8" s="20">
+        <v>1</v>
+      </c>
+      <c r="G8" s="20">
+        <v>1</v>
+      </c>
+      <c r="H8" s="53">
+        <v>1</v>
+      </c>
+      <c r="I8" s="22" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" s="19" t="s">
+        <v>241</v>
+      </c>
+      <c r="B9" s="52">
+        <v>7</v>
+      </c>
+      <c r="C9" s="25">
+        <v>35</v>
+      </c>
+      <c r="D9" s="20">
+        <v>4</v>
+      </c>
+      <c r="E9" s="20">
+        <v>4</v>
+      </c>
+      <c r="F9" s="20">
+        <v>3</v>
+      </c>
+      <c r="G9" s="20">
+        <v>2</v>
+      </c>
+      <c r="H9" s="53">
+        <v>1</v>
+      </c>
+      <c r="I9" s="22" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" s="19" t="s">
+        <v>243</v>
+      </c>
+      <c r="B10" s="52">
+        <v>7</v>
+      </c>
+      <c r="C10" s="25">
+        <v>35</v>
+      </c>
+      <c r="D10" s="20">
+        <v>1</v>
+      </c>
+      <c r="E10" s="20">
+        <v>1</v>
+      </c>
+      <c r="F10" s="20">
+        <v>1</v>
+      </c>
+      <c r="G10" s="20">
+        <v>1</v>
+      </c>
+      <c r="H10" s="53">
+        <v>1</v>
+      </c>
+      <c r="I10" s="22" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" s="19" t="s">
+        <v>245</v>
+      </c>
+      <c r="B11" s="52">
+        <v>7</v>
+      </c>
+      <c r="C11" s="25">
+        <v>60</v>
+      </c>
+      <c r="D11" s="20">
+        <v>1</v>
+      </c>
+      <c r="E11" s="20">
+        <v>1</v>
+      </c>
+      <c r="F11" s="20">
+        <v>1</v>
+      </c>
+      <c r="G11" s="20">
+        <v>1</v>
+      </c>
+      <c r="H11" s="53">
+        <v>0</v>
+      </c>
+      <c r="I11" s="22" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" s="19" t="s">
+        <v>247</v>
+      </c>
+      <c r="B12" s="52">
+        <v>7</v>
+      </c>
+      <c r="C12" s="25">
+        <v>38</v>
+      </c>
+      <c r="D12" s="20">
+        <v>1</v>
+      </c>
+      <c r="E12" s="20">
+        <v>1</v>
+      </c>
+      <c r="F12" s="20">
+        <v>1</v>
+      </c>
+      <c r="G12" s="20">
+        <v>0</v>
+      </c>
+      <c r="H12" s="53">
+        <v>0</v>
+      </c>
+      <c r="I12" s="22" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" s="19" t="s">
+        <v>249</v>
+      </c>
+      <c r="B13" s="52">
+        <v>7</v>
+      </c>
+      <c r="C13" s="25">
+        <v>30</v>
+      </c>
+      <c r="D13" s="20">
+        <v>2</v>
+      </c>
+      <c r="E13" s="20">
+        <v>2</v>
+      </c>
+      <c r="F13" s="20">
+        <v>2</v>
+      </c>
+      <c r="G13" s="20">
+        <v>1</v>
+      </c>
+      <c r="H13" s="53">
+        <v>0</v>
+      </c>
+      <c r="I13" s="22" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="25" x14ac:dyDescent="0.25">
+      <c r="A14" s="19" t="s">
+        <v>251</v>
+      </c>
+      <c r="B14" s="52">
+        <v>10</v>
+      </c>
+      <c r="C14" s="25">
+        <v>0</v>
+      </c>
+      <c r="D14" s="20">
+        <v>1</v>
+      </c>
+      <c r="E14" s="20">
+        <v>1</v>
+      </c>
+      <c r="F14" s="20">
+        <v>1</v>
+      </c>
+      <c r="G14" s="20">
+        <v>1</v>
+      </c>
+      <c r="H14" s="53">
+        <v>0</v>
+      </c>
+      <c r="I14" s="22" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="25" x14ac:dyDescent="0.25">
+      <c r="A15" s="19" t="s">
+        <v>253</v>
+      </c>
+      <c r="B15" s="52">
+        <v>5</v>
+      </c>
+      <c r="C15" s="25">
+        <v>0</v>
+      </c>
+      <c r="D15" s="20">
+        <v>1</v>
+      </c>
+      <c r="E15" s="20">
+        <v>1</v>
+      </c>
+      <c r="F15" s="20">
+        <v>1</v>
+      </c>
+      <c r="G15" s="20">
+        <v>1</v>
+      </c>
+      <c r="H15" s="53">
+        <v>0</v>
+      </c>
+      <c r="I15" s="22" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="13" x14ac:dyDescent="0.3">
+      <c r="A16" s="4" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="13" x14ac:dyDescent="0.3">
+      <c r="A18" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="B18" s="2"/>
+      <c r="C18" s="2"/>
+      <c r="D18" s="14">
+        <f>SUM(D7:D15)</f>
+        <v>15</v>
+      </c>
+      <c r="E18" s="14">
+        <f>SUM(E7:E15)</f>
+        <v>15</v>
+      </c>
+      <c r="F18" s="14">
+        <f>SUM(F7:F15)</f>
+        <v>13</v>
+      </c>
+      <c r="G18" s="14">
+        <f>SUM(G7:G15)</f>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="13" x14ac:dyDescent="0.3">
+      <c r="A19" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="B19" s="2"/>
+      <c r="C19" s="2"/>
+      <c r="D19" s="14">
+        <f>SUMPRODUCT(D7:D15,$H$7:$H$15)</f>
+        <v>6</v>
+      </c>
+      <c r="E19" s="14">
+        <f>SUMPRODUCT(E7:E15,$H$7:$H$15)</f>
+        <v>6</v>
+      </c>
+      <c r="F19" s="14">
+        <f>SUMPRODUCT(F7:F15,$H$7:$H$15)</f>
+        <v>5</v>
+      </c>
+      <c r="G19" s="14">
+        <f>SUMPRODUCT(G7:G15,$H$7:$H$15)</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="13" x14ac:dyDescent="0.3">
+      <c r="A20" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="B20" s="2"/>
+      <c r="C20" s="2"/>
+      <c r="D20" s="14">
+        <f>SUMPRODUCT(D7:D15,$B$7:$B$15,--($C$7:$C$15&gt;0))-IF(D$4="Restaurant",SUMPRODUCT(D7:D15,$B$7:$B$15,$H$7:$H$15,--($C$7:$C$15&gt;0)),0)</f>
+        <v>98</v>
+      </c>
+      <c r="E20" s="14">
+        <f>SUMPRODUCT(E7:E15,$B$7:$B$15,--($C$7:$C$15&gt;0))-IF(E$4="Restaurant",SUMPRODUCT(E7:E15,$B$7:$B$15,$H$7:$H$15,--($C$7:$C$15&gt;0)),0)</f>
+        <v>98</v>
+      </c>
+      <c r="F20" s="14">
+        <f>SUMPRODUCT(F7:F15,$B$7:$B$15,--($C$7:$C$15&gt;0))-IF(F$4="Restaurant",SUMPRODUCT(F7:F15,$B$7:$B$15,$H$7:$H$15,--($C$7:$C$15&gt;0)),0)</f>
+        <v>82</v>
+      </c>
+      <c r="G20" s="14">
+        <f>SUMPRODUCT(G7:G15,$B$7:$B$15,--($C$7:$C$15&gt;0))-IF(G$4="Restaurant",SUMPRODUCT(G7:G15,$B$7:$B$15,$H$7:$H$15,--($C$7:$C$15&gt;0)),0)</f>
+        <v>52</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="13" x14ac:dyDescent="0.3">
+      <c r="A21" s="45" t="s">
+        <v>259</v>
+      </c>
+      <c r="B21" s="45"/>
+      <c r="C21" s="45"/>
+      <c r="D21" s="46">
+        <f>SUMPRODUCT(D7:D15,$B$7:$B$15,$C$7:$C$15)-IF(D$4="Restaurant",SUMPRODUCT(D7:D15,$B$7:$B$15,$C$7:$C$15,$H$7:$H$15),0)</f>
+        <v>3636</v>
+      </c>
+      <c r="E21" s="46">
+        <f>SUMPRODUCT(E7:E15,$B$7:$B$15,$C$7:$C$15)-IF(E$4="Restaurant",SUMPRODUCT(E7:E15,$B$7:$B$15,$C$7:$C$15,$H$7:$H$15),0)</f>
+        <v>3636</v>
+      </c>
+      <c r="F21" s="46">
+        <f>SUMPRODUCT(F7:F15,$B$7:$B$15,$C$7:$C$15)-IF(F$4="Restaurant",SUMPRODUCT(F7:F15,$B$7:$B$15,$C$7:$C$15,$H$7:$H$15),0)</f>
+        <v>3076</v>
+      </c>
+      <c r="G21" s="46">
+        <f>SUMPRODUCT(G7:G15,$B$7:$B$15,$C$7:$C$15)-IF(G$4="Restaurant",SUMPRODUCT(G7:G15,$B$7:$B$15,$C$7:$C$15,$H$7:$H$15),0)</f>
+        <v>2040</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="13" x14ac:dyDescent="0.3">
+      <c r="A23" s="4" t="s">
+        <v>260</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4:G4" xr:uid="{9B663A6E-5B92-4772-A1ED-AA5999827DF6}">
+      <formula1>"Nous,Restaurant"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62A8117B-BF63-41C1-92C8-4FEDF95C8C14}">
   <dimension ref="A1:P35"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
@@ -2594,23 +3179,23 @@
   <sheetData>
     <row r="1" spans="1:16" ht="18" x14ac:dyDescent="0.4">
       <c r="A1" s="3" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="2" spans="1:16" ht="13" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="3" spans="1:16" ht="13" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C3" s="32">
         <v>46327</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="13" x14ac:dyDescent="0.3">
@@ -2618,7 +3203,7 @@
         <v>31</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C5" s="33">
         <f t="shared" ref="C5:N5" si="0">IF($C$3="","Mois "&amp;(COLUMN()-2),EDATE($C$3,COLUMN()-3))</f>
@@ -2677,7 +3262,7 @@
     </row>
     <row r="6" spans="1:16" ht="13" x14ac:dyDescent="0.3">
       <c r="A6" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="B6" s="10"/>
       <c r="C6" s="10"/>
@@ -2697,7 +3282,7 @@
     </row>
     <row r="7" spans="1:16" ht="13" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B7" s="14">
         <f>SUM(C7:N7)</f>
@@ -2740,15 +3325,15 @@
         <v>0</v>
       </c>
       <c r="O7" s="11" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="P7" s="11" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="8" spans="1:16" ht="13" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B8" s="14">
         <f>SUM(C8:N8)</f>
@@ -2791,15 +3376,15 @@
         <v>1</v>
       </c>
       <c r="O8" s="11" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="P8" s="11" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="9" spans="1:16" ht="13" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B9" s="14">
         <f>SUM(C9:N9)</f>
@@ -2842,15 +3427,15 @@
         <v>0</v>
       </c>
       <c r="O9" s="11" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="P9" s="11" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="10" spans="1:16" ht="13" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B10" s="14">
         <f>SUM(C10:N10)</f>
@@ -2893,15 +3478,15 @@
         <v>2</v>
       </c>
       <c r="O10" s="11" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="P10" s="11" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="11" spans="1:16" ht="13" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B11" s="14">
         <f>SUM(C11:N11)</f>
@@ -2958,7 +3543,7 @@
     </row>
     <row r="12" spans="1:16" ht="13" x14ac:dyDescent="0.3">
       <c r="A12" s="10" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B12" s="10"/>
       <c r="C12" s="10"/>
@@ -2978,7 +3563,7 @@
     </row>
     <row r="13" spans="1:16" ht="13" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B13" s="17">
         <f>SUM(C13:N13)</f>
@@ -3035,11 +3620,11 @@
     </row>
     <row r="14" spans="1:16" ht="13" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B14" s="17">
         <f>SUM(C14:N14)</f>
-        <v>125539.17857142857</v>
+        <v>154313.17857142858</v>
       </c>
       <c r="C14" s="34">
         <f>C7*'Prix et marges'!$C$34+C8*'Prix et marges'!$D$34+C9*'Prix et marges'!$E$34+C10*'Prix et marges'!$F$34</f>
@@ -3051,31 +3636,31 @@
       </c>
       <c r="E14" s="34">
         <f>E7*'Prix et marges'!$C$34+E8*'Prix et marges'!$D$34+E9*'Prix et marges'!$E$34+E10*'Prix et marges'!$F$34</f>
-        <v>5773.7142857142853</v>
+        <v>8539.7142857142862</v>
       </c>
       <c r="F14" s="34">
         <f>F7*'Prix et marges'!$C$34+F8*'Prix et marges'!$D$34+F9*'Prix et marges'!$E$34+F10*'Prix et marges'!$F$34</f>
-        <v>12209.428571428572</v>
+        <v>13935.428571428572</v>
       </c>
       <c r="G14" s="34">
         <f>G7*'Prix et marges'!$C$34+G8*'Prix et marges'!$D$34+G9*'Prix et marges'!$E$34+G10*'Prix et marges'!$F$34</f>
-        <v>7988.25</v>
+        <v>10544.25</v>
       </c>
       <c r="H14" s="34">
         <f>H7*'Prix et marges'!$C$34+H8*'Prix et marges'!$D$34+H9*'Prix et marges'!$E$34+H10*'Prix et marges'!$F$34</f>
-        <v>12577.285714285714</v>
+        <v>16433.285714285714</v>
       </c>
       <c r="I14" s="34">
         <f>I7*'Prix et marges'!$C$34+I8*'Prix et marges'!$D$34+I9*'Prix et marges'!$E$34+I10*'Prix et marges'!$F$34</f>
-        <v>19013</v>
+        <v>21829</v>
       </c>
       <c r="J14" s="34">
         <f>J7*'Prix et marges'!$C$34+J8*'Prix et marges'!$D$34+J9*'Prix et marges'!$E$34+J10*'Prix et marges'!$F$34</f>
-        <v>14791.821428571428</v>
+        <v>18437.821428571428</v>
       </c>
       <c r="K14" s="34">
         <f>K7*'Prix et marges'!$C$34+K8*'Prix et marges'!$D$34+K9*'Prix et marges'!$E$34+K10*'Prix et marges'!$F$34</f>
-        <v>5773.7142857142853</v>
+        <v>8539.7142857142862</v>
       </c>
       <c r="L14" s="34">
         <f>L7*'Prix et marges'!$C$34+L8*'Prix et marges'!$D$34+L9*'Prix et marges'!$E$34+L10*'Prix et marges'!$F$34</f>
@@ -3083,20 +3668,20 @@
       </c>
       <c r="M14" s="34">
         <f>M7*'Prix et marges'!$C$34+M8*'Prix et marges'!$D$34+M9*'Prix et marges'!$E$34+M10*'Prix et marges'!$F$34</f>
-        <v>25816.571428571428</v>
+        <v>29722.571428571428</v>
       </c>
       <c r="N14" s="34">
         <f>N7*'Prix et marges'!$C$34+N8*'Prix et marges'!$D$34+N9*'Prix et marges'!$E$34+N10*'Prix et marges'!$F$34</f>
-        <v>21595.392857142855</v>
+        <v>26331.392857142855</v>
       </c>
     </row>
     <row r="15" spans="1:16" ht="13" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B15" s="17">
         <f>SUM(C15:N15)</f>
-        <v>-3583.8214285714357</v>
+        <v>-32357.821428571442</v>
       </c>
       <c r="C15" s="17">
         <f t="shared" ref="C15:N15" si="2">C13-C14</f>
@@ -3108,31 +3693,31 @@
       </c>
       <c r="E15" s="17">
         <f t="shared" si="2"/>
-        <v>-854.07142857142935</v>
+        <v>-3620.0714285714303</v>
       </c>
       <c r="F15" s="17">
         <f t="shared" si="2"/>
-        <v>-2352.2857142857156</v>
+        <v>-4078.2857142857156</v>
       </c>
       <c r="G15" s="17">
         <f t="shared" si="2"/>
-        <v>-863.25000000000091</v>
+        <v>-3419.2500000000009</v>
       </c>
       <c r="H15" s="17">
         <f t="shared" si="2"/>
-        <v>378.07142857142753</v>
+        <v>-3477.9285714285725</v>
       </c>
       <c r="I15" s="17">
         <f t="shared" si="2"/>
-        <v>-1120.1428571428587</v>
+        <v>-3936.1428571428587</v>
       </c>
       <c r="J15" s="17">
         <f t="shared" si="2"/>
-        <v>368.89285714285688</v>
+        <v>-3277.1071428571431</v>
       </c>
       <c r="K15" s="17">
         <f t="shared" si="2"/>
-        <v>-854.07142857142935</v>
+        <v>-3620.0714285714303</v>
       </c>
       <c r="L15" s="17">
         <f t="shared" si="2"/>
@@ -3140,16 +3725,16 @@
       </c>
       <c r="M15" s="17">
         <f t="shared" si="2"/>
-        <v>112</v>
+        <v>-3794</v>
       </c>
       <c r="N15" s="17">
         <f t="shared" si="2"/>
-        <v>1601.0357142857138</v>
+        <v>-3134.9642857142862</v>
       </c>
     </row>
     <row r="16" spans="1:16" ht="13" x14ac:dyDescent="0.3">
       <c r="A16" s="10" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B16" s="10"/>
       <c r="C16" s="10"/>
@@ -3169,10 +3754,10 @@
     </row>
     <row r="17" spans="1:16" ht="13" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B17" s="17">
-        <f t="shared" ref="B17:B32" si="3">SUM(C17:N17)</f>
+        <f t="shared" ref="B17:B30" si="3">SUM(C17:N17)</f>
         <v>0</v>
       </c>
       <c r="C17" s="15">
@@ -3212,15 +3797,15 @@
         <v>0</v>
       </c>
       <c r="O17" s="11" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="P17" s="11" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="18" spans="1:16" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B18" s="42">
         <f>SUM(C18:N18)</f>
@@ -3263,15 +3848,15 @@
         <v>0</v>
       </c>
       <c r="O18" s="40" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="P18" s="40" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
     </row>
     <row r="19" spans="1:16" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="B19" s="42">
         <f>SUM(C19:N19)</f>
@@ -3314,15 +3899,15 @@
         <v>0</v>
       </c>
       <c r="O19" s="40" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="P19" s="40" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
     </row>
     <row r="20" spans="1:16" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B20" s="42">
         <f>SUM(C20:N20)</f>
@@ -3365,15 +3950,15 @@
         <v>0</v>
       </c>
       <c r="O20" s="40" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="P20" s="40" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
     </row>
     <row r="21" spans="1:16" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A21" s="44" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="B21" s="42">
         <f>SUM(C21:N21)</f>
@@ -3430,7 +4015,7 @@
     </row>
     <row r="22" spans="1:16" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A22" s="43" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B22" s="43"/>
       <c r="C22" s="43"/>
@@ -3450,7 +4035,7 @@
     </row>
     <row r="23" spans="1:16" ht="13" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B23" s="17">
         <f t="shared" si="3"/>
@@ -3493,15 +4078,15 @@
         <v>0</v>
       </c>
       <c r="O23" s="11" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="P23" s="11" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="24" spans="1:16" ht="13" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B24" s="17">
         <f t="shared" si="3"/>
@@ -3544,15 +4129,15 @@
         <v>80</v>
       </c>
       <c r="O24" s="11" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="P24" s="11" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="25" spans="1:16" ht="13" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B25" s="17">
         <f t="shared" si="3"/>
@@ -3595,15 +4180,15 @@
         <v>300</v>
       </c>
       <c r="O25" s="11" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="P25" s="11" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="26" spans="1:16" ht="13" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B26" s="17">
         <f t="shared" si="3"/>
@@ -3646,15 +4231,15 @@
         <v>50</v>
       </c>
       <c r="O26" s="11" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="P26" s="11" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
     </row>
     <row r="27" spans="1:16" ht="13" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B27" s="17">
         <f t="shared" si="3"/>
@@ -3697,15 +4282,15 @@
         <v>100</v>
       </c>
       <c r="O27" s="11" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="P27" s="11" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
     </row>
     <row r="28" spans="1:16" ht="13" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B28" s="17">
         <f t="shared" si="3"/>
@@ -3748,15 +4333,15 @@
         <v>30</v>
       </c>
       <c r="O28" s="11" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="P28" s="11" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="29" spans="1:16" ht="13" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B29" s="17">
         <f t="shared" si="3"/>
@@ -3799,15 +4384,15 @@
         <v>50</v>
       </c>
       <c r="O29" s="11" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="P29" s="11" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
     <row r="30" spans="1:16" ht="13" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B30" s="17">
         <f t="shared" si="3"/>
@@ -3850,15 +4435,15 @@
         <v>0</v>
       </c>
       <c r="O30" s="11" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="P30" s="11" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="31" spans="1:16" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A31" s="44" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="B31" s="42">
         <f>SUM(C31:N31)</f>
@@ -3915,7 +4500,7 @@
     </row>
     <row r="32" spans="1:16" ht="13" x14ac:dyDescent="0.3">
       <c r="A32" s="45" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B32" s="46">
         <f>SUM(C32:N32)</f>
@@ -3972,7 +4557,7 @@
     </row>
     <row r="33" spans="1:16" ht="13" x14ac:dyDescent="0.3">
       <c r="A33" s="10" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B33" s="10"/>
       <c r="C33" s="10"/>
@@ -3992,11 +4577,11 @@
     </row>
     <row r="34" spans="1:16" ht="13" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B34" s="17">
         <f>SUM(C34:N34)</f>
-        <v>-16255.821428571435</v>
+        <v>-45029.821428571435</v>
       </c>
       <c r="C34" s="17">
         <f t="shared" ref="C34:N34" si="7">C15-C32</f>
@@ -4008,31 +4593,31 @@
       </c>
       <c r="E34" s="17">
         <f t="shared" si="7"/>
-        <v>-2664.0714285714294</v>
+        <v>-5430.0714285714303</v>
       </c>
       <c r="F34" s="17">
         <f t="shared" si="7"/>
-        <v>-4162.2857142857156</v>
+        <v>-5888.2857142857156</v>
       </c>
       <c r="G34" s="17">
         <f t="shared" si="7"/>
-        <v>-1473.2500000000009</v>
+        <v>-4029.2500000000009</v>
       </c>
       <c r="H34" s="17">
         <f t="shared" si="7"/>
-        <v>-231.92857142857247</v>
+        <v>-4087.9285714285725</v>
       </c>
       <c r="I34" s="17">
         <f t="shared" si="7"/>
-        <v>-1730.1428571428587</v>
+        <v>-4546.1428571428587</v>
       </c>
       <c r="J34" s="17">
         <f t="shared" si="7"/>
-        <v>-241.10714285714312</v>
+        <v>-3887.1071428571431</v>
       </c>
       <c r="K34" s="17">
         <f t="shared" si="7"/>
-        <v>-1464.0714285714294</v>
+        <v>-4230.0714285714303</v>
       </c>
       <c r="L34" s="17">
         <f t="shared" si="7"/>
@@ -4040,20 +4625,20 @@
       </c>
       <c r="M34" s="17">
         <f t="shared" si="7"/>
-        <v>-498</v>
+        <v>-4404</v>
       </c>
       <c r="N34" s="17">
         <f t="shared" si="7"/>
-        <v>991.03571428571377</v>
+        <v>-3744.9642857142862</v>
       </c>
     </row>
     <row r="35" spans="1:16" ht="13" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="B35" s="17">
         <f>N35</f>
-        <v>-16255.821428571435</v>
+        <v>-45029.821428571435</v>
       </c>
       <c r="C35" s="17">
         <f>C34</f>
@@ -4065,43 +4650,43 @@
       </c>
       <c r="E35" s="17">
         <f t="shared" si="8"/>
-        <v>-6836.0714285714294</v>
+        <v>-9602.0714285714312</v>
       </c>
       <c r="F35" s="17">
         <f t="shared" si="8"/>
-        <v>-10998.357142857145</v>
+        <v>-15490.357142857147</v>
       </c>
       <c r="G35" s="17">
         <f t="shared" si="8"/>
-        <v>-12471.607142857145</v>
+        <v>-19519.607142857149</v>
       </c>
       <c r="H35" s="17">
         <f t="shared" si="8"/>
-        <v>-12703.535714285717</v>
+        <v>-23607.535714285721</v>
       </c>
       <c r="I35" s="17">
         <f t="shared" si="8"/>
-        <v>-14433.678571428576</v>
+        <v>-28153.67857142858</v>
       </c>
       <c r="J35" s="17">
         <f t="shared" si="8"/>
-        <v>-14674.785714285719</v>
+        <v>-32040.785714285725</v>
       </c>
       <c r="K35" s="17">
         <f t="shared" si="8"/>
-        <v>-16138.857142857149</v>
+        <v>-36270.857142857152</v>
       </c>
       <c r="L35" s="17">
         <f t="shared" si="8"/>
-        <v>-16748.857142857149</v>
+        <v>-36880.857142857152</v>
       </c>
       <c r="M35" s="17">
         <f t="shared" si="8"/>
-        <v>-17246.857142857149</v>
+        <v>-41284.857142857152</v>
       </c>
       <c r="N35" s="17">
         <f t="shared" si="8"/>
-        <v>-16255.821428571435</v>
+        <v>-45029.821428571435</v>
       </c>
     </row>
   </sheetData>
@@ -4114,7 +4699,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9898DBE-F173-4946-8908-F62FA6ACEF06}">
   <dimension ref="A1:N27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
@@ -4127,20 +4712,20 @@
   <sheetData>
     <row r="1" spans="1:14" ht="18" x14ac:dyDescent="0.4">
       <c r="A1" s="3" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="2" spans="1:14" ht="13" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="5" spans="1:14" ht="13" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C5" s="33">
         <f>IF('Budget mensuel'!$C$3="","Mois "&amp;(COLUMN()-2),EDATE('Budget mensuel'!$C$3,COLUMN()-3))</f>
@@ -4193,7 +4778,7 @@
     </row>
     <row r="6" spans="1:14" ht="13" x14ac:dyDescent="0.3">
       <c r="A6" s="10" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="B6" s="10"/>
       <c r="C6" s="10"/>
@@ -4211,7 +4796,7 @@
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B7" s="13">
         <f>SUM(C7:N7)</f>
@@ -4268,7 +4853,7 @@
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B8" s="13">
         <f>SUM(C8:N8)</f>
@@ -4289,7 +4874,7 @@
     </row>
     <row r="9" spans="1:14" ht="13" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B9" s="14">
         <f>SUM(C9:N9)</f>
@@ -4346,7 +4931,7 @@
     </row>
     <row r="11" spans="1:14" ht="13" x14ac:dyDescent="0.3">
       <c r="A11" s="10" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B11" s="10"/>
       <c r="C11" s="10"/>
@@ -4364,7 +4949,7 @@
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B12" s="16">
         <f>SUM(C12:N12)</f>
@@ -4421,7 +5006,7 @@
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B13" s="16">
         <f>SUM(C13:N13)</f>
@@ -4442,7 +5027,7 @@
     </row>
     <row r="14" spans="1:14" ht="13" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B14" s="17">
         <f>SUM(C14:N14)</f>
@@ -4499,7 +5084,7 @@
     </row>
     <row r="16" spans="1:14" ht="13" x14ac:dyDescent="0.3">
       <c r="A16" s="10" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B16" s="10"/>
       <c r="C16" s="10"/>
@@ -4517,7 +5102,7 @@
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B17" s="16">
         <f>SUM(C17:N17)</f>
@@ -4574,7 +5159,7 @@
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B18" s="16">
         <f>SUM(C18:N18)</f>
@@ -4595,7 +5180,7 @@
     </row>
     <row r="19" spans="1:14" ht="13" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B19" s="17">
         <f>SUM(C19:N19)</f>
@@ -4652,7 +5237,7 @@
     </row>
     <row r="21" spans="1:14" ht="13" x14ac:dyDescent="0.3">
       <c r="A21" s="10" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="B21" s="10"/>
       <c r="C21" s="10"/>
@@ -4670,11 +5255,11 @@
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B22" s="16">
         <f>SUM(C22:N22)</f>
-        <v>-16255.821428571435</v>
+        <v>-45029.821428571435</v>
       </c>
       <c r="C22" s="36">
         <f>'Budget mensuel'!C34</f>
@@ -4686,31 +5271,31 @@
       </c>
       <c r="E22" s="36">
         <f>'Budget mensuel'!E34</f>
-        <v>-2664.0714285714294</v>
+        <v>-5430.0714285714303</v>
       </c>
       <c r="F22" s="36">
         <f>'Budget mensuel'!F34</f>
-        <v>-4162.2857142857156</v>
+        <v>-5888.2857142857156</v>
       </c>
       <c r="G22" s="36">
         <f>'Budget mensuel'!G34</f>
-        <v>-1473.2500000000009</v>
+        <v>-4029.2500000000009</v>
       </c>
       <c r="H22" s="36">
         <f>'Budget mensuel'!H34</f>
-        <v>-231.92857142857247</v>
+        <v>-4087.9285714285725</v>
       </c>
       <c r="I22" s="36">
         <f>'Budget mensuel'!I34</f>
-        <v>-1730.1428571428587</v>
+        <v>-4546.1428571428587</v>
       </c>
       <c r="J22" s="36">
         <f>'Budget mensuel'!J34</f>
-        <v>-241.10714285714312</v>
+        <v>-3887.1071428571431</v>
       </c>
       <c r="K22" s="36">
         <f>'Budget mensuel'!K34</f>
-        <v>-1464.0714285714294</v>
+        <v>-4230.0714285714303</v>
       </c>
       <c r="L22" s="36">
         <f>'Budget mensuel'!L34</f>
@@ -4718,16 +5303,16 @@
       </c>
       <c r="M22" s="36">
         <f>'Budget mensuel'!M34</f>
-        <v>-498</v>
+        <v>-4404</v>
       </c>
       <c r="N22" s="36">
         <f>'Budget mensuel'!N34</f>
-        <v>991.03571428571377</v>
+        <v>-3744.9642857142862</v>
       </c>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B23" s="16">
         <f>SUM(C23:N23)</f>
@@ -4748,7 +5333,7 @@
     </row>
     <row r="24" spans="1:14" ht="13" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B24" s="17">
         <f>SUM(C24:N24)</f>
@@ -4805,7 +5390,7 @@
     </row>
     <row r="26" spans="1:14" ht="13" x14ac:dyDescent="0.3">
       <c r="A26" s="10" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="B26" s="10"/>
       <c r="C26" s="10"/>
@@ -4823,7 +5408,7 @@
     </row>
     <row r="27" spans="1:14" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="7" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="C27" s="18"/>
       <c r="D27" s="18"/>
@@ -4843,7 +5428,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42FB26B6-A531-4D48-8F04-B3463A220999}">
   <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
@@ -4858,12 +5443,12 @@
   <sheetData>
     <row r="1" spans="1:7" ht="18" x14ac:dyDescent="0.4">
       <c r="A1" s="3" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="13" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="13" x14ac:dyDescent="0.25">
@@ -4874,13 +5459,13 @@
         <v>32</v>
       </c>
       <c r="C5" s="6" t="s">
+        <v>161</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="E5" s="6" t="s">
         <v>163</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>164</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>165</v>
       </c>
       <c r="F5" s="6" t="s">
         <v>37</v>
@@ -4891,7 +5476,7 @@
     </row>
     <row r="6" spans="1:7" ht="13" x14ac:dyDescent="0.3">
       <c r="A6" s="10" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="B6" s="10"/>
       <c r="C6" s="10"/>
@@ -4902,10 +5487,10 @@
     </row>
     <row r="7" spans="1:7" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A7" s="19" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C7" s="37">
         <f>'Budget mensuel'!$B$7</f>
@@ -4918,18 +5503,18 @@
         <v>12</v>
       </c>
       <c r="F7" s="21" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G7" s="22" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A8" s="19" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C8" s="37">
         <f>'Budget mensuel'!$B$8</f>
@@ -4942,18 +5527,18 @@
         <v>12</v>
       </c>
       <c r="F8" s="21" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G8" s="22" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A9" s="19" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C9" s="37">
         <f>'Budget mensuel'!$B$9</f>
@@ -4966,18 +5551,18 @@
         <v>12</v>
       </c>
       <c r="F9" s="21" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G9" s="22" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A10" s="19" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="B10" s="19" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C10" s="37">
         <f>'Budget mensuel'!$B$10</f>
@@ -4990,18 +5575,18 @@
         <v>48</v>
       </c>
       <c r="F10" s="21" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G10" s="22" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="13" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C11" s="24">
         <f t="shared" ref="C11:E11" si="0">SUM(C7:C10)</f>
@@ -5020,7 +5605,7 @@
     </row>
     <row r="12" spans="1:7" ht="13" x14ac:dyDescent="0.25">
       <c r="A12" s="29" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="B12" s="29"/>
       <c r="C12" s="29"/>
@@ -5031,7 +5616,7 @@
     </row>
     <row r="13" spans="1:7" ht="13" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B13" s="8" t="s">
         <v>56</v>
@@ -5053,76 +5638,76 @@
     </row>
     <row r="14" spans="1:7" ht="13" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B14" s="8" t="s">
         <v>56</v>
       </c>
       <c r="C14" s="38">
         <f>C7*'Prix et marges'!$C$34+C8*'Prix et marges'!$D$34+C9*'Prix et marges'!$E$34+C10*'Prix et marges'!$F$34</f>
-        <v>125539.17857142858</v>
+        <v>154313.17857142858</v>
       </c>
       <c r="D14" s="38">
         <f>D7*'Prix et marges'!$C$34+D8*'Prix et marges'!$D$34+D9*'Prix et marges'!$E$34+D10*'Prix et marges'!$F$34</f>
-        <v>371056.85714285716</v>
+        <v>453600.85714285716</v>
       </c>
       <c r="E14" s="38">
         <f>E7*'Prix et marges'!$C$34+E8*'Prix et marges'!$D$34+E9*'Prix et marges'!$E$34+E10*'Prix et marges'!$F$34</f>
-        <v>638228.14285714296</v>
+        <v>775124.14285714296</v>
       </c>
       <c r="F14" s="21"/>
       <c r="G14" s="22"/>
     </row>
     <row r="15" spans="1:7" ht="13" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B15" s="8" t="s">
         <v>56</v>
       </c>
       <c r="C15" s="28">
         <f t="shared" ref="C15:E15" si="1">C13-C14</f>
-        <v>-3583.8214285714494</v>
+        <v>-32357.821428571449</v>
       </c>
       <c r="D15" s="28">
         <f t="shared" si="1"/>
-        <v>-2985.428571428638</v>
+        <v>-85529.428571428638</v>
       </c>
       <c r="E15" s="28">
         <f t="shared" si="1"/>
-        <v>10307.571428571246</v>
+        <v>-126588.42857142875</v>
       </c>
       <c r="F15" s="21"/>
       <c r="G15" s="22"/>
     </row>
     <row r="16" spans="1:7" ht="13" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B16" s="8" t="s">
         <v>64</v>
       </c>
       <c r="C16" s="31">
         <f t="shared" ref="C16:E16" si="2">IF(C13&gt;0,C15/C13,0)</f>
-        <v>-2.9386338677795033E-2</v>
+        <v>-0.26532513361153837</v>
       </c>
       <c r="D16" s="31">
         <f t="shared" si="2"/>
-        <v>-8.1110032990492787E-3</v>
+        <v>-0.23237182223947236</v>
       </c>
       <c r="E16" s="31">
         <f t="shared" si="2"/>
-        <v>1.589360647612726E-2</v>
+        <v>-0.19519114488683328</v>
       </c>
       <c r="F16" s="21"/>
       <c r="G16" s="22"/>
     </row>
     <row r="17" spans="1:7" customFormat="1" ht="29" x14ac:dyDescent="0.35">
-      <c r="A17" s="51" t="s">
-        <v>221</v>
-      </c>
-      <c r="B17" s="51" t="s">
-        <v>170</v>
+      <c r="A17" t="s">
+        <v>219</v>
+      </c>
+      <c r="B17" t="s">
+        <v>168</v>
       </c>
       <c r="C17" s="50">
         <f>'Budget mensuel'!$B$21</f>
@@ -5137,18 +5722,18 @@
         <v>168206.14799999999</v>
       </c>
       <c r="F17" s="40" t="s">
-        <v>90</v>
-      </c>
-      <c r="G17" s="52" t="s">
-        <v>223</v>
+        <v>89</v>
+      </c>
+      <c r="G17" s="51" t="s">
+        <v>221</v>
       </c>
     </row>
     <row r="18" spans="1:7" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A18" s="51" t="s">
-        <v>222</v>
-      </c>
-      <c r="B18" s="51" t="s">
-        <v>170</v>
+      <c r="A18" t="s">
+        <v>220</v>
+      </c>
+      <c r="B18" t="s">
+        <v>168</v>
       </c>
       <c r="C18" s="50">
         <f>'Budget mensuel'!$B$31</f>
@@ -5163,18 +5748,18 @@
         <v>57800</v>
       </c>
       <c r="F18" s="40" t="s">
-        <v>90</v>
-      </c>
-      <c r="G18" s="52" t="s">
-        <v>224</v>
+        <v>89</v>
+      </c>
+      <c r="G18" s="51" t="s">
+        <v>222</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="13" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C19" s="28">
         <f t="shared" ref="C19:E19" si="3">C17+C18</f>
@@ -5190,34 +5775,34 @@
       </c>
       <c r="F19" s="21"/>
       <c r="G19" s="22" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="13" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="B20" s="8" t="s">
         <v>56</v>
       </c>
       <c r="C20" s="28">
         <f t="shared" ref="C20:E20" si="4">C15-C19</f>
-        <v>-16255.821428571449</v>
+        <v>-45029.821428571449</v>
       </c>
       <c r="D20" s="28">
         <f t="shared" si="4"/>
-        <v>-59771.576571428639</v>
+        <v>-142315.57657142862</v>
       </c>
       <c r="E20" s="28">
         <f t="shared" si="4"/>
-        <v>-215698.57657142874</v>
+        <v>-352594.57657142874</v>
       </c>
       <c r="F20" s="21"/>
       <c r="G20" s="22"/>
     </row>
     <row r="21" spans="1:7" ht="13" x14ac:dyDescent="0.25">
       <c r="A21" s="29" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B21" s="29"/>
       <c r="C21" s="29"/>
@@ -5228,7 +5813,7 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="19" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="B22" s="19" t="s">
         <v>56</v>
@@ -5243,62 +5828,62 @@
         <v>10000</v>
       </c>
       <c r="F22" s="21" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G22" s="22" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="13" x14ac:dyDescent="0.25">
       <c r="A23" s="8" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="C23" s="28">
         <f t="shared" ref="C23:E23" si="5">C20-C22</f>
-        <v>-19255.821428571449</v>
+        <v>-48029.821428571449</v>
       </c>
       <c r="D23" s="28">
         <f t="shared" si="5"/>
-        <v>-64771.576571428639</v>
+        <v>-147315.57657142862</v>
       </c>
       <c r="E23" s="28">
         <f t="shared" si="5"/>
-        <v>-225698.57657142874</v>
+        <v>-362594.57657142874</v>
       </c>
       <c r="F23" s="21"/>
       <c r="G23" s="22"/>
     </row>
     <row r="24" spans="1:7" ht="13" x14ac:dyDescent="0.25">
       <c r="A24" s="8" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="C24" s="28">
         <f>C23</f>
-        <v>-19255.821428571449</v>
+        <v>-48029.821428571449</v>
       </c>
       <c r="D24" s="28">
         <f t="shared" ref="D24:E24" si="6">C24+D23</f>
-        <v>-84027.398000000088</v>
+        <v>-195345.39800000007</v>
       </c>
       <c r="E24" s="28">
         <f t="shared" si="6"/>
-        <v>-309725.97457142884</v>
+        <v>-557939.97457142884</v>
       </c>
       <c r="F24" s="21"/>
       <c r="G24" s="22"/>
     </row>
     <row r="25" spans="1:7" ht="13" x14ac:dyDescent="0.25">
       <c r="A25" s="8" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C25" s="39">
         <f t="shared" ref="C25:E25" si="7">IF(C11&gt;0,IF(C15&gt;0,C19/(C15/C11),0),0)</f>
@@ -5310,26 +5895,26 @@
       </c>
       <c r="E25" s="39">
         <f t="shared" si="7"/>
-        <v>1841.8030438651526</v>
+        <v>0</v>
       </c>
       <c r="F25" s="21"/>
       <c r="G25" s="22"/>
     </row>
     <row r="27" spans="1:7" ht="13" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="C27" s="17">
         <f>MAX(0,-MIN(C24:E24))</f>
-        <v>309725.97457142884</v>
+        <v>557939.97457142884</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="13" x14ac:dyDescent="0.3">
       <c r="A29" s="4" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
   </sheetData>
@@ -5342,7 +5927,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C299EF4-2BFD-4A30-9CB8-0FD18304D49C}">
   <dimension ref="A1:I27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
@@ -5359,28 +5944,28 @@
   <sheetData>
     <row r="1" spans="1:9" ht="18" x14ac:dyDescent="0.4">
       <c r="A1" s="3" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="13" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="13" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C4" s="47">
         <v>0.45</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="13" x14ac:dyDescent="0.3">
       <c r="A6" s="10" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B6" s="10"/>
       <c r="C6" s="10"/>
@@ -5396,22 +5981,22 @@
         <v>31</v>
       </c>
       <c r="B7" s="6" t="s">
+        <v>196</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>197</v>
+      </c>
+      <c r="D7" s="6" t="s">
         <v>198</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="E7" s="6" t="s">
         <v>199</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="F7" s="6" t="s">
         <v>200</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="G7" s="6" t="s">
         <v>201</v>
-      </c>
-      <c r="F7" s="6" t="s">
-        <v>202</v>
-      </c>
-      <c r="G7" s="6" t="s">
-        <v>203</v>
       </c>
       <c r="H7" s="6" t="s">
         <v>37</v>
@@ -5422,7 +6007,7 @@
     </row>
     <row r="8" spans="1:9" ht="25" x14ac:dyDescent="0.25">
       <c r="A8" s="21" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="B8" s="20">
         <v>2</v>
@@ -5445,15 +6030,15 @@
         <v>87000</v>
       </c>
       <c r="H8" s="21" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I8" s="22" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="25" x14ac:dyDescent="0.25">
       <c r="A9" s="21" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="B9" s="20">
         <v>1</v>
@@ -5476,15 +6061,15 @@
         <v>32486.147999999997</v>
       </c>
       <c r="H9" s="21" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I9" s="22" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="25" x14ac:dyDescent="0.25">
       <c r="A10" s="21" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="B10" s="20">
         <v>1</v>
@@ -5507,10 +6092,10 @@
         <v>48720</v>
       </c>
       <c r="H10" s="21" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I10" s="22" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
@@ -5549,7 +6134,7 @@
     </row>
     <row r="13" spans="1:9" ht="13" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="B13" s="24">
         <f>SUM(B8:B12)</f>
@@ -5582,7 +6167,7 @@
     </row>
     <row r="15" spans="1:9" ht="13" x14ac:dyDescent="0.25">
       <c r="A15" s="29" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="B15" s="29"/>
       <c r="C15" s="29"/>
@@ -5602,10 +6187,10 @@
       <c r="D16" s="49"/>
       <c r="E16" s="49"/>
       <c r="F16" s="49" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="G16" s="49" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="H16" s="49" t="s">
         <v>37</v>
@@ -5616,7 +6201,7 @@
     </row>
     <row r="17" spans="1:9" ht="25" x14ac:dyDescent="0.25">
       <c r="A17" s="19" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B17" s="19"/>
       <c r="C17" s="19"/>
@@ -5629,15 +6214,15 @@
         <v>10800</v>
       </c>
       <c r="H17" s="21" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I17" s="22" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="19" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="B18" s="19"/>
       <c r="C18" s="19"/>
@@ -5650,15 +6235,15 @@
         <v>3000</v>
       </c>
       <c r="H18" s="21" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I18" s="22" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="19" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B19" s="19"/>
       <c r="C19" s="19"/>
@@ -5671,15 +6256,15 @@
         <v>30000</v>
       </c>
       <c r="H19" s="21" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I19" s="22" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="25" x14ac:dyDescent="0.25">
       <c r="A20" s="19" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B20" s="19"/>
       <c r="C20" s="19"/>
@@ -5692,15 +6277,15 @@
         <v>2000</v>
       </c>
       <c r="H20" s="21" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I20" s="22" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="19" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B21" s="19"/>
       <c r="C21" s="19"/>
@@ -5713,15 +6298,15 @@
         <v>6000</v>
       </c>
       <c r="H21" s="21" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I21" s="22" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="19" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B22" s="19"/>
       <c r="C22" s="19"/>
@@ -5734,15 +6319,15 @@
         <v>1000</v>
       </c>
       <c r="H22" s="21" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I22" s="22" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="19" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B23" s="19"/>
       <c r="C23" s="19"/>
@@ -5755,15 +6340,15 @@
         <v>4000</v>
       </c>
       <c r="H23" s="21" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I23" s="22" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="19" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="B24" s="19"/>
       <c r="C24" s="19"/>
@@ -5776,15 +6361,15 @@
         <v>1000</v>
       </c>
       <c r="H24" s="21" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I24" s="22" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="25" spans="1:9" ht="13" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="B25" s="2"/>
       <c r="C25" s="2"/>
@@ -5801,7 +6386,7 @@
     </row>
     <row r="27" spans="1:9" ht="13" x14ac:dyDescent="0.3">
       <c r="A27" s="45" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B27" s="45"/>
       <c r="C27" s="45"/>

</xml_diff>

<commit_message>
Finance : scénario de staffing S3 des Opérations retenu (28/10/2026)
- Staffing : personnel toujours fourni par nous ; effectifs S3 pour les soirées récurrentes, S0 pour les pilotes
- Budget : surcoût d'équipe des deux pilotes (1 155 €) ajouté aux coûts directs
- Trésorerie et tableau de bord recalculés ; fiche des données manquantes et README mis à jour

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/2 FINANCE/PREVISIONS/2026 1027 Modèle - Budget, plan financier, prix et marges.xlsx
+++ b/2 FINANCE/PREVISIONS/2026 1027 Modèle - Budget, plan financier, prix et marges.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vians\Documents\Claude\Projects\HEC-GEMM-Groupe-7\2 FINANCE\PREVISIONS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CCD5C6A-B0F7-4AAD-B84C-98FD8DDC5033}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98E0FF28-2BF8-4335-BED1-F9CA1EC27576}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{09426CC5-4BCC-48B7-8854-C5C8E2CE30D1}"/>
   </bookViews>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="428" uniqueCount="266">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="461" uniqueCount="287">
   <si>
     <t>Prévisions — budget, plan financier, prix et marges</t>
   </si>
@@ -725,24 +725,6 @@
     <t>Mis à jour le 28/10/2026 : frais généraux divisés en ressources humaines (fondateurs, salariés, charges sociales, stagiaires et indépendants) et frais matériels et de fonctionnement (locaux, outils, marketing, assurance, honoraires, banque, déplacements, autres). Année 1 : budget mensuel. Années 2 et 3 : onglet « Frais généraux 3 ans ».</t>
   </si>
   <si>
-    <t>Staffing d'une soirée : effectifs des Opérations × heures × coût horaire</t>
-  </si>
-  <si>
-    <t>Effectifs repris du calculateur des Opérations (propositions, catégorie C2). Heures et coûts horaires : hypothèses temporaires, aucun devis à ce jour.</t>
-  </si>
-  <si>
-    <t>Service de salle fourni par :</t>
-  </si>
-  <si>
-    <t>Nous</t>
-  </si>
-  <si>
-    <t>Question non tranchée (Produit, pricing point 3 ; Opérations, note § 3.4). « Restaurant » sort les postes de salle du coût ; la part du restaurateur (Prix et marges, ligne 19) devrait alors augmenter.</t>
-  </si>
-  <si>
-    <t>Rôle</t>
-  </si>
-  <si>
     <t>Heures par personne</t>
   </si>
   <si>
@@ -824,18 +806,9 @@
     <t>Heures de travail payées</t>
   </si>
   <si>
-    <t>Coût de l'équipe de la soirée (€ HT)</t>
-  </si>
-  <si>
-    <t>Source des effectifs : 6 OPERATIONS/PRODUCTION/2026 1028 Calculateur de staffing par événement.xlsx et 2026 1028 Typologie des événements, process et staffing.md (Opérations, 28/10/2026 ; colonnes Pilote 1, Le Voyage, Pilote 2 et Table d'affaires). Pour une soirée récurrente en criticité C1, le serveur de réserve et l'interlocuteur client ne sont pas nécessaires.</t>
-  </si>
-  <si>
     <t>P / H</t>
   </si>
   <si>
-    <t>Onglet Staffing : effectifs des Opérations (P, 6 OPERATIONS/PRODUCTION/2026 1028 Calculateur de staffing par événement.xlsx et 2026 1028 Typologie des événements, process et staffing.md) × heures et coûts horaires (H). Remplace la cible du Produit (14 / 12 / 11 % du prix HT) utilisée le 27/10/2026</t>
-  </si>
-  <si>
     <t>Équipe de service, brigade, sommelier et plonge</t>
   </si>
   <si>
@@ -843,6 +816,96 @@
   </si>
   <si>
     <t>Mis à jour le 28/10/2026 : le coût de l'équipe de chaque soirée (Prix et marges, ligne 26) est calculé dans l'onglet « Staffing » à partir des effectifs proposés par les Opérations (6 OPERATIONS/PRODUCTION/2026 1028 Calculateur de staffing par événement.xlsx et 2026 1028 Typologie des événements, process et staffing.md), multipliés par des heures et des coûts horaires en hypothèse (H). Le choix « service de salle fourni par le restaurant » y est modifiable.</t>
+  </si>
+  <si>
+    <t>Staffing d'une soirée : scénario S0 (pilotes) et scénario S3 (soirées récurrentes)</t>
+  </si>
+  <si>
+    <t>Effectifs repris des Opérations (propositions). Heures et coûts horaires : hypothèses temporaires (H), aucun devis à ce jour.</t>
+  </si>
+  <si>
+    <t>Personnel de la soirée (salle, sommellerie, brigade, plonge) : toujours fourni et payé par Fou d'un soir.</t>
+  </si>
+  <si>
+    <t>Orientation du responsable Opérations du 28/10/2026, à porter au registre des décisions par la Direction (6 OPERATIONS/PRODUCTION/2026 1028 Scénarios de staffing - leviers de coût.md, § 3). Remplace l'option « salle fournie par le restaurant ».</t>
+  </si>
+  <si>
+    <t>Rôle (scénario S0 : équipe complète, criticité C2)</t>
+  </si>
+  <si>
+    <t>Coût de l'équipe S0, pilotes (€ HT)</t>
+  </si>
+  <si>
+    <t>Source S0 : 6 OPERATIONS/PRODUCTION/2026 1028 Calculateur de staffing par événement.xlsx (Opérations, 28/10/2026). Source S3 : 6 OPERATIONS/PRODUCTION/2026 1028 Scénarios de staffing - leviers de coût.md (§ 4 et 5).</t>
+  </si>
+  <si>
+    <t>Rôle (scénario S3 : soirées récurrentes optimisées)</t>
+  </si>
+  <si>
+    <t>P (Opérations) : inchangé</t>
+  </si>
+  <si>
+    <t>P (Opérations), levier L2 : 1 serveur pour 9 couverts (24 couverts : 3 au lieu de 4 ; 20 couverts : 3, inchangé)</t>
+  </si>
+  <si>
+    <t>P (Opérations), levier L1 : soirée récurrente classée C1, pas de serveur de réserve. Privatisation : I (Finance), maintenue en C2, contrat client</t>
+  </si>
+  <si>
+    <t>P (Opérations) : aide sommelier maintenu (levier L4 écarté, § 6.3)</t>
+  </si>
+  <si>
+    <t>P (Opérations), levier L3 : vaisselle sale reprise par le loueur, −1 plongeur (réponse d'Options attendue). Privatisation : I (Finance), 1 plongeur maintenu</t>
+  </si>
+  <si>
+    <t>P (Opérations) : fondateur, non rémunéré la première année</t>
+  </si>
+  <si>
+    <t>P (Opérations) : pas nécessaire en C1. Privatisation maintenue (contrat client). Coût nul</t>
+  </si>
+  <si>
+    <t>Personnes mobilisées S3, hors chef</t>
+  </si>
+  <si>
+    <t>Coût de l'équipe S3, soirées récurrentes (€ HT)</t>
+  </si>
+  <si>
+    <t>Surcoût d'une soirée pilote (S0 − S3)</t>
+  </si>
+  <si>
+    <t>Le coût de référence d'une soirée (Prix et marges, ligne 26) est celui de S3. Les deux pilotes (Premier soir et La Grande Nuit) gardent l'équipe complète S0 : leur surcoût (ligne 40) est ajouté au budget comme un coût de test (Budget mensuel, lignes 37 à 40).</t>
+  </si>
+  <si>
+    <t>Non chiffré : le levier L3 rend la location de vaisselle un peu plus chère (montant attendu du loueur Options).</t>
+  </si>
+  <si>
+    <t>Onglet Staffing, scénario S3 des Opérations (soirées récurrentes : leviers L1, L2 et L3 ; 6 OPERATIONS/PRODUCTION/2026 1028 Scénarios de staffing - leviers de coût.md) : effectifs P × heures et coûts horaires H. Les pilotes (S0) sont comptés à part dans le budget</t>
+  </si>
+  <si>
+    <t>Soirées pilotes (équipe complète S0, coût de test)</t>
+  </si>
+  <si>
+    <t>Pilote Premier soir (nombre)</t>
+  </si>
+  <si>
+    <t>Pilote La Grande Nuit (nombre)</t>
+  </si>
+  <si>
+    <t>Surcoût d'équipe des pilotes (inclus dans les coûts directs)</t>
+  </si>
+  <si>
+    <t>Plan des pilotes du Produit (5 PRODUIT/Fou d'un soir plan des deux soirées pilotes.md : Pilote 1 Premier soir, Pilote 2 La Grande Nuit), placés sur la première soirée de chaque offre du budget</t>
+  </si>
+  <si>
+    <t>Idem</t>
+  </si>
+  <si>
+    <t>Équipe complète des pilotes (P, Opérations, 6 OPERATIONS/PRODUCTION/2026 1028 Scénarios de staffing - leviers de coût.md, § 6.1) ; montant : Staffing, ligne 40</t>
+  </si>
+  <si>
+    <t>Scénario S3</t>
+  </si>
+  <si>
+    <t>Mis à jour le 28/10/2026 : le coût de l'équipe d'une soirée (Prix et marges, ligne 26) suit le scénario S3 des Opérations pour les soirées récurrentes (6 OPERATIONS/PRODUCTION/2026 1028 Scénarios de staffing - leviers de coût.md). Les deux pilotes gardent l'équipe complète (S0) : leur surcoût est ajouté aux coûts directs du budget (Budget mensuel, lignes 37 à 40). Le personnel est toujours fourni par Fou d'un soir.</t>
   </si>
 </sst>
 </file>
@@ -1027,7 +1090,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1137,6 +1200,19 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="167" fontId="10" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="169" fontId="7" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
   </cellXfs>
@@ -1473,7 +1549,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FBA644DB-8C71-4A8A-A457-0A27A3813ADD}">
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.6328125" style="1" customWidth="1"/>
@@ -1605,10 +1681,18 @@
     </row>
     <row r="18" spans="1:2" ht="50" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
-        <v>264</v>
+        <v>255</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>265</v>
+        <v>256</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="50" x14ac:dyDescent="0.25">
+      <c r="A19" s="8" t="s">
+        <v>285</v>
+      </c>
+      <c r="B19" s="9" t="s">
+        <v>286</v>
       </c>
     </row>
   </sheetData>
@@ -2211,34 +2295,34 @@
       <c r="H25" s="22"/>
       <c r="I25" s="21"/>
     </row>
-    <row r="26" spans="1:9" ht="62.5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" ht="50" x14ac:dyDescent="0.25">
       <c r="A26" s="19" t="s">
-        <v>263</v>
+        <v>254</v>
       </c>
       <c r="B26" s="19" t="s">
         <v>56</v>
       </c>
       <c r="C26" s="54">
-        <f>Staffing!D21</f>
-        <v>3636</v>
+        <f>Staffing!D39</f>
+        <v>2936</v>
       </c>
       <c r="D26" s="54">
-        <f>Staffing!E21</f>
-        <v>3636</v>
+        <f>Staffing!E39</f>
+        <v>2936</v>
       </c>
       <c r="E26" s="54">
-        <f>Staffing!F21</f>
-        <v>3076</v>
+        <f>Staffing!F39</f>
+        <v>2621</v>
       </c>
       <c r="F26" s="54">
-        <f>Staffing!G21</f>
+        <f>Staffing!G39</f>
         <v>2040</v>
       </c>
       <c r="G26" s="21" t="s">
-        <v>261</v>
+        <v>253</v>
       </c>
       <c r="H26" s="22" t="s">
-        <v>262</v>
+        <v>277</v>
       </c>
       <c r="I26" s="21" t="s">
         <v>102</v>
@@ -2454,15 +2538,15 @@
       </c>
       <c r="C34" s="28">
         <f t="shared" ref="C34:F34" si="7">C19+C22+C25+C26+C27+C28+C29+C32+C33</f>
-        <v>8539.7142857142862</v>
+        <v>7839.7142857142853</v>
       </c>
       <c r="D34" s="28">
         <f t="shared" si="7"/>
-        <v>10544.25</v>
+        <v>9844.25</v>
       </c>
       <c r="E34" s="28">
         <f t="shared" si="7"/>
-        <v>13935.428571428572</v>
+        <v>13480.428571428572</v>
       </c>
       <c r="F34" s="28">
         <f t="shared" si="7"/>
@@ -2494,15 +2578,15 @@
       </c>
       <c r="C36" s="28">
         <f t="shared" ref="C36:F36" si="8">C17-C34</f>
-        <v>-3620.0714285714303</v>
+        <v>-2920.0714285714294</v>
       </c>
       <c r="D36" s="28">
         <f t="shared" si="8"/>
-        <v>-3419.2500000000009</v>
+        <v>-2719.2500000000009</v>
       </c>
       <c r="E36" s="28">
         <f t="shared" si="8"/>
-        <v>-4078.2857142857156</v>
+        <v>-3623.2857142857156</v>
       </c>
       <c r="F36" s="28">
         <f t="shared" si="8"/>
@@ -2521,15 +2605,15 @@
       </c>
       <c r="C37" s="31">
         <f t="shared" ref="C37:F37" si="9">IF(C17&gt;0,C36/C17,0)</f>
-        <v>-0.73584029038112575</v>
+        <v>-0.59355353901996399</v>
       </c>
       <c r="D37" s="31">
         <f t="shared" si="9"/>
-        <v>-0.47989473684210543</v>
+        <v>-0.38164912280701774</v>
       </c>
       <c r="E37" s="31">
         <f t="shared" si="9"/>
-        <v>-0.41373913043478278</v>
+        <v>-0.36757971014492768</v>
       </c>
       <c r="F37" s="31">
         <f t="shared" si="9"/>
@@ -2548,15 +2632,15 @@
       </c>
       <c r="C38" s="27">
         <f t="shared" ref="C38:F38" si="10">IF(C9&gt;0,C36/C9,0)</f>
-        <v>-190.53007518797003</v>
+        <v>-153.68796992481208</v>
       </c>
       <c r="D38" s="27">
         <f t="shared" si="10"/>
-        <v>-179.96052631578951</v>
+        <v>-143.11842105263162</v>
       </c>
       <c r="E38" s="27">
         <f t="shared" si="10"/>
-        <v>-254.89285714285722</v>
+        <v>-226.45535714285722</v>
       </c>
       <c r="F38" s="27">
         <f t="shared" si="10"/>
@@ -2629,15 +2713,15 @@
       </c>
       <c r="C41" s="31">
         <f t="shared" ref="C41:F41" si="13">C37</f>
-        <v>-0.73584029038112575</v>
+        <v>-0.59355353901996399</v>
       </c>
       <c r="D41" s="31">
         <f t="shared" si="13"/>
-        <v>-0.47989473684210543</v>
+        <v>-0.38164912280701774</v>
       </c>
       <c r="E41" s="31">
         <f t="shared" si="13"/>
-        <v>-0.41373913043478278</v>
+        <v>-0.36757971014492768</v>
       </c>
       <c r="F41" s="31">
         <f t="shared" si="13"/>
@@ -2656,15 +2740,15 @@
       </c>
       <c r="C42" s="27">
         <f t="shared" ref="C42:F42" si="14">IF(AND(C9&gt;0,1-C21-C30-C31&gt;0),((C19+C20+C26+C27+C28+C29+C33+C9*(C23+C24))/(1-C21-C30-C31)-C14-C16)/C9*(1+C12),0)</f>
-        <v>506.86350021394958</v>
+        <v>464.92939666238772</v>
       </c>
       <c r="D42" s="27">
         <f t="shared" si="14"/>
-        <v>635.7984898005185</v>
+        <v>591.6195198918067</v>
       </c>
       <c r="E42" s="27">
         <f t="shared" si="14"/>
-        <v>1012.9411764705883</v>
+        <v>976.91176470588243</v>
       </c>
       <c r="F42" s="27">
         <f t="shared" si="14"/>
@@ -2683,15 +2767,15 @@
       </c>
       <c r="C43" s="31">
         <f t="shared" ref="C43:F43" si="15">IF(AND(C7&gt;0,C13*(1-C21-C30-C31)-(C23+C24)&gt;0),MAX(0,(C19+C20+C26+C27+C28+C29+C33-(C14+C16)*(1-C21-C30-C31))/(C13*(1-C21-C30-C31)-(C23+C24)))/C7,0)</f>
-        <v>1.680058897770299</v>
+        <v>1.5082737343991026</v>
       </c>
       <c r="D43" s="31">
         <f t="shared" si="15"/>
-        <v>1.3896467296257435</v>
+        <v>1.2672263029031132</v>
       </c>
       <c r="E43" s="31">
         <f t="shared" si="15"/>
-        <v>1.3385906989906613</v>
+        <v>1.2785020281105555</v>
       </c>
       <c r="F43" s="31">
         <f t="shared" si="15"/>
@@ -2716,7 +2800,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{838C2CEE-3AA8-4CB7-9962-F225A7B6E75A}">
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I43"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="36.6328125" style="1" customWidth="1"/>
@@ -2731,46 +2815,38 @@
   <sheetData>
     <row r="1" spans="1:9" ht="18" x14ac:dyDescent="0.4">
       <c r="A1" s="3" t="s">
-        <v>226</v>
+        <v>257</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="13" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" ht="250.5" x14ac:dyDescent="0.3">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="38" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>228</v>
-      </c>
-      <c r="D4" s="11" t="s">
-        <v>229</v>
-      </c>
-      <c r="E4" s="11" t="s">
-        <v>229</v>
-      </c>
-      <c r="F4" s="11" t="s">
-        <v>229</v>
-      </c>
-      <c r="G4" s="11" t="s">
-        <v>229</v>
-      </c>
+        <v>259</v>
+      </c>
+      <c r="D4" s="55"/>
+      <c r="E4" s="55"/>
+      <c r="F4" s="55"/>
+      <c r="G4" s="55"/>
       <c r="H4" s="1" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="I4" s="7" t="s">
-        <v>230</v>
+        <v>260</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>231</v>
+        <v>261</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>233</v>
+        <v>227</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>118</v>
@@ -2782,18 +2858,18 @@
         <v>120</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>234</v>
+        <v>228</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="I6" s="6" t="s">
-        <v>236</v>
+        <v>230</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="25" x14ac:dyDescent="0.25">
       <c r="A7" s="19" t="s">
-        <v>237</v>
+        <v>231</v>
       </c>
       <c r="B7" s="52">
         <v>9</v>
@@ -2817,12 +2893,12 @@
         <v>0</v>
       </c>
       <c r="I7" s="22" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="19" t="s">
-        <v>239</v>
+        <v>233</v>
       </c>
       <c r="B8" s="52">
         <v>8</v>
@@ -2846,12 +2922,12 @@
         <v>1</v>
       </c>
       <c r="I8" s="22" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="19" t="s">
-        <v>241</v>
+        <v>235</v>
       </c>
       <c r="B9" s="52">
         <v>7</v>
@@ -2875,12 +2951,12 @@
         <v>1</v>
       </c>
       <c r="I9" s="22" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="19" t="s">
-        <v>243</v>
+        <v>237</v>
       </c>
       <c r="B10" s="52">
         <v>7</v>
@@ -2904,12 +2980,12 @@
         <v>1</v>
       </c>
       <c r="I10" s="22" t="s">
-        <v>244</v>
+        <v>238</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="19" t="s">
-        <v>245</v>
+        <v>239</v>
       </c>
       <c r="B11" s="52">
         <v>7</v>
@@ -2933,12 +3009,12 @@
         <v>0</v>
       </c>
       <c r="I11" s="22" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="19" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="B12" s="52">
         <v>7</v>
@@ -2962,12 +3038,12 @@
         <v>0</v>
       </c>
       <c r="I12" s="22" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="19" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
       <c r="B13" s="52">
         <v>7</v>
@@ -2991,12 +3067,12 @@
         <v>0</v>
       </c>
       <c r="I13" s="22" t="s">
-        <v>250</v>
+        <v>244</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="25" x14ac:dyDescent="0.25">
       <c r="A14" s="19" t="s">
-        <v>251</v>
+        <v>245</v>
       </c>
       <c r="B14" s="52">
         <v>10</v>
@@ -3020,12 +3096,12 @@
         <v>0</v>
       </c>
       <c r="I14" s="22" t="s">
-        <v>252</v>
+        <v>246</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="25" x14ac:dyDescent="0.25">
       <c r="A15" s="19" t="s">
-        <v>253</v>
+        <v>247</v>
       </c>
       <c r="B15" s="52">
         <v>5</v>
@@ -3049,17 +3125,17 @@
         <v>0</v>
       </c>
       <c r="I15" s="22" t="s">
-        <v>254</v>
+        <v>248</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="13" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" ht="13" x14ac:dyDescent="0.3">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="13" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
@@ -3080,9 +3156,9 @@
         <v>9</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="13" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:9" ht="13" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
-        <v>257</v>
+        <v>251</v>
       </c>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
@@ -3103,70 +3179,516 @@
         <v>4</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="13" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:9" ht="13" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
       <c r="D20" s="14">
-        <f>SUMPRODUCT(D7:D15,$B$7:$B$15,--($C$7:$C$15&gt;0))-IF(D$4="Restaurant",SUMPRODUCT(D7:D15,$B$7:$B$15,$H$7:$H$15,--($C$7:$C$15&gt;0)),0)</f>
+        <f>SUMPRODUCT(D7:D15,$B$7:$B$15,--($C$7:$C$15&gt;0))</f>
         <v>98</v>
       </c>
       <c r="E20" s="14">
-        <f>SUMPRODUCT(E7:E15,$B$7:$B$15,--($C$7:$C$15&gt;0))-IF(E$4="Restaurant",SUMPRODUCT(E7:E15,$B$7:$B$15,$H$7:$H$15,--($C$7:$C$15&gt;0)),0)</f>
+        <f>SUMPRODUCT(E7:E15,$B$7:$B$15,--($C$7:$C$15&gt;0))</f>
         <v>98</v>
       </c>
       <c r="F20" s="14">
-        <f>SUMPRODUCT(F7:F15,$B$7:$B$15,--($C$7:$C$15&gt;0))-IF(F$4="Restaurant",SUMPRODUCT(F7:F15,$B$7:$B$15,$H$7:$H$15,--($C$7:$C$15&gt;0)),0)</f>
+        <f>SUMPRODUCT(F7:F15,$B$7:$B$15,--($C$7:$C$15&gt;0))</f>
         <v>82</v>
       </c>
       <c r="G20" s="14">
-        <f>SUMPRODUCT(G7:G15,$B$7:$B$15,--($C$7:$C$15&gt;0))-IF(G$4="Restaurant",SUMPRODUCT(G7:G15,$B$7:$B$15,$H$7:$H$15,--($C$7:$C$15&gt;0)),0)</f>
+        <f>SUMPRODUCT(G7:G15,$B$7:$B$15,--($C$7:$C$15&gt;0))</f>
         <v>52</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="13" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:9" ht="13" x14ac:dyDescent="0.3">
       <c r="A21" s="45" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="B21" s="45"/>
       <c r="C21" s="45"/>
       <c r="D21" s="46">
-        <f>SUMPRODUCT(D7:D15,$B$7:$B$15,$C$7:$C$15)-IF(D$4="Restaurant",SUMPRODUCT(D7:D15,$B$7:$B$15,$C$7:$C$15,$H$7:$H$15),0)</f>
+        <f>SUMPRODUCT(D7:D15,$B$7:$B$15,$C$7:$C$15)</f>
         <v>3636</v>
       </c>
       <c r="E21" s="46">
-        <f>SUMPRODUCT(E7:E15,$B$7:$B$15,$C$7:$C$15)-IF(E$4="Restaurant",SUMPRODUCT(E7:E15,$B$7:$B$15,$C$7:$C$15,$H$7:$H$15),0)</f>
+        <f>SUMPRODUCT(E7:E15,$B$7:$B$15,$C$7:$C$15)</f>
         <v>3636</v>
       </c>
       <c r="F21" s="46">
-        <f>SUMPRODUCT(F7:F15,$B$7:$B$15,$C$7:$C$15)-IF(F$4="Restaurant",SUMPRODUCT(F7:F15,$B$7:$B$15,$C$7:$C$15,$H$7:$H$15),0)</f>
+        <f>SUMPRODUCT(F7:F15,$B$7:$B$15,$C$7:$C$15)</f>
         <v>3076</v>
       </c>
       <c r="G21" s="46">
-        <f>SUMPRODUCT(G7:G15,$B$7:$B$15,$C$7:$C$15)-IF(G$4="Restaurant",SUMPRODUCT(G7:G15,$B$7:$B$15,$C$7:$C$15,$H$7:$H$15),0)</f>
+        <f>SUMPRODUCT(G7:G15,$B$7:$B$15,$C$7:$C$15)</f>
         <v>2040</v>
       </c>
     </row>
-    <row r="23" spans="1:7" ht="13" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:9" ht="13" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
-        <v>260</v>
+        <v>263</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" ht="42" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="6" t="s">
+        <v>264</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>226</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>227</v>
+      </c>
+      <c r="D25" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E25" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="F25" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="G25" s="6" t="s">
+        <v>228</v>
+      </c>
+      <c r="H25" s="6" t="s">
+        <v>229</v>
+      </c>
+      <c r="I25" s="6" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A26" s="56" t="str">
+        <f>A7</f>
+        <v>Brigade (second, commis)</v>
+      </c>
+      <c r="B26" s="57">
+        <f>B7</f>
+        <v>9</v>
+      </c>
+      <c r="C26" s="58">
+        <f>C7</f>
+        <v>35</v>
+      </c>
+      <c r="D26" s="20">
+        <v>3</v>
+      </c>
+      <c r="E26" s="20">
+        <v>3</v>
+      </c>
+      <c r="F26" s="20">
+        <v>2</v>
+      </c>
+      <c r="G26" s="20">
+        <v>1</v>
+      </c>
+      <c r="H26" s="59">
+        <f>H7</f>
+        <v>0</v>
+      </c>
+      <c r="I26" s="22" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A27" s="56" t="str">
+        <f>A8</f>
+        <v>Maître d'hôtel</v>
+      </c>
+      <c r="B27" s="57">
+        <f>B8</f>
+        <v>8</v>
+      </c>
+      <c r="C27" s="58">
+        <f>C8</f>
+        <v>45</v>
+      </c>
+      <c r="D27" s="20">
+        <v>1</v>
+      </c>
+      <c r="E27" s="20">
+        <v>1</v>
+      </c>
+      <c r="F27" s="20">
+        <v>1</v>
+      </c>
+      <c r="G27" s="20">
+        <v>1</v>
+      </c>
+      <c r="H27" s="59">
+        <f>H8</f>
+        <v>1</v>
+      </c>
+      <c r="I27" s="22" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" ht="25" x14ac:dyDescent="0.25">
+      <c r="A28" s="56" t="str">
+        <f>A9</f>
+        <v>Serveurs (base)</v>
+      </c>
+      <c r="B28" s="57">
+        <f>B9</f>
+        <v>7</v>
+      </c>
+      <c r="C28" s="58">
+        <f>C9</f>
+        <v>35</v>
+      </c>
+      <c r="D28" s="20">
+        <v>3</v>
+      </c>
+      <c r="E28" s="20">
+        <v>3</v>
+      </c>
+      <c r="F28" s="20">
+        <v>3</v>
+      </c>
+      <c r="G28" s="20">
+        <v>2</v>
+      </c>
+      <c r="H28" s="59">
+        <f>H9</f>
+        <v>1</v>
+      </c>
+      <c r="I28" s="22" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" ht="25" x14ac:dyDescent="0.25">
+      <c r="A29" s="56" t="str">
+        <f>A10</f>
+        <v>Serveur de réserve</v>
+      </c>
+      <c r="B29" s="57">
+        <f>B10</f>
+        <v>7</v>
+      </c>
+      <c r="C29" s="58">
+        <f>C10</f>
+        <v>35</v>
+      </c>
+      <c r="D29" s="20">
+        <v>0</v>
+      </c>
+      <c r="E29" s="20">
+        <v>0</v>
+      </c>
+      <c r="F29" s="20">
+        <v>0</v>
+      </c>
+      <c r="G29" s="20">
+        <v>1</v>
+      </c>
+      <c r="H29" s="59">
+        <f>H10</f>
+        <v>1</v>
+      </c>
+      <c r="I29" s="22" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A30" s="56" t="str">
+        <f>A11</f>
+        <v>Sommelier invité</v>
+      </c>
+      <c r="B30" s="57">
+        <f>B11</f>
+        <v>7</v>
+      </c>
+      <c r="C30" s="58">
+        <f>C11</f>
+        <v>60</v>
+      </c>
+      <c r="D30" s="20">
+        <v>1</v>
+      </c>
+      <c r="E30" s="20">
+        <v>1</v>
+      </c>
+      <c r="F30" s="20">
+        <v>1</v>
+      </c>
+      <c r="G30" s="20">
+        <v>1</v>
+      </c>
+      <c r="H30" s="59">
+        <f>H11</f>
+        <v>0</v>
+      </c>
+      <c r="I30" s="22" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A31" s="56" t="str">
+        <f>A12</f>
+        <v>Aide sommelier</v>
+      </c>
+      <c r="B31" s="57">
+        <f>B12</f>
+        <v>7</v>
+      </c>
+      <c r="C31" s="58">
+        <f>C12</f>
+        <v>38</v>
+      </c>
+      <c r="D31" s="20">
+        <v>1</v>
+      </c>
+      <c r="E31" s="20">
+        <v>1</v>
+      </c>
+      <c r="F31" s="20">
+        <v>1</v>
+      </c>
+      <c r="G31" s="20">
+        <v>0</v>
+      </c>
+      <c r="H31" s="59">
+        <f>H12</f>
+        <v>0</v>
+      </c>
+      <c r="I31" s="22" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" ht="25" x14ac:dyDescent="0.25">
+      <c r="A32" s="56" t="str">
+        <f>A13</f>
+        <v>Plongeurs</v>
+      </c>
+      <c r="B32" s="57">
+        <f>B13</f>
+        <v>7</v>
+      </c>
+      <c r="C32" s="58">
+        <f>C13</f>
+        <v>30</v>
+      </c>
+      <c r="D32" s="20">
+        <v>1</v>
+      </c>
+      <c r="E32" s="20">
+        <v>1</v>
+      </c>
+      <c r="F32" s="20">
+        <v>1</v>
+      </c>
+      <c r="G32" s="20">
+        <v>1</v>
+      </c>
+      <c r="H32" s="59">
+        <f>H13</f>
+        <v>0</v>
+      </c>
+      <c r="I32" s="22" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A33" s="56" t="str">
+        <f>A14</f>
+        <v>Responsable de production (nous)</v>
+      </c>
+      <c r="B33" s="57">
+        <f>B14</f>
+        <v>10</v>
+      </c>
+      <c r="C33" s="58">
+        <f>C14</f>
+        <v>0</v>
+      </c>
+      <c r="D33" s="20">
+        <v>1</v>
+      </c>
+      <c r="E33" s="20">
+        <v>1</v>
+      </c>
+      <c r="F33" s="20">
+        <v>1</v>
+      </c>
+      <c r="G33" s="20">
+        <v>1</v>
+      </c>
+      <c r="H33" s="59">
+        <f>H14</f>
+        <v>0</v>
+      </c>
+      <c r="I33" s="22" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A34" s="56" t="str">
+        <f>A15</f>
+        <v>Interlocuteur client (Ventes)</v>
+      </c>
+      <c r="B34" s="57">
+        <f>B15</f>
+        <v>5</v>
+      </c>
+      <c r="C34" s="58">
+        <f>C15</f>
+        <v>0</v>
+      </c>
+      <c r="D34" s="20">
+        <v>0</v>
+      </c>
+      <c r="E34" s="20">
+        <v>0</v>
+      </c>
+      <c r="F34" s="20">
+        <v>0</v>
+      </c>
+      <c r="G34" s="20">
+        <v>1</v>
+      </c>
+      <c r="H34" s="59">
+        <f>H15</f>
+        <v>0</v>
+      </c>
+      <c r="I34" s="22" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" ht="13" x14ac:dyDescent="0.3">
+      <c r="A36" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="B36" s="2"/>
+      <c r="C36" s="2"/>
+      <c r="D36" s="14">
+        <f>SUM(D26:D34)</f>
+        <v>11</v>
+      </c>
+      <c r="E36" s="14">
+        <f>SUM(E26:E34)</f>
+        <v>11</v>
+      </c>
+      <c r="F36" s="14">
+        <f>SUM(F26:F34)</f>
+        <v>10</v>
+      </c>
+      <c r="G36" s="14">
+        <f>SUM(G26:G34)</f>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" ht="13" x14ac:dyDescent="0.3">
+      <c r="A37" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="B37" s="2"/>
+      <c r="C37" s="2"/>
+      <c r="D37" s="14">
+        <f>SUMPRODUCT(D26:D34,$H$26:$H$34)</f>
+        <v>4</v>
+      </c>
+      <c r="E37" s="14">
+        <f>SUMPRODUCT(E26:E34,$H$26:$H$34)</f>
+        <v>4</v>
+      </c>
+      <c r="F37" s="14">
+        <f>SUMPRODUCT(F26:F34,$H$26:$H$34)</f>
+        <v>4</v>
+      </c>
+      <c r="G37" s="14">
+        <f>SUMPRODUCT(G26:G34,$H$26:$H$34)</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" ht="13" x14ac:dyDescent="0.3">
+      <c r="A38" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="B38" s="2"/>
+      <c r="C38" s="2"/>
+      <c r="D38" s="14">
+        <f>SUMPRODUCT(D26:D34,$B$26:$B$34,--($C$26:$C$34&gt;0))</f>
+        <v>77</v>
+      </c>
+      <c r="E38" s="14">
+        <f>SUMPRODUCT(E26:E34,$B$26:$B$34,--($C$26:$C$34&gt;0))</f>
+        <v>77</v>
+      </c>
+      <c r="F38" s="14">
+        <f>SUMPRODUCT(F26:F34,$B$26:$B$34,--($C$26:$C$34&gt;0))</f>
+        <v>68</v>
+      </c>
+      <c r="G38" s="14">
+        <f>SUMPRODUCT(G26:G34,$B$26:$B$34,--($C$26:$C$34&gt;0))</f>
+        <v>52</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" ht="13" x14ac:dyDescent="0.3">
+      <c r="A39" s="45" t="s">
+        <v>273</v>
+      </c>
+      <c r="B39" s="45"/>
+      <c r="C39" s="45"/>
+      <c r="D39" s="46">
+        <f>SUMPRODUCT(D26:D34,$B$26:$B$34,$C$26:$C$34)</f>
+        <v>2936</v>
+      </c>
+      <c r="E39" s="46">
+        <f>SUMPRODUCT(E26:E34,$B$26:$B$34,$C$26:$C$34)</f>
+        <v>2936</v>
+      </c>
+      <c r="F39" s="46">
+        <f>SUMPRODUCT(F26:F34,$B$26:$B$34,$C$26:$C$34)</f>
+        <v>2621</v>
+      </c>
+      <c r="G39" s="46">
+        <f>SUMPRODUCT(G26:G34,$B$26:$B$34,$C$26:$C$34)</f>
+        <v>2040</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" ht="13" x14ac:dyDescent="0.3">
+      <c r="A40" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="B40" s="2"/>
+      <c r="C40" s="2"/>
+      <c r="D40" s="17">
+        <f>D21-D39</f>
+        <v>700</v>
+      </c>
+      <c r="E40" s="17">
+        <f>E21-E39</f>
+        <v>700</v>
+      </c>
+      <c r="F40" s="17">
+        <f>F21-F39</f>
+        <v>455</v>
+      </c>
+      <c r="G40" s="17">
+        <f>G21-G39</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" ht="13" x14ac:dyDescent="0.3">
+      <c r="A42" s="4" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" ht="13" x14ac:dyDescent="0.3">
+      <c r="A43" s="4" t="s">
+        <v>276</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4:G4" xr:uid="{9B663A6E-5B92-4772-A1ED-AA5999827DF6}">
-      <formula1>"Nous,Restaurant"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62A8117B-BF63-41C1-92C8-4FEDF95C8C14}">
-  <dimension ref="A1:P35"/>
+  <dimension ref="A1:P40"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="44.6328125" style="1" customWidth="1"/>
@@ -3624,55 +4146,55 @@
       </c>
       <c r="B14" s="17">
         <f>SUM(C14:N14)</f>
-        <v>154313.17857142858</v>
+        <v>149903.17857142858</v>
       </c>
       <c r="C14" s="34">
-        <f>C7*'Prix et marges'!$C$34+C8*'Prix et marges'!$D$34+C9*'Prix et marges'!$E$34+C10*'Prix et marges'!$F$34</f>
+        <f>C7*'Prix et marges'!$C$34+C8*'Prix et marges'!$D$34+C9*'Prix et marges'!$E$34+C10*'Prix et marges'!$F$34+C40</f>
         <v>0</v>
       </c>
       <c r="D14" s="34">
-        <f>D7*'Prix et marges'!$C$34+D8*'Prix et marges'!$D$34+D9*'Prix et marges'!$E$34+D10*'Prix et marges'!$F$34</f>
+        <f>D7*'Prix et marges'!$C$34+D8*'Prix et marges'!$D$34+D9*'Prix et marges'!$E$34+D10*'Prix et marges'!$F$34+D40</f>
         <v>0</v>
       </c>
       <c r="E14" s="34">
-        <f>E7*'Prix et marges'!$C$34+E8*'Prix et marges'!$D$34+E9*'Prix et marges'!$E$34+E10*'Prix et marges'!$F$34</f>
+        <f>E7*'Prix et marges'!$C$34+E8*'Prix et marges'!$D$34+E9*'Prix et marges'!$E$34+E10*'Prix et marges'!$F$34+E40</f>
         <v>8539.7142857142862</v>
       </c>
       <c r="F14" s="34">
-        <f>F7*'Prix et marges'!$C$34+F8*'Prix et marges'!$D$34+F9*'Prix et marges'!$E$34+F10*'Prix et marges'!$F$34</f>
+        <f>F7*'Prix et marges'!$C$34+F8*'Prix et marges'!$D$34+F9*'Prix et marges'!$E$34+F10*'Prix et marges'!$F$34+F40</f>
         <v>13935.428571428572</v>
       </c>
       <c r="G14" s="34">
-        <f>G7*'Prix et marges'!$C$34+G8*'Prix et marges'!$D$34+G9*'Prix et marges'!$E$34+G10*'Prix et marges'!$F$34</f>
-        <v>10544.25</v>
+        <f>G7*'Prix et marges'!$C$34+G8*'Prix et marges'!$D$34+G9*'Prix et marges'!$E$34+G10*'Prix et marges'!$F$34+G40</f>
+        <v>9844.25</v>
       </c>
       <c r="H14" s="34">
-        <f>H7*'Prix et marges'!$C$34+H8*'Prix et marges'!$D$34+H9*'Prix et marges'!$E$34+H10*'Prix et marges'!$F$34</f>
-        <v>16433.285714285714</v>
+        <f>H7*'Prix et marges'!$C$34+H8*'Prix et marges'!$D$34+H9*'Prix et marges'!$E$34+H10*'Prix et marges'!$F$34+H40</f>
+        <v>15733.285714285714</v>
       </c>
       <c r="I14" s="34">
-        <f>I7*'Prix et marges'!$C$34+I8*'Prix et marges'!$D$34+I9*'Prix et marges'!$E$34+I10*'Prix et marges'!$F$34</f>
-        <v>21829</v>
+        <f>I7*'Prix et marges'!$C$34+I8*'Prix et marges'!$D$34+I9*'Prix et marges'!$E$34+I10*'Prix et marges'!$F$34+I40</f>
+        <v>21374</v>
       </c>
       <c r="J14" s="34">
-        <f>J7*'Prix et marges'!$C$34+J8*'Prix et marges'!$D$34+J9*'Prix et marges'!$E$34+J10*'Prix et marges'!$F$34</f>
-        <v>18437.821428571428</v>
+        <f>J7*'Prix et marges'!$C$34+J8*'Prix et marges'!$D$34+J9*'Prix et marges'!$E$34+J10*'Prix et marges'!$F$34+J40</f>
+        <v>17737.821428571428</v>
       </c>
       <c r="K14" s="34">
-        <f>K7*'Prix et marges'!$C$34+K8*'Prix et marges'!$D$34+K9*'Prix et marges'!$E$34+K10*'Prix et marges'!$F$34</f>
-        <v>8539.7142857142862</v>
+        <f>K7*'Prix et marges'!$C$34+K8*'Prix et marges'!$D$34+K9*'Prix et marges'!$E$34+K10*'Prix et marges'!$F$34+K40</f>
+        <v>7839.7142857142853</v>
       </c>
       <c r="L14" s="34">
-        <f>L7*'Prix et marges'!$C$34+L8*'Prix et marges'!$D$34+L9*'Prix et marges'!$E$34+L10*'Prix et marges'!$F$34</f>
+        <f>L7*'Prix et marges'!$C$34+L8*'Prix et marges'!$D$34+L9*'Prix et marges'!$E$34+L10*'Prix et marges'!$F$34+L40</f>
         <v>0</v>
       </c>
       <c r="M14" s="34">
-        <f>M7*'Prix et marges'!$C$34+M8*'Prix et marges'!$D$34+M9*'Prix et marges'!$E$34+M10*'Prix et marges'!$F$34</f>
-        <v>29722.571428571428</v>
+        <f>M7*'Prix et marges'!$C$34+M8*'Prix et marges'!$D$34+M9*'Prix et marges'!$E$34+M10*'Prix et marges'!$F$34+M40</f>
+        <v>29267.571428571428</v>
       </c>
       <c r="N14" s="34">
-        <f>N7*'Prix et marges'!$C$34+N8*'Prix et marges'!$D$34+N9*'Prix et marges'!$E$34+N10*'Prix et marges'!$F$34</f>
-        <v>26331.392857142855</v>
+        <f>N7*'Prix et marges'!$C$34+N8*'Prix et marges'!$D$34+N9*'Prix et marges'!$E$34+N10*'Prix et marges'!$F$34+N40</f>
+        <v>25631.392857142855</v>
       </c>
     </row>
     <row r="15" spans="1:16" ht="13" x14ac:dyDescent="0.3">
@@ -3681,7 +4203,7 @@
       </c>
       <c r="B15" s="17">
         <f>SUM(C15:N15)</f>
-        <v>-32357.821428571442</v>
+        <v>-27947.821428571438</v>
       </c>
       <c r="C15" s="17">
         <f t="shared" ref="C15:N15" si="2">C13-C14</f>
@@ -3701,23 +4223,23 @@
       </c>
       <c r="G15" s="17">
         <f t="shared" si="2"/>
-        <v>-3419.2500000000009</v>
+        <v>-2719.2500000000009</v>
       </c>
       <c r="H15" s="17">
         <f t="shared" si="2"/>
-        <v>-3477.9285714285725</v>
+        <v>-2777.9285714285725</v>
       </c>
       <c r="I15" s="17">
         <f t="shared" si="2"/>
-        <v>-3936.1428571428587</v>
+        <v>-3481.1428571428587</v>
       </c>
       <c r="J15" s="17">
         <f t="shared" si="2"/>
-        <v>-3277.1071428571431</v>
+        <v>-2577.1071428571431</v>
       </c>
       <c r="K15" s="17">
         <f t="shared" si="2"/>
-        <v>-3620.0714285714303</v>
+        <v>-2920.0714285714294</v>
       </c>
       <c r="L15" s="17">
         <f t="shared" si="2"/>
@@ -3725,11 +4247,11 @@
       </c>
       <c r="M15" s="17">
         <f t="shared" si="2"/>
-        <v>-3794</v>
+        <v>-3339</v>
       </c>
       <c r="N15" s="17">
         <f t="shared" si="2"/>
-        <v>-3134.9642857142862</v>
+        <v>-2434.9642857142862</v>
       </c>
     </row>
     <row r="16" spans="1:16" ht="13" x14ac:dyDescent="0.3">
@@ -4581,7 +5103,7 @@
       </c>
       <c r="B34" s="17">
         <f>SUM(C34:N34)</f>
-        <v>-45029.821428571435</v>
+        <v>-40619.821428571435</v>
       </c>
       <c r="C34" s="17">
         <f t="shared" ref="C34:N34" si="7">C15-C32</f>
@@ -4601,23 +5123,23 @@
       </c>
       <c r="G34" s="17">
         <f t="shared" si="7"/>
-        <v>-4029.2500000000009</v>
+        <v>-3329.2500000000009</v>
       </c>
       <c r="H34" s="17">
         <f t="shared" si="7"/>
-        <v>-4087.9285714285725</v>
+        <v>-3387.9285714285725</v>
       </c>
       <c r="I34" s="17">
         <f t="shared" si="7"/>
-        <v>-4546.1428571428587</v>
+        <v>-4091.1428571428587</v>
       </c>
       <c r="J34" s="17">
         <f t="shared" si="7"/>
-        <v>-3887.1071428571431</v>
+        <v>-3187.1071428571431</v>
       </c>
       <c r="K34" s="17">
         <f t="shared" si="7"/>
-        <v>-4230.0714285714303</v>
+        <v>-3530.0714285714294</v>
       </c>
       <c r="L34" s="17">
         <f t="shared" si="7"/>
@@ -4625,11 +5147,11 @@
       </c>
       <c r="M34" s="17">
         <f t="shared" si="7"/>
-        <v>-4404</v>
+        <v>-3949</v>
       </c>
       <c r="N34" s="17">
         <f t="shared" si="7"/>
-        <v>-3744.9642857142862</v>
+        <v>-3044.9642857142862</v>
       </c>
     </row>
     <row r="35" spans="1:16" ht="13" x14ac:dyDescent="0.3">
@@ -4638,7 +5160,7 @@
       </c>
       <c r="B35" s="17">
         <f>N35</f>
-        <v>-45029.821428571435</v>
+        <v>-40619.821428571435</v>
       </c>
       <c r="C35" s="17">
         <f>C34</f>
@@ -4658,40 +5180,225 @@
       </c>
       <c r="G35" s="17">
         <f t="shared" si="8"/>
-        <v>-19519.607142857149</v>
+        <v>-18819.607142857149</v>
       </c>
       <c r="H35" s="17">
         <f t="shared" si="8"/>
-        <v>-23607.535714285721</v>
+        <v>-22207.535714285721</v>
       </c>
       <c r="I35" s="17">
         <f t="shared" si="8"/>
-        <v>-28153.67857142858</v>
+        <v>-26298.67857142858</v>
       </c>
       <c r="J35" s="17">
         <f t="shared" si="8"/>
-        <v>-32040.785714285725</v>
+        <v>-29485.785714285725</v>
       </c>
       <c r="K35" s="17">
         <f t="shared" si="8"/>
-        <v>-36270.857142857152</v>
+        <v>-33015.857142857152</v>
       </c>
       <c r="L35" s="17">
         <f t="shared" si="8"/>
-        <v>-36880.857142857152</v>
+        <v>-33625.857142857152</v>
       </c>
       <c r="M35" s="17">
         <f t="shared" si="8"/>
-        <v>-41284.857142857152</v>
+        <v>-37574.857142857152</v>
       </c>
       <c r="N35" s="17">
         <f t="shared" si="8"/>
-        <v>-45029.821428571435</v>
+        <v>-40619.821428571435</v>
+      </c>
+    </row>
+    <row r="37" spans="1:16" ht="13" x14ac:dyDescent="0.3">
+      <c r="A37" s="10" t="s">
+        <v>278</v>
+      </c>
+      <c r="B37" s="10"/>
+      <c r="C37" s="10"/>
+      <c r="D37" s="10"/>
+      <c r="E37" s="10"/>
+      <c r="F37" s="10"/>
+      <c r="G37" s="10"/>
+      <c r="H37" s="10"/>
+      <c r="I37" s="10"/>
+      <c r="J37" s="10"/>
+      <c r="K37" s="10"/>
+      <c r="L37" s="10"/>
+      <c r="M37" s="10"/>
+      <c r="N37" s="10"/>
+      <c r="O37" s="10"/>
+      <c r="P37" s="10"/>
+    </row>
+    <row r="38" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A38" s="1" t="s">
+        <v>279</v>
+      </c>
+      <c r="B38" s="13">
+        <f>SUM(C38:N38)</f>
+        <v>1</v>
+      </c>
+      <c r="C38" s="12">
+        <v>0</v>
+      </c>
+      <c r="D38" s="12">
+        <v>0</v>
+      </c>
+      <c r="E38" s="12">
+        <v>1</v>
+      </c>
+      <c r="F38" s="12">
+        <v>0</v>
+      </c>
+      <c r="G38" s="12">
+        <v>0</v>
+      </c>
+      <c r="H38" s="12">
+        <v>0</v>
+      </c>
+      <c r="I38" s="12">
+        <v>0</v>
+      </c>
+      <c r="J38" s="12">
+        <v>0</v>
+      </c>
+      <c r="K38" s="12">
+        <v>0</v>
+      </c>
+      <c r="L38" s="12">
+        <v>0</v>
+      </c>
+      <c r="M38" s="12">
+        <v>0</v>
+      </c>
+      <c r="N38" s="12">
+        <v>0</v>
+      </c>
+      <c r="O38" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="P38" s="1" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="39" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A39" s="1" t="s">
+        <v>280</v>
+      </c>
+      <c r="B39" s="13">
+        <f>SUM(C39:N39)</f>
+        <v>1</v>
+      </c>
+      <c r="C39" s="12">
+        <v>0</v>
+      </c>
+      <c r="D39" s="12">
+        <v>0</v>
+      </c>
+      <c r="E39" s="12">
+        <v>0</v>
+      </c>
+      <c r="F39" s="12">
+        <v>1</v>
+      </c>
+      <c r="G39" s="12">
+        <v>0</v>
+      </c>
+      <c r="H39" s="12">
+        <v>0</v>
+      </c>
+      <c r="I39" s="12">
+        <v>0</v>
+      </c>
+      <c r="J39" s="12">
+        <v>0</v>
+      </c>
+      <c r="K39" s="12">
+        <v>0</v>
+      </c>
+      <c r="L39" s="12">
+        <v>0</v>
+      </c>
+      <c r="M39" s="12">
+        <v>0</v>
+      </c>
+      <c r="N39" s="12">
+        <v>0</v>
+      </c>
+      <c r="O39" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="P39" s="1" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="40" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A40" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="B40" s="16">
+        <f>SUM(C40:N40)</f>
+        <v>1155</v>
+      </c>
+      <c r="C40" s="16">
+        <f>C38*Staffing!$D$40+C39*Staffing!$F$40</f>
+        <v>0</v>
+      </c>
+      <c r="D40" s="16">
+        <f>D38*Staffing!$D$40+D39*Staffing!$F$40</f>
+        <v>0</v>
+      </c>
+      <c r="E40" s="16">
+        <f>E38*Staffing!$D$40+E39*Staffing!$F$40</f>
+        <v>700</v>
+      </c>
+      <c r="F40" s="16">
+        <f>F38*Staffing!$D$40+F39*Staffing!$F$40</f>
+        <v>455</v>
+      </c>
+      <c r="G40" s="16">
+        <f>G38*Staffing!$D$40+G39*Staffing!$F$40</f>
+        <v>0</v>
+      </c>
+      <c r="H40" s="16">
+        <f>H38*Staffing!$D$40+H39*Staffing!$F$40</f>
+        <v>0</v>
+      </c>
+      <c r="I40" s="16">
+        <f>I38*Staffing!$D$40+I39*Staffing!$F$40</f>
+        <v>0</v>
+      </c>
+      <c r="J40" s="16">
+        <f>J38*Staffing!$D$40+J39*Staffing!$F$40</f>
+        <v>0</v>
+      </c>
+      <c r="K40" s="16">
+        <f>K38*Staffing!$D$40+K39*Staffing!$F$40</f>
+        <v>0</v>
+      </c>
+      <c r="L40" s="16">
+        <f>L38*Staffing!$D$40+L39*Staffing!$F$40</f>
+        <v>0</v>
+      </c>
+      <c r="M40" s="16">
+        <f>M38*Staffing!$D$40+M39*Staffing!$F$40</f>
+        <v>0</v>
+      </c>
+      <c r="N40" s="16">
+        <f>N38*Staffing!$D$40+N39*Staffing!$F$40</f>
+        <v>0</v>
+      </c>
+      <c r="O40" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="P40" s="1" t="s">
+        <v>284</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O7:O16 O31 O17:O30" xr:uid="{31226B02-E24A-4164-8201-A9757FEFEA83}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O7:O31" xr:uid="{31226B02-E24A-4164-8201-A9757FEFEA83}">
       <formula1>"F,I,P,H"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5259,7 +5966,7 @@
       </c>
       <c r="B22" s="16">
         <f>SUM(C22:N22)</f>
-        <v>-45029.821428571435</v>
+        <v>-40619.821428571435</v>
       </c>
       <c r="C22" s="36">
         <f>'Budget mensuel'!C34</f>
@@ -5279,23 +5986,23 @@
       </c>
       <c r="G22" s="36">
         <f>'Budget mensuel'!G34</f>
-        <v>-4029.2500000000009</v>
+        <v>-3329.2500000000009</v>
       </c>
       <c r="H22" s="36">
         <f>'Budget mensuel'!H34</f>
-        <v>-4087.9285714285725</v>
+        <v>-3387.9285714285725</v>
       </c>
       <c r="I22" s="36">
         <f>'Budget mensuel'!I34</f>
-        <v>-4546.1428571428587</v>
+        <v>-4091.1428571428587</v>
       </c>
       <c r="J22" s="36">
         <f>'Budget mensuel'!J34</f>
-        <v>-3887.1071428571431</v>
+        <v>-3187.1071428571431</v>
       </c>
       <c r="K22" s="36">
         <f>'Budget mensuel'!K34</f>
-        <v>-4230.0714285714303</v>
+        <v>-3530.0714285714294</v>
       </c>
       <c r="L22" s="36">
         <f>'Budget mensuel'!L34</f>
@@ -5303,11 +6010,11 @@
       </c>
       <c r="M22" s="36">
         <f>'Budget mensuel'!M34</f>
-        <v>-4404</v>
+        <v>-3949</v>
       </c>
       <c r="N22" s="36">
         <f>'Budget mensuel'!N34</f>
-        <v>-3744.9642857142862</v>
+        <v>-3044.9642857142862</v>
       </c>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.25">
@@ -5644,16 +6351,16 @@
         <v>56</v>
       </c>
       <c r="C14" s="38">
-        <f>C7*'Prix et marges'!$C$34+C8*'Prix et marges'!$D$34+C9*'Prix et marges'!$E$34+C10*'Prix et marges'!$F$34</f>
-        <v>154313.17857142858</v>
+        <f>C7*'Prix et marges'!$C$34+C8*'Prix et marges'!$D$34+C9*'Prix et marges'!$E$34+C10*'Prix et marges'!$F$34+'Budget mensuel'!$B$40</f>
+        <v>149903.17857142858</v>
       </c>
       <c r="D14" s="38">
         <f>D7*'Prix et marges'!$C$34+D8*'Prix et marges'!$D$34+D9*'Prix et marges'!$E$34+D10*'Prix et marges'!$F$34</f>
-        <v>453600.85714285716</v>
+        <v>438760.85714285716</v>
       </c>
       <c r="E14" s="38">
         <f>E7*'Prix et marges'!$C$34+E8*'Prix et marges'!$D$34+E9*'Prix et marges'!$E$34+E10*'Prix et marges'!$F$34</f>
-        <v>775124.14285714296</v>
+        <v>752864.14285714296</v>
       </c>
       <c r="F14" s="21"/>
       <c r="G14" s="22"/>
@@ -5667,15 +6374,15 @@
       </c>
       <c r="C15" s="28">
         <f t="shared" ref="C15:E15" si="1">C13-C14</f>
-        <v>-32357.821428571449</v>
+        <v>-27947.821428571449</v>
       </c>
       <c r="D15" s="28">
         <f t="shared" si="1"/>
-        <v>-85529.428571428638</v>
+        <v>-70689.428571428638</v>
       </c>
       <c r="E15" s="28">
         <f t="shared" si="1"/>
-        <v>-126588.42857142875</v>
+        <v>-104328.42857142875</v>
       </c>
       <c r="F15" s="21"/>
       <c r="G15" s="22"/>
@@ -5689,15 +6396,15 @@
       </c>
       <c r="C16" s="31">
         <f t="shared" ref="C16:E16" si="2">IF(C13&gt;0,C15/C13,0)</f>
-        <v>-0.26532513361153837</v>
+        <v>-0.22916436049491198</v>
       </c>
       <c r="D16" s="31">
         <f t="shared" si="2"/>
-        <v>-0.23237182223947236</v>
+        <v>-0.1920535610324085</v>
       </c>
       <c r="E16" s="31">
         <f t="shared" si="2"/>
-        <v>-0.19519114488683328</v>
+        <v>-0.16086766892450055</v>
       </c>
       <c r="F16" s="21"/>
       <c r="G16" s="22"/>
@@ -5787,15 +6494,15 @@
       </c>
       <c r="C20" s="28">
         <f t="shared" ref="C20:E20" si="4">C15-C19</f>
-        <v>-45029.821428571449</v>
+        <v>-40619.821428571449</v>
       </c>
       <c r="D20" s="28">
         <f t="shared" si="4"/>
-        <v>-142315.57657142862</v>
+        <v>-127475.57657142864</v>
       </c>
       <c r="E20" s="28">
         <f t="shared" si="4"/>
-        <v>-352594.57657142874</v>
+        <v>-330334.57657142874</v>
       </c>
       <c r="F20" s="21"/>
       <c r="G20" s="22"/>
@@ -5843,15 +6550,15 @@
       </c>
       <c r="C23" s="28">
         <f t="shared" ref="C23:E23" si="5">C20-C22</f>
-        <v>-48029.821428571449</v>
+        <v>-43619.821428571449</v>
       </c>
       <c r="D23" s="28">
         <f t="shared" si="5"/>
-        <v>-147315.57657142862</v>
+        <v>-132475.57657142862</v>
       </c>
       <c r="E23" s="28">
         <f t="shared" si="5"/>
-        <v>-362594.57657142874</v>
+        <v>-340334.57657142874</v>
       </c>
       <c r="F23" s="21"/>
       <c r="G23" s="22"/>
@@ -5865,15 +6572,15 @@
       </c>
       <c r="C24" s="28">
         <f>C23</f>
-        <v>-48029.821428571449</v>
+        <v>-43619.821428571449</v>
       </c>
       <c r="D24" s="28">
         <f t="shared" ref="D24:E24" si="6">C24+D23</f>
-        <v>-195345.39800000007</v>
+        <v>-176095.39800000007</v>
       </c>
       <c r="E24" s="28">
         <f t="shared" si="6"/>
-        <v>-557939.97457142884</v>
+        <v>-516429.97457142884</v>
       </c>
       <c r="F24" s="21"/>
       <c r="G24" s="22"/>
@@ -5909,7 +6616,7 @@
       </c>
       <c r="C27" s="17">
         <f>MAX(0,-MIN(C24:E24))</f>
-        <v>557939.97457142884</v>
+        <v>516429.97457142884</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="13" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Finance : TVA dans la trésorerie et CFE dans les frais généraux (28/10/2026)
- Prévisions : onglet TVA (taux par poste en hypothèse, collectée, déductible, reversée, crédit reporté) ; CFE en années 2 et 3
- Trésorerie : ventes encaissées TTC, TVA payée et reversée dans « Impôts et TVA »
- Tableau de bord, fiche des données manquantes et README mis à jour

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/2 FINANCE/PREVISIONS/2026 1027 Modèle - Budget, plan financier, prix et marges.xlsx
+++ b/2 FINANCE/PREVISIONS/2026 1027 Modèle - Budget, plan financier, prix et marges.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vians\Documents\Claude\Projects\HEC-GEMM-Groupe-7\2 FINANCE\PREVISIONS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98E0FF28-2BF8-4335-BED1-F9CA1EC27576}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F55C2F6-4C18-4A9D-B247-0FED85B16C82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{09426CC5-4BCC-48B7-8854-C5C8E2CE30D1}"/>
   </bookViews>
@@ -17,9 +17,10 @@
     <sheet name="Prix et marges" sheetId="2" r:id="rId2"/>
     <sheet name="Staffing" sheetId="7" r:id="rId3"/>
     <sheet name="Budget mensuel" sheetId="3" r:id="rId4"/>
-    <sheet name="Prévu et réel" sheetId="4" r:id="rId5"/>
-    <sheet name="Plan financier 3 ans" sheetId="5" r:id="rId6"/>
-    <sheet name="Frais généraux 3 ans" sheetId="6" r:id="rId7"/>
+    <sheet name="TVA" sheetId="8" r:id="rId5"/>
+    <sheet name="Prévu et réel" sheetId="4" r:id="rId6"/>
+    <sheet name="Plan financier 3 ans" sheetId="5" r:id="rId7"/>
+    <sheet name="Frais généraux 3 ans" sheetId="6" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -45,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="461" uniqueCount="287">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="585" uniqueCount="361">
   <si>
     <t>Prévisions — budget, plan financier, prix et marges</t>
   </si>
@@ -906,19 +907,242 @@
   </si>
   <si>
     <t>Mis à jour le 28/10/2026 : le coût de l'équipe d'une soirée (Prix et marges, ligne 26) suit le scénario S3 des Opérations pour les soirées récurrentes (6 OPERATIONS/PRODUCTION/2026 1028 Scénarios de staffing - leviers de coût.md). Les deux pilotes gardent l'équipe complète (S0) : leur surcoût est ajouté aux coûts directs du budget (Budget mensuel, lignes 37 à 40). Le personnel est toujours fourni par Fou d'un soir.</t>
+  </si>
+  <si>
+    <t>Cotisation foncière des entreprises (CFE)</t>
+  </si>
+  <si>
+    <t>H : cotisation minimum (pas de local en année 2, coworking en année 3), dont le montant dépend de la commune et du chiffre d'affaires. Pas de CFE l'année de création (2026), donc rien en année 1 (novembre 2026 à octobre 2027) ; à confirmer par l'expert-comptable (donnée n° 6)</t>
+  </si>
+  <si>
+    <t>TVA : collectée, déductible et reversée, mois par mois (année 1)</t>
+  </si>
+  <si>
+    <t>Effet de la TVA sur la trésorerie. Le compte de résultat reste hors taxes : la TVA ne change ni la marge ni le résultat, seulement le calendrier des encaissements et des décaissements.</t>
+  </si>
+  <si>
+    <t>Paramètre</t>
+  </si>
+  <si>
+    <t>Choix retenu</t>
+  </si>
+  <si>
+    <t>Source et explication</t>
+  </si>
+  <si>
+    <t>Régime</t>
+  </si>
+  <si>
+    <t>Réel normal, déclaration mensuelle</t>
+  </si>
+  <si>
+    <t>H : la TVA nette d'un mois est reversée à l'État le mois suivant ; à confirmer par l'expert-comptable (donnée n° 6)</t>
+  </si>
+  <si>
+    <t>Crédit de TVA</t>
+  </si>
+  <si>
+    <t>Reporté sur les mois suivants</t>
+  </si>
+  <si>
+    <t>H prudente : aucune demande de remboursement. Un remboursement du crédit peut être demandé ; il améliorerait la trésorerie ; à confirmer par l'expert-comptable (donnée n° 6)</t>
+  </si>
+  <si>
+    <t>TVA collectée sur les ventes</t>
+  </si>
+  <si>
+    <t>Taux moyen de chaque offre (Prix et marges, ligne 12)</t>
+  </si>
+  <si>
+    <t>H : 12 % (10 % sur la restauration, 20 % sur les boissons alcoolisées), déjà utilisé pour passer du TTC au HT</t>
+  </si>
+  <si>
+    <t>Coût d'une soirée</t>
+  </si>
+  <si>
+    <t>Ligne de Prix et marges</t>
+  </si>
+  <si>
+    <t>Taux de TVA déductible</t>
+  </si>
+  <si>
+    <t>Lieu (mise à disposition)</t>
+  </si>
+  <si>
+    <t>H : location facturée avec TVA à 20 %</t>
+  </si>
+  <si>
+    <t>Chef (cachet)</t>
+  </si>
+  <si>
+    <t>H prudente : chef indépendant en franchise de TVA, qui ne facture pas de TVA</t>
+  </si>
+  <si>
+    <t>Matières premières</t>
+  </si>
+  <si>
+    <t>23 × convives</t>
+  </si>
+  <si>
+    <t>H : taux réduit des produits alimentaires (5,5 %)</t>
+  </si>
+  <si>
+    <t>Boissons (vins, alcools)</t>
+  </si>
+  <si>
+    <t>24 × convives</t>
+  </si>
+  <si>
+    <t>H : boissons alcoolisées à 20 %</t>
+  </si>
+  <si>
+    <t>Équipe (extras, brigade, plonge)</t>
+  </si>
+  <si>
+    <t>26 et surcoût des pilotes</t>
+  </si>
+  <si>
+    <t>H : extras facturés par une agence avec TVA à 20 % ; 0 % s'ils étaient salariés en direct</t>
+  </si>
+  <si>
+    <t>Ménage</t>
+  </si>
+  <si>
+    <t>H : assurance exonérée de TVA</t>
+  </si>
+  <si>
+    <t>Décor et fleurs</t>
+  </si>
+  <si>
+    <t>30 × chiffre d'affaires</t>
+  </si>
+  <si>
+    <t>H : services financiers exonérés de TVA</t>
+  </si>
+  <si>
+    <t>Commission d'apporteur</t>
+  </si>
+  <si>
+    <t>31 × chiffre d'affaires</t>
+  </si>
+  <si>
+    <t>Photographe</t>
+  </si>
+  <si>
+    <t>H : 0 % si le photographe est en franchise de TVA</t>
+  </si>
+  <si>
+    <t>Par soirée</t>
+  </si>
+  <si>
+    <t>Privatisation</t>
+  </si>
+  <si>
+    <t>Chiffre d'affaires HT</t>
+  </si>
+  <si>
+    <t>Taux de TVA collectée</t>
+  </si>
+  <si>
+    <t>TVA collectée</t>
+  </si>
+  <si>
+    <t>TVA déductible sur les coûts directs</t>
+  </si>
+  <si>
+    <t>TVA nette de la soirée</t>
+  </si>
+  <si>
+    <t>Frais généraux et investissements</t>
+  </si>
+  <si>
+    <t>Ligne du budget</t>
+  </si>
+  <si>
+    <t>Locaux</t>
+  </si>
+  <si>
+    <t>Logiciels et outils</t>
+  </si>
+  <si>
+    <t>H : dîners de concierges au restaurant à 10 %, le reste à 20 % ; 20 % retenu</t>
+  </si>
+  <si>
+    <t>Assurance RC professionnelle</t>
+  </si>
+  <si>
+    <t>H : assurance exonérée</t>
+  </si>
+  <si>
+    <t>Honoraires</t>
+  </si>
+  <si>
+    <t>H : services bancaires exonérés</t>
+  </si>
+  <si>
+    <t>H : transports à 10 %</t>
+  </si>
+  <si>
+    <t>H prudente : frais de greffe sans TVA</t>
+  </si>
+  <si>
+    <t>Investissements de l'année 1 (en novembre)</t>
+  </si>
+  <si>
+    <t>Plan financier, ligne 22</t>
+  </si>
+  <si>
+    <t>Mois par mois</t>
+  </si>
+  <si>
+    <t>TVA reversée à l'État (due du mois précédent)</t>
+  </si>
+  <si>
+    <t>Crédit de TVA à reporter</t>
+  </si>
+  <si>
+    <t>TVA due au titre du mois</t>
+  </si>
+  <si>
+    <t>Crédit de TVA reporté du mois précédent</t>
+  </si>
+  <si>
+    <t>TVA nette du mois (collectée − déductible)</t>
+  </si>
+  <si>
+    <t>TVA déductible sur les investissements</t>
+  </si>
+  <si>
+    <t>TVA déductible sur les frais généraux</t>
+  </si>
+  <si>
+    <t>Effet de la TVA sur la trésorerie</t>
+  </si>
+  <si>
+    <t>Ligne 51 : reprise dans la trésorerie (2 FINANCE/TRESORERIE, Suivi mensuel) : la TVA collectée s'ajoute aux ventes encaissées, la TVA payée aux fournisseurs et la TVA reversée à l'État vont dans « Impôts et TVA ». Colonne Total, ligne 49 : crédit restant en fin d'année ; la TVA due en octobre est payée en novembre 2027, hors de l'horizon.</t>
+  </si>
+  <si>
+    <t>Non modélisés : impôt sur les sociétés (le plan reste en perte sur 3 ans) ; TVA des années 2 et 3 (effet de calendrier, sans effet sur le résultat). Bons cadeaux : traitement de TVA à préciser avec le Juridique.</t>
+  </si>
+  <si>
+    <t>TVA et CFE</t>
+  </si>
+  <si>
+    <t>Mis à jour le 28/10/2026 : onglet « TVA » (taux par poste en hypothèse, TVA collectée, déductible et reversée chaque mois, crédit reporté) ; son effet sur la trésorerie (ligne 51) est repris dans 2 FINANCE/TRESORERIE. CFE ajoutée aux frais généraux des années 2 et 3 (onglet Frais généraux 3 ans, ligne 24). Le compte de résultat reste hors taxes ; pas d'impôt sur les sociétés (pertes).</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="6">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="#,##0;\-#,##0;&quot;-&quot;"/>
     <numFmt numFmtId="165" formatCode="0.0%;\-0.0%;&quot;-&quot;"/>
     <numFmt numFmtId="166" formatCode="#,##0.00\ &quot;€&quot;;\-#,##0.00\ &quot;€&quot;;&quot;-&quot;"/>
     <numFmt numFmtId="167" formatCode="#,##0\ &quot;€&quot;;\-#,##0\ &quot;€&quot;;&quot;-&quot;"/>
     <numFmt numFmtId="168" formatCode="mmm\ yyyy"/>
     <numFmt numFmtId="169" formatCode="#,##0.0;\-#,##0.0;&quot;-&quot;"/>
+    <numFmt numFmtId="170" formatCode="mmm\ yy"/>
   </numFmts>
   <fonts count="15" x14ac:knownFonts="1">
     <font>
@@ -1090,7 +1314,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1202,7 +1426,7 @@
     <xf numFmtId="167" fontId="10" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
@@ -1215,6 +1439,9 @@
     <xf numFmtId="1" fontId="7" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="165" fontId="7" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="170" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1549,7 +1776,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FBA644DB-8C71-4A8A-A457-0A27A3813ADD}">
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.6328125" style="1" customWidth="1"/>
@@ -1693,6 +1920,14 @@
       </c>
       <c r="B19" s="9" t="s">
         <v>286</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A20" s="8" t="s">
+        <v>359</v>
+      </c>
+      <c r="B20" s="9" t="s">
+        <v>360</v>
       </c>
     </row>
   </sheetData>
@@ -3261,15 +3496,15 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="56" t="str">
-        <f>A7</f>
+        <f t="shared" ref="A26:C34" si="0">A7</f>
         <v>Brigade (second, commis)</v>
       </c>
       <c r="B26" s="57">
-        <f>B7</f>
+        <f t="shared" si="0"/>
         <v>9</v>
       </c>
       <c r="C26" s="58">
-        <f>C7</f>
+        <f t="shared" si="0"/>
         <v>35</v>
       </c>
       <c r="D26" s="20">
@@ -3285,7 +3520,7 @@
         <v>1</v>
       </c>
       <c r="H26" s="59">
-        <f>H7</f>
+        <f t="shared" ref="H26:H34" si="1">H7</f>
         <v>0</v>
       </c>
       <c r="I26" s="22" t="s">
@@ -3294,15 +3529,15 @@
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="56" t="str">
-        <f>A8</f>
+        <f t="shared" si="0"/>
         <v>Maître d'hôtel</v>
       </c>
       <c r="B27" s="57">
-        <f>B8</f>
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="C27" s="58">
-        <f>C8</f>
+        <f t="shared" si="0"/>
         <v>45</v>
       </c>
       <c r="D27" s="20">
@@ -3318,7 +3553,7 @@
         <v>1</v>
       </c>
       <c r="H27" s="59">
-        <f>H8</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="I27" s="22" t="s">
@@ -3327,15 +3562,15 @@
     </row>
     <row r="28" spans="1:9" ht="25" x14ac:dyDescent="0.25">
       <c r="A28" s="56" t="str">
-        <f>A9</f>
+        <f t="shared" si="0"/>
         <v>Serveurs (base)</v>
       </c>
       <c r="B28" s="57">
-        <f>B9</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="C28" s="58">
-        <f>C9</f>
+        <f t="shared" si="0"/>
         <v>35</v>
       </c>
       <c r="D28" s="20">
@@ -3351,7 +3586,7 @@
         <v>2</v>
       </c>
       <c r="H28" s="59">
-        <f>H9</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="I28" s="22" t="s">
@@ -3360,15 +3595,15 @@
     </row>
     <row r="29" spans="1:9" ht="25" x14ac:dyDescent="0.25">
       <c r="A29" s="56" t="str">
-        <f>A10</f>
+        <f t="shared" si="0"/>
         <v>Serveur de réserve</v>
       </c>
       <c r="B29" s="57">
-        <f>B10</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="C29" s="58">
-        <f>C10</f>
+        <f t="shared" si="0"/>
         <v>35</v>
       </c>
       <c r="D29" s="20">
@@ -3384,7 +3619,7 @@
         <v>1</v>
       </c>
       <c r="H29" s="59">
-        <f>H10</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="I29" s="22" t="s">
@@ -3393,15 +3628,15 @@
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="56" t="str">
-        <f>A11</f>
+        <f t="shared" si="0"/>
         <v>Sommelier invité</v>
       </c>
       <c r="B30" s="57">
-        <f>B11</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="C30" s="58">
-        <f>C11</f>
+        <f t="shared" si="0"/>
         <v>60</v>
       </c>
       <c r="D30" s="20">
@@ -3417,7 +3652,7 @@
         <v>1</v>
       </c>
       <c r="H30" s="59">
-        <f>H11</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="I30" s="22" t="s">
@@ -3426,15 +3661,15 @@
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="56" t="str">
-        <f>A12</f>
+        <f t="shared" si="0"/>
         <v>Aide sommelier</v>
       </c>
       <c r="B31" s="57">
-        <f>B12</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="C31" s="58">
-        <f>C12</f>
+        <f t="shared" si="0"/>
         <v>38</v>
       </c>
       <c r="D31" s="20">
@@ -3450,7 +3685,7 @@
         <v>0</v>
       </c>
       <c r="H31" s="59">
-        <f>H12</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="I31" s="22" t="s">
@@ -3459,15 +3694,15 @@
     </row>
     <row r="32" spans="1:9" ht="25" x14ac:dyDescent="0.25">
       <c r="A32" s="56" t="str">
-        <f>A13</f>
+        <f t="shared" si="0"/>
         <v>Plongeurs</v>
       </c>
       <c r="B32" s="57">
-        <f>B13</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="C32" s="58">
-        <f>C13</f>
+        <f t="shared" si="0"/>
         <v>30</v>
       </c>
       <c r="D32" s="20">
@@ -3483,7 +3718,7 @@
         <v>1</v>
       </c>
       <c r="H32" s="59">
-        <f>H13</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="I32" s="22" t="s">
@@ -3492,15 +3727,15 @@
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="56" t="str">
-        <f>A14</f>
+        <f t="shared" si="0"/>
         <v>Responsable de production (nous)</v>
       </c>
       <c r="B33" s="57">
-        <f>B14</f>
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="C33" s="58">
-        <f>C14</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="D33" s="20">
@@ -3516,7 +3751,7 @@
         <v>1</v>
       </c>
       <c r="H33" s="59">
-        <f>H14</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="I33" s="22" t="s">
@@ -3525,15 +3760,15 @@
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" s="56" t="str">
-        <f>A15</f>
+        <f t="shared" si="0"/>
         <v>Interlocuteur client (Ventes)</v>
       </c>
       <c r="B34" s="57">
-        <f>B15</f>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="C34" s="58">
-        <f>C15</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="D34" s="20">
@@ -3549,7 +3784,7 @@
         <v>1</v>
       </c>
       <c r="H34" s="59">
-        <f>H15</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="I34" s="22" t="s">
@@ -5407,6 +5642,1215 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F5433A9-AD53-45CF-A6E8-3A1C7CC9CABA}">
+  <dimension ref="A1:N54"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="44.6328125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="24.6328125" style="1" customWidth="1"/>
+    <col min="3" max="6" width="13.6328125" style="1" customWidth="1"/>
+    <col min="7" max="14" width="12.6328125" style="1" customWidth="1"/>
+    <col min="15" max="16384" width="10.90625" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="18" x14ac:dyDescent="0.4">
+      <c r="A1" s="3" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="13" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="26" x14ac:dyDescent="0.25">
+      <c r="A4" s="6" t="s">
+        <v>291</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>292</v>
+      </c>
+      <c r="C4" s="6"/>
+      <c r="D4" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>294</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>295</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="E5" s="62" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>297</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>298</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="E6" s="62" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>300</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>301</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="E7" s="62" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="39" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
+        <v>303</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>304</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>305</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>306</v>
+      </c>
+      <c r="B10" s="1">
+        <v>19</v>
+      </c>
+      <c r="C10" s="47">
+        <v>0.2</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="E10" s="62" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="B11" s="1">
+        <v>22</v>
+      </c>
+      <c r="C11" s="47">
+        <v>0</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="E11" s="62" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>310</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>311</v>
+      </c>
+      <c r="C12" s="47">
+        <v>5.5E-2</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="E12" s="62" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>313</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>314</v>
+      </c>
+      <c r="C13" s="47">
+        <v>0.2</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="E13" s="62" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>316</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>317</v>
+      </c>
+      <c r="C14" s="47">
+        <v>0.2</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="E14" s="62" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="B15" s="1">
+        <v>27</v>
+      </c>
+      <c r="C15" s="47">
+        <v>0.2</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="E15" s="62" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B16" s="1">
+        <v>28</v>
+      </c>
+      <c r="C16" s="47">
+        <v>0</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="E16" s="62" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>321</v>
+      </c>
+      <c r="B17" s="1">
+        <v>29</v>
+      </c>
+      <c r="C17" s="47">
+        <v>0.2</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="E17" s="62" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>322</v>
+      </c>
+      <c r="C18" s="47">
+        <v>0</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="E18" s="62" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>324</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>325</v>
+      </c>
+      <c r="C19" s="47">
+        <v>0.2</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="E19" s="62" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="B20" s="1">
+        <v>33</v>
+      </c>
+      <c r="C20" s="47">
+        <v>0.2</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="E20" s="62" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="26" x14ac:dyDescent="0.25">
+      <c r="A22" s="6" t="s">
+        <v>328</v>
+      </c>
+      <c r="B22" s="6"/>
+      <c r="C22" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="D22" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="E22" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="F22" s="6" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
+        <v>330</v>
+      </c>
+      <c r="C23" s="16">
+        <f>'Prix et marges'!C17</f>
+        <v>4919.642857142856</v>
+      </c>
+      <c r="D23" s="16">
+        <f>'Prix et marges'!D17</f>
+        <v>7124.9999999999991</v>
+      </c>
+      <c r="E23" s="16">
+        <f>'Prix et marges'!E17</f>
+        <v>9857.1428571428569</v>
+      </c>
+      <c r="F23" s="16">
+        <f>'Prix et marges'!F17</f>
+        <v>8035.7142857142853</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="C24" s="60">
+        <f>'Prix et marges'!C12</f>
+        <v>0.12</v>
+      </c>
+      <c r="D24" s="60">
+        <f>'Prix et marges'!D12</f>
+        <v>0.12</v>
+      </c>
+      <c r="E24" s="60">
+        <f>'Prix et marges'!E12</f>
+        <v>0.12</v>
+      </c>
+      <c r="F24" s="60">
+        <f>'Prix et marges'!F12</f>
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="C25" s="16">
+        <f>C23*C24</f>
+        <v>590.35714285714266</v>
+      </c>
+      <c r="D25" s="16">
+        <f>D23*D24</f>
+        <v>854.99999999999989</v>
+      </c>
+      <c r="E25" s="16">
+        <f>E23*E24</f>
+        <v>1182.8571428571429</v>
+      </c>
+      <c r="F25" s="16">
+        <f>F23*F24</f>
+        <v>964.28571428571422</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
+        <v>333</v>
+      </c>
+      <c r="C26" s="16">
+        <f>'Prix et marges'!C19*$C$10+'Prix et marges'!C22*$C$11+'Prix et marges'!C9*'Prix et marges'!C23*$C$12+'Prix et marges'!C9*'Prix et marges'!C24*$C$13+'Prix et marges'!C26*$C$14+'Prix et marges'!C27*$C$15+'Prix et marges'!C28*$C$16+'Prix et marges'!C29*$C$17+'Prix et marges'!C30*'Prix et marges'!C17*$C$18+'Prix et marges'!C31*'Prix et marges'!C17*$C$19+'Prix et marges'!C33*$C$20</f>
+        <v>1180.6750000000002</v>
+      </c>
+      <c r="D26" s="16">
+        <f>'Prix et marges'!D19*$C$10+'Prix et marges'!D22*$C$11+'Prix et marges'!D9*'Prix et marges'!D23*$C$12+'Prix et marges'!D9*'Prix et marges'!D24*$C$13+'Prix et marges'!D26*$C$14+'Prix et marges'!D27*$C$15+'Prix et marges'!D28*$C$16+'Prix et marges'!D29*$C$17+'Prix et marges'!D30*'Prix et marges'!D17*$C$18+'Prix et marges'!D31*'Prix et marges'!D17*$C$19+'Prix et marges'!D33*$C$20</f>
+        <v>1323.2</v>
+      </c>
+      <c r="E26" s="16">
+        <f>'Prix et marges'!E19*$C$10+'Prix et marges'!E22*$C$11+'Prix et marges'!E9*'Prix et marges'!E23*$C$12+'Prix et marges'!E9*'Prix et marges'!E24*$C$13+'Prix et marges'!E26*$C$14+'Prix et marges'!E27*$C$15+'Prix et marges'!E28*$C$16+'Prix et marges'!E29*$C$17+'Prix et marges'!E30*'Prix et marges'!E17*$C$18+'Prix et marges'!E31*'Prix et marges'!E17*$C$19+'Prix et marges'!E33*$C$20</f>
+        <v>1662.5428571428572</v>
+      </c>
+      <c r="F26" s="16">
+        <f>'Prix et marges'!F19*$C$10+'Prix et marges'!F22*$C$11+'Prix et marges'!F9*'Prix et marges'!F23*$C$12+'Prix et marges'!F9*'Prix et marges'!F24*$C$13+'Prix et marges'!F26*$C$14+'Prix et marges'!F27*$C$15+'Prix et marges'!F28*$C$16+'Prix et marges'!F29*$C$17+'Prix et marges'!F30*'Prix et marges'!F17*$C$18+'Prix et marges'!F31*'Prix et marges'!F17*$C$19+'Prix et marges'!F33*$C$20</f>
+        <v>1116.2142857142858</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" s="1" t="s">
+        <v>334</v>
+      </c>
+      <c r="C27" s="16">
+        <f>C25-C26</f>
+        <v>-590.31785714285752</v>
+      </c>
+      <c r="D27" s="16">
+        <f>D25-D26</f>
+        <v>-468.20000000000016</v>
+      </c>
+      <c r="E27" s="16">
+        <f>E25-E26</f>
+        <v>-479.68571428571431</v>
+      </c>
+      <c r="F27" s="16">
+        <f>F25-F26</f>
+        <v>-151.92857142857156</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="65" x14ac:dyDescent="0.25">
+      <c r="A29" s="6" t="s">
+        <v>335</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>336</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>305</v>
+      </c>
+      <c r="D29" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="E29" s="6" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" s="1" t="s">
+        <v>337</v>
+      </c>
+      <c r="B30" s="1">
+        <v>23</v>
+      </c>
+      <c r="C30" s="47">
+        <v>0.2</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="E30" s="62" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="B31" s="1">
+        <v>24</v>
+      </c>
+      <c r="C31" s="47">
+        <v>0.2</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="E31" s="62" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="B32" s="1">
+        <v>25</v>
+      </c>
+      <c r="C32" s="47">
+        <v>0.2</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="E32" s="62" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="33" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A33" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="B33" s="1">
+        <v>26</v>
+      </c>
+      <c r="C33" s="47">
+        <v>0</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="E33" s="62" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A34" s="1" t="s">
+        <v>342</v>
+      </c>
+      <c r="B34" s="1">
+        <v>27</v>
+      </c>
+      <c r="C34" s="47">
+        <v>0.2</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="E34" s="62" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="35" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A35" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="B35" s="1">
+        <v>28</v>
+      </c>
+      <c r="C35" s="47">
+        <v>0</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="E35" s="62" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="36" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A36" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="B36" s="1">
+        <v>29</v>
+      </c>
+      <c r="C36" s="47">
+        <v>0.1</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="E36" s="62" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A37" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B37" s="1">
+        <v>30</v>
+      </c>
+      <c r="C37" s="47">
+        <v>0</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="E37" s="62" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A38" s="1" t="s">
+        <v>346</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>347</v>
+      </c>
+      <c r="C38" s="47">
+        <v>0.2</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="E38" s="62" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14" ht="13" x14ac:dyDescent="0.3">
+      <c r="A40" s="2" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="41" spans="1:14" ht="26" x14ac:dyDescent="0.3">
+      <c r="A41" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B41" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="C41" s="61">
+        <f>'Budget mensuel'!C5</f>
+        <v>46327</v>
+      </c>
+      <c r="D41" s="61">
+        <f>'Budget mensuel'!D5</f>
+        <v>46357</v>
+      </c>
+      <c r="E41" s="61">
+        <f>'Budget mensuel'!E5</f>
+        <v>46388</v>
+      </c>
+      <c r="F41" s="61">
+        <f>'Budget mensuel'!F5</f>
+        <v>46419</v>
+      </c>
+      <c r="G41" s="61">
+        <f>'Budget mensuel'!G5</f>
+        <v>46447</v>
+      </c>
+      <c r="H41" s="61">
+        <f>'Budget mensuel'!H5</f>
+        <v>46478</v>
+      </c>
+      <c r="I41" s="61">
+        <f>'Budget mensuel'!I5</f>
+        <v>46508</v>
+      </c>
+      <c r="J41" s="61">
+        <f>'Budget mensuel'!J5</f>
+        <v>46539</v>
+      </c>
+      <c r="K41" s="61">
+        <f>'Budget mensuel'!K5</f>
+        <v>46569</v>
+      </c>
+      <c r="L41" s="61">
+        <f>'Budget mensuel'!L5</f>
+        <v>46600</v>
+      </c>
+      <c r="M41" s="61">
+        <f>'Budget mensuel'!M5</f>
+        <v>46631</v>
+      </c>
+      <c r="N41" s="61">
+        <f>'Budget mensuel'!N5</f>
+        <v>46661</v>
+      </c>
+    </row>
+    <row r="42" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A42" s="1" t="s">
+        <v>300</v>
+      </c>
+      <c r="B42" s="16">
+        <f>SUM(C42:N42)</f>
+        <v>14634.642857142855</v>
+      </c>
+      <c r="C42" s="16">
+        <f>'Budget mensuel'!C7*$C$25+'Budget mensuel'!C8*$D$25+'Budget mensuel'!C9*$E$25+'Budget mensuel'!C10*$F$25</f>
+        <v>0</v>
+      </c>
+      <c r="D42" s="16">
+        <f>'Budget mensuel'!D7*$C$25+'Budget mensuel'!D8*$D$25+'Budget mensuel'!D9*$E$25+'Budget mensuel'!D10*$F$25</f>
+        <v>0</v>
+      </c>
+      <c r="E42" s="16">
+        <f>'Budget mensuel'!E7*$C$25+'Budget mensuel'!E8*$D$25+'Budget mensuel'!E9*$E$25+'Budget mensuel'!E10*$F$25</f>
+        <v>590.35714285714266</v>
+      </c>
+      <c r="F42" s="16">
+        <f>'Budget mensuel'!F7*$C$25+'Budget mensuel'!F8*$D$25+'Budget mensuel'!F9*$E$25+'Budget mensuel'!F10*$F$25</f>
+        <v>1182.8571428571429</v>
+      </c>
+      <c r="G42" s="16">
+        <f>'Budget mensuel'!G7*$C$25+'Budget mensuel'!G8*$D$25+'Budget mensuel'!G9*$E$25+'Budget mensuel'!G10*$F$25</f>
+        <v>854.99999999999989</v>
+      </c>
+      <c r="H42" s="16">
+        <f>'Budget mensuel'!H7*$C$25+'Budget mensuel'!H8*$D$25+'Budget mensuel'!H9*$E$25+'Budget mensuel'!H10*$F$25</f>
+        <v>1554.6428571428569</v>
+      </c>
+      <c r="I42" s="16">
+        <f>'Budget mensuel'!I7*$C$25+'Budget mensuel'!I8*$D$25+'Budget mensuel'!I9*$E$25+'Budget mensuel'!I10*$F$25</f>
+        <v>2147.1428571428569</v>
+      </c>
+      <c r="J42" s="16">
+        <f>'Budget mensuel'!J7*$C$25+'Budget mensuel'!J8*$D$25+'Budget mensuel'!J9*$E$25+'Budget mensuel'!J10*$F$25</f>
+        <v>1819.2857142857142</v>
+      </c>
+      <c r="K42" s="16">
+        <f>'Budget mensuel'!K7*$C$25+'Budget mensuel'!K8*$D$25+'Budget mensuel'!K9*$E$25+'Budget mensuel'!K10*$F$25</f>
+        <v>590.35714285714266</v>
+      </c>
+      <c r="L42" s="16">
+        <f>'Budget mensuel'!L7*$C$25+'Budget mensuel'!L8*$D$25+'Budget mensuel'!L9*$E$25+'Budget mensuel'!L10*$F$25</f>
+        <v>0</v>
+      </c>
+      <c r="M42" s="16">
+        <f>'Budget mensuel'!M7*$C$25+'Budget mensuel'!M8*$D$25+'Budget mensuel'!M9*$E$25+'Budget mensuel'!M10*$F$25</f>
+        <v>3111.4285714285716</v>
+      </c>
+      <c r="N42" s="16">
+        <f>'Budget mensuel'!N7*$C$25+'Budget mensuel'!N8*$D$25+'Budget mensuel'!N9*$E$25+'Budget mensuel'!N10*$F$25</f>
+        <v>2783.5714285714284</v>
+      </c>
+    </row>
+    <row r="43" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A43" s="1" t="s">
+        <v>333</v>
+      </c>
+      <c r="B43" s="16">
+        <f>SUM(C43:N43)</f>
+        <v>20543.75357142857</v>
+      </c>
+      <c r="C43" s="16">
+        <f>'Budget mensuel'!C7*$C$26+'Budget mensuel'!C8*$D$26+'Budget mensuel'!C9*$E$26+'Budget mensuel'!C10*$F$26+'Budget mensuel'!C40*$C$14</f>
+        <v>0</v>
+      </c>
+      <c r="D43" s="16">
+        <f>'Budget mensuel'!D7*$C$26+'Budget mensuel'!D8*$D$26+'Budget mensuel'!D9*$E$26+'Budget mensuel'!D10*$F$26+'Budget mensuel'!D40*$C$14</f>
+        <v>0</v>
+      </c>
+      <c r="E43" s="16">
+        <f>'Budget mensuel'!E7*$C$26+'Budget mensuel'!E8*$D$26+'Budget mensuel'!E9*$E$26+'Budget mensuel'!E10*$F$26+'Budget mensuel'!E40*$C$14</f>
+        <v>1320.6750000000002</v>
+      </c>
+      <c r="F43" s="16">
+        <f>'Budget mensuel'!F7*$C$26+'Budget mensuel'!F8*$D$26+'Budget mensuel'!F9*$E$26+'Budget mensuel'!F10*$F$26+'Budget mensuel'!F40*$C$14</f>
+        <v>1753.5428571428572</v>
+      </c>
+      <c r="G43" s="16">
+        <f>'Budget mensuel'!G7*$C$26+'Budget mensuel'!G8*$D$26+'Budget mensuel'!G9*$E$26+'Budget mensuel'!G10*$F$26+'Budget mensuel'!G40*$C$14</f>
+        <v>1323.2</v>
+      </c>
+      <c r="H43" s="16">
+        <f>'Budget mensuel'!H7*$C$26+'Budget mensuel'!H8*$D$26+'Budget mensuel'!H9*$E$26+'Budget mensuel'!H10*$F$26+'Budget mensuel'!H40*$C$14</f>
+        <v>2296.889285714286</v>
+      </c>
+      <c r="I43" s="16">
+        <f>'Budget mensuel'!I7*$C$26+'Budget mensuel'!I8*$D$26+'Budget mensuel'!I9*$E$26+'Budget mensuel'!I10*$F$26+'Budget mensuel'!I40*$C$14</f>
+        <v>2778.7571428571428</v>
+      </c>
+      <c r="J43" s="16">
+        <f>'Budget mensuel'!J7*$C$26+'Budget mensuel'!J8*$D$26+'Budget mensuel'!J9*$E$26+'Budget mensuel'!J10*$F$26+'Budget mensuel'!J40*$C$14</f>
+        <v>2439.4142857142861</v>
+      </c>
+      <c r="K43" s="16">
+        <f>'Budget mensuel'!K7*$C$26+'Budget mensuel'!K8*$D$26+'Budget mensuel'!K9*$E$26+'Budget mensuel'!K10*$F$26+'Budget mensuel'!K40*$C$14</f>
+        <v>1180.6750000000002</v>
+      </c>
+      <c r="L43" s="16">
+        <f>'Budget mensuel'!L7*$C$26+'Budget mensuel'!L8*$D$26+'Budget mensuel'!L9*$E$26+'Budget mensuel'!L10*$F$26+'Budget mensuel'!L40*$C$14</f>
+        <v>0</v>
+      </c>
+      <c r="M43" s="16">
+        <f>'Budget mensuel'!M7*$C$26+'Budget mensuel'!M8*$D$26+'Budget mensuel'!M9*$E$26+'Budget mensuel'!M10*$F$26+'Budget mensuel'!M40*$C$14</f>
+        <v>3894.971428571429</v>
+      </c>
+      <c r="N43" s="16">
+        <f>'Budget mensuel'!N7*$C$26+'Budget mensuel'!N8*$D$26+'Budget mensuel'!N9*$E$26+'Budget mensuel'!N10*$F$26+'Budget mensuel'!N40*$C$14</f>
+        <v>3555.6285714285714</v>
+      </c>
+    </row>
+    <row r="44" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A44" s="1" t="s">
+        <v>355</v>
+      </c>
+      <c r="B44" s="16">
+        <f>SUM(C44:N44)</f>
+        <v>2232</v>
+      </c>
+      <c r="C44" s="16">
+        <f>'Budget mensuel'!C23*$C$30+'Budget mensuel'!C24*$C$31+'Budget mensuel'!C25*$C$32+'Budget mensuel'!C26*$C$33+'Budget mensuel'!C27*$C$34+'Budget mensuel'!C28*$C$35+'Budget mensuel'!C29*$C$36+'Budget mensuel'!C30*$C$37</f>
+        <v>401</v>
+      </c>
+      <c r="D44" s="16">
+        <f>'Budget mensuel'!D23*$C$30+'Budget mensuel'!D24*$C$31+'Budget mensuel'!D25*$C$32+'Budget mensuel'!D26*$C$33+'Budget mensuel'!D27*$C$34+'Budget mensuel'!D28*$C$35+'Budget mensuel'!D29*$C$36+'Budget mensuel'!D30*$C$37</f>
+        <v>341</v>
+      </c>
+      <c r="E44" s="16">
+        <f>'Budget mensuel'!E23*$C$30+'Budget mensuel'!E24*$C$31+'Budget mensuel'!E25*$C$32+'Budget mensuel'!E26*$C$33+'Budget mensuel'!E27*$C$34+'Budget mensuel'!E28*$C$35+'Budget mensuel'!E29*$C$36+'Budget mensuel'!E30*$C$37</f>
+        <v>341</v>
+      </c>
+      <c r="F44" s="16">
+        <f>'Budget mensuel'!F23*$C$30+'Budget mensuel'!F24*$C$31+'Budget mensuel'!F25*$C$32+'Budget mensuel'!F26*$C$33+'Budget mensuel'!F27*$C$34+'Budget mensuel'!F28*$C$35+'Budget mensuel'!F29*$C$36+'Budget mensuel'!F30*$C$37</f>
+        <v>341</v>
+      </c>
+      <c r="G44" s="16">
+        <f>'Budget mensuel'!G23*$C$30+'Budget mensuel'!G24*$C$31+'Budget mensuel'!G25*$C$32+'Budget mensuel'!G26*$C$33+'Budget mensuel'!G27*$C$34+'Budget mensuel'!G28*$C$35+'Budget mensuel'!G29*$C$36+'Budget mensuel'!G30*$C$37</f>
+        <v>101</v>
+      </c>
+      <c r="H44" s="16">
+        <f>'Budget mensuel'!H23*$C$30+'Budget mensuel'!H24*$C$31+'Budget mensuel'!H25*$C$32+'Budget mensuel'!H26*$C$33+'Budget mensuel'!H27*$C$34+'Budget mensuel'!H28*$C$35+'Budget mensuel'!H29*$C$36+'Budget mensuel'!H30*$C$37</f>
+        <v>101</v>
+      </c>
+      <c r="I44" s="16">
+        <f>'Budget mensuel'!I23*$C$30+'Budget mensuel'!I24*$C$31+'Budget mensuel'!I25*$C$32+'Budget mensuel'!I26*$C$33+'Budget mensuel'!I27*$C$34+'Budget mensuel'!I28*$C$35+'Budget mensuel'!I29*$C$36+'Budget mensuel'!I30*$C$37</f>
+        <v>101</v>
+      </c>
+      <c r="J44" s="16">
+        <f>'Budget mensuel'!J23*$C$30+'Budget mensuel'!J24*$C$31+'Budget mensuel'!J25*$C$32+'Budget mensuel'!J26*$C$33+'Budget mensuel'!J27*$C$34+'Budget mensuel'!J28*$C$35+'Budget mensuel'!J29*$C$36+'Budget mensuel'!J30*$C$37</f>
+        <v>101</v>
+      </c>
+      <c r="K44" s="16">
+        <f>'Budget mensuel'!K23*$C$30+'Budget mensuel'!K24*$C$31+'Budget mensuel'!K25*$C$32+'Budget mensuel'!K26*$C$33+'Budget mensuel'!K27*$C$34+'Budget mensuel'!K28*$C$35+'Budget mensuel'!K29*$C$36+'Budget mensuel'!K30*$C$37</f>
+        <v>101</v>
+      </c>
+      <c r="L44" s="16">
+        <f>'Budget mensuel'!L23*$C$30+'Budget mensuel'!L24*$C$31+'Budget mensuel'!L25*$C$32+'Budget mensuel'!L26*$C$33+'Budget mensuel'!L27*$C$34+'Budget mensuel'!L28*$C$35+'Budget mensuel'!L29*$C$36+'Budget mensuel'!L30*$C$37</f>
+        <v>101</v>
+      </c>
+      <c r="M44" s="16">
+        <f>'Budget mensuel'!M23*$C$30+'Budget mensuel'!M24*$C$31+'Budget mensuel'!M25*$C$32+'Budget mensuel'!M26*$C$33+'Budget mensuel'!M27*$C$34+'Budget mensuel'!M28*$C$35+'Budget mensuel'!M29*$C$36+'Budget mensuel'!M30*$C$37</f>
+        <v>101</v>
+      </c>
+      <c r="N44" s="16">
+        <f>'Budget mensuel'!N23*$C$30+'Budget mensuel'!N24*$C$31+'Budget mensuel'!N25*$C$32+'Budget mensuel'!N26*$C$33+'Budget mensuel'!N27*$C$34+'Budget mensuel'!N28*$C$35+'Budget mensuel'!N29*$C$36+'Budget mensuel'!N30*$C$37</f>
+        <v>101</v>
+      </c>
+    </row>
+    <row r="45" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A45" s="1" t="s">
+        <v>354</v>
+      </c>
+      <c r="B45" s="16">
+        <f>SUM(C45:N45)</f>
+        <v>600</v>
+      </c>
+      <c r="C45" s="16">
+        <f>'Plan financier 3 ans'!$C$22*$C$38</f>
+        <v>600</v>
+      </c>
+      <c r="D45" s="16">
+        <v>0</v>
+      </c>
+      <c r="E45" s="16">
+        <v>0</v>
+      </c>
+      <c r="F45" s="16">
+        <v>0</v>
+      </c>
+      <c r="G45" s="16">
+        <v>0</v>
+      </c>
+      <c r="H45" s="16">
+        <v>0</v>
+      </c>
+      <c r="I45" s="16">
+        <v>0</v>
+      </c>
+      <c r="J45" s="16">
+        <v>0</v>
+      </c>
+      <c r="K45" s="16">
+        <v>0</v>
+      </c>
+      <c r="L45" s="16">
+        <v>0</v>
+      </c>
+      <c r="M45" s="16">
+        <v>0</v>
+      </c>
+      <c r="N45" s="16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:14" ht="13" x14ac:dyDescent="0.3">
+      <c r="A46" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="B46" s="17">
+        <f>SUM(C46:N46)</f>
+        <v>-8741.1107142857163</v>
+      </c>
+      <c r="C46" s="17">
+        <f>C42-C43-C44-C45</f>
+        <v>-1001</v>
+      </c>
+      <c r="D46" s="17">
+        <f>D42-D43-D44-D45</f>
+        <v>-341</v>
+      </c>
+      <c r="E46" s="17">
+        <f>E42-E43-E44-E45</f>
+        <v>-1071.3178571428575</v>
+      </c>
+      <c r="F46" s="17">
+        <f>F42-F43-F44-F45</f>
+        <v>-911.68571428571431</v>
+      </c>
+      <c r="G46" s="17">
+        <f>G42-G43-G44-G45</f>
+        <v>-569.20000000000016</v>
+      </c>
+      <c r="H46" s="17">
+        <f>H42-H43-H44-H45</f>
+        <v>-843.24642857142908</v>
+      </c>
+      <c r="I46" s="17">
+        <f>I42-I43-I44-I45</f>
+        <v>-732.61428571428587</v>
+      </c>
+      <c r="J46" s="17">
+        <f>J42-J43-J44-J45</f>
+        <v>-721.12857142857183</v>
+      </c>
+      <c r="K46" s="17">
+        <f>K42-K43-K44-K45</f>
+        <v>-691.31785714285752</v>
+      </c>
+      <c r="L46" s="17">
+        <f>L42-L43-L44-L45</f>
+        <v>-101</v>
+      </c>
+      <c r="M46" s="17">
+        <f>M42-M43-M44-M45</f>
+        <v>-884.54285714285743</v>
+      </c>
+      <c r="N46" s="17">
+        <f>N42-N43-N44-N45</f>
+        <v>-873.05714285714294</v>
+      </c>
+    </row>
+    <row r="47" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A47" s="1" t="s">
+        <v>352</v>
+      </c>
+      <c r="B47" s="16">
+        <f>C47</f>
+        <v>0</v>
+      </c>
+      <c r="C47" s="16">
+        <v>0</v>
+      </c>
+      <c r="D47" s="16">
+        <f>C49</f>
+        <v>1001</v>
+      </c>
+      <c r="E47" s="16">
+        <f>D49</f>
+        <v>1342</v>
+      </c>
+      <c r="F47" s="16">
+        <f>E49</f>
+        <v>2413.3178571428575</v>
+      </c>
+      <c r="G47" s="16">
+        <f>F49</f>
+        <v>3325.0035714285718</v>
+      </c>
+      <c r="H47" s="16">
+        <f>G49</f>
+        <v>3894.2035714285721</v>
+      </c>
+      <c r="I47" s="16">
+        <f>H49</f>
+        <v>4737.4500000000007</v>
+      </c>
+      <c r="J47" s="16">
+        <f>I49</f>
+        <v>5470.0642857142866</v>
+      </c>
+      <c r="K47" s="16">
+        <f>J49</f>
+        <v>6191.192857142858</v>
+      </c>
+      <c r="L47" s="16">
+        <f>K49</f>
+        <v>6882.5107142857159</v>
+      </c>
+      <c r="M47" s="16">
+        <f>L49</f>
+        <v>6983.5107142857159</v>
+      </c>
+      <c r="N47" s="16">
+        <f>M49</f>
+        <v>7868.0535714285734</v>
+      </c>
+    </row>
+    <row r="48" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A48" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="B48" s="16">
+        <f>SUM(C48:N48)</f>
+        <v>0</v>
+      </c>
+      <c r="C48" s="16">
+        <f>MAX(0,C46-C47)</f>
+        <v>0</v>
+      </c>
+      <c r="D48" s="16">
+        <f>MAX(0,D46-D47)</f>
+        <v>0</v>
+      </c>
+      <c r="E48" s="16">
+        <f>MAX(0,E46-E47)</f>
+        <v>0</v>
+      </c>
+      <c r="F48" s="16">
+        <f>MAX(0,F46-F47)</f>
+        <v>0</v>
+      </c>
+      <c r="G48" s="16">
+        <f>MAX(0,G46-G47)</f>
+        <v>0</v>
+      </c>
+      <c r="H48" s="16">
+        <f>MAX(0,H46-H47)</f>
+        <v>0</v>
+      </c>
+      <c r="I48" s="16">
+        <f>MAX(0,I46-I47)</f>
+        <v>0</v>
+      </c>
+      <c r="J48" s="16">
+        <f>MAX(0,J46-J47)</f>
+        <v>0</v>
+      </c>
+      <c r="K48" s="16">
+        <f>MAX(0,K46-K47)</f>
+        <v>0</v>
+      </c>
+      <c r="L48" s="16">
+        <f>MAX(0,L46-L47)</f>
+        <v>0</v>
+      </c>
+      <c r="M48" s="16">
+        <f>MAX(0,M46-M47)</f>
+        <v>0</v>
+      </c>
+      <c r="N48" s="16">
+        <f>MAX(0,N46-N47)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A49" s="1" t="s">
+        <v>350</v>
+      </c>
+      <c r="B49" s="16">
+        <f>N49</f>
+        <v>8741.1107142857163</v>
+      </c>
+      <c r="C49" s="16">
+        <f>MAX(0,C47-C46)</f>
+        <v>1001</v>
+      </c>
+      <c r="D49" s="16">
+        <f>MAX(0,D47-D46)</f>
+        <v>1342</v>
+      </c>
+      <c r="E49" s="16">
+        <f>MAX(0,E47-E46)</f>
+        <v>2413.3178571428575</v>
+      </c>
+      <c r="F49" s="16">
+        <f>MAX(0,F47-F46)</f>
+        <v>3325.0035714285718</v>
+      </c>
+      <c r="G49" s="16">
+        <f>MAX(0,G47-G46)</f>
+        <v>3894.2035714285721</v>
+      </c>
+      <c r="H49" s="16">
+        <f>MAX(0,H47-H46)</f>
+        <v>4737.4500000000007</v>
+      </c>
+      <c r="I49" s="16">
+        <f>MAX(0,I47-I46)</f>
+        <v>5470.0642857142866</v>
+      </c>
+      <c r="J49" s="16">
+        <f>MAX(0,J47-J46)</f>
+        <v>6191.192857142858</v>
+      </c>
+      <c r="K49" s="16">
+        <f>MAX(0,K47-K46)</f>
+        <v>6882.5107142857159</v>
+      </c>
+      <c r="L49" s="16">
+        <f>MAX(0,L47-L46)</f>
+        <v>6983.5107142857159</v>
+      </c>
+      <c r="M49" s="16">
+        <f>MAX(0,M47-M46)</f>
+        <v>7868.0535714285734</v>
+      </c>
+      <c r="N49" s="16">
+        <f>MAX(0,N47-N46)</f>
+        <v>8741.1107142857163</v>
+      </c>
+    </row>
+    <row r="50" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A50" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="B50" s="16">
+        <f>SUM(C50:N50)</f>
+        <v>0</v>
+      </c>
+      <c r="C50" s="16">
+        <v>0</v>
+      </c>
+      <c r="D50" s="16">
+        <f>C48</f>
+        <v>0</v>
+      </c>
+      <c r="E50" s="16">
+        <f>D48</f>
+        <v>0</v>
+      </c>
+      <c r="F50" s="16">
+        <f>E48</f>
+        <v>0</v>
+      </c>
+      <c r="G50" s="16">
+        <f>F48</f>
+        <v>0</v>
+      </c>
+      <c r="H50" s="16">
+        <f>G48</f>
+        <v>0</v>
+      </c>
+      <c r="I50" s="16">
+        <f>H48</f>
+        <v>0</v>
+      </c>
+      <c r="J50" s="16">
+        <f>I48</f>
+        <v>0</v>
+      </c>
+      <c r="K50" s="16">
+        <f>J48</f>
+        <v>0</v>
+      </c>
+      <c r="L50" s="16">
+        <f>K48</f>
+        <v>0</v>
+      </c>
+      <c r="M50" s="16">
+        <f>L48</f>
+        <v>0</v>
+      </c>
+      <c r="N50" s="16">
+        <f>M48</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:14" ht="13" x14ac:dyDescent="0.3">
+      <c r="A51" s="45" t="s">
+        <v>356</v>
+      </c>
+      <c r="B51" s="46">
+        <f>SUM(C51:N51)</f>
+        <v>-8741.1107142857163</v>
+      </c>
+      <c r="C51" s="46">
+        <f>C42-C43-C44-C45-C50</f>
+        <v>-1001</v>
+      </c>
+      <c r="D51" s="46">
+        <f>D42-D43-D44-D45-D50</f>
+        <v>-341</v>
+      </c>
+      <c r="E51" s="46">
+        <f>E42-E43-E44-E45-E50</f>
+        <v>-1071.3178571428575</v>
+      </c>
+      <c r="F51" s="46">
+        <f>F42-F43-F44-F45-F50</f>
+        <v>-911.68571428571431</v>
+      </c>
+      <c r="G51" s="46">
+        <f>G42-G43-G44-G45-G50</f>
+        <v>-569.20000000000016</v>
+      </c>
+      <c r="H51" s="46">
+        <f>H42-H43-H44-H45-H50</f>
+        <v>-843.24642857142908</v>
+      </c>
+      <c r="I51" s="46">
+        <f>I42-I43-I44-I45-I50</f>
+        <v>-732.61428571428587</v>
+      </c>
+      <c r="J51" s="46">
+        <f>J42-J43-J44-J45-J50</f>
+        <v>-721.12857142857183</v>
+      </c>
+      <c r="K51" s="46">
+        <f>K42-K43-K44-K45-K50</f>
+        <v>-691.31785714285752</v>
+      </c>
+      <c r="L51" s="46">
+        <f>L42-L43-L44-L45-L50</f>
+        <v>-101</v>
+      </c>
+      <c r="M51" s="46">
+        <f>M42-M43-M44-M45-M50</f>
+        <v>-884.54285714285743</v>
+      </c>
+      <c r="N51" s="46">
+        <f>N42-N43-N44-N45-N50</f>
+        <v>-873.05714285714294</v>
+      </c>
+    </row>
+    <row r="53" spans="1:14" ht="13" x14ac:dyDescent="0.3">
+      <c r="A53" s="4" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="54" spans="1:14" ht="13" x14ac:dyDescent="0.3">
+      <c r="A54" s="4" t="s">
+        <v>358</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9898DBE-F173-4946-8908-F62FA6ACEF06}">
   <dimension ref="A1:N27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
@@ -6135,7 +7579,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42FB26B6-A531-4D48-8F04-B3463A220999}">
   <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
@@ -6447,12 +7891,12 @@
         <v>12672</v>
       </c>
       <c r="D18" s="50">
-        <f>'Frais généraux 3 ans'!$F$25</f>
-        <v>24300</v>
+        <f>'Frais généraux 3 ans'!$F$26</f>
+        <v>24600</v>
       </c>
       <c r="E18" s="50">
-        <f>'Frais généraux 3 ans'!$G$25</f>
-        <v>57800</v>
+        <f>'Frais généraux 3 ans'!$G$26</f>
+        <v>58400</v>
       </c>
       <c r="F18" s="40" t="s">
         <v>89</v>
@@ -6474,11 +7918,11 @@
       </c>
       <c r="D19" s="28">
         <f t="shared" si="3"/>
-        <v>56786.148000000001</v>
+        <v>57086.148000000001</v>
       </c>
       <c r="E19" s="28">
         <f t="shared" si="3"/>
-        <v>226006.14799999999</v>
+        <v>226606.14799999999</v>
       </c>
       <c r="F19" s="21"/>
       <c r="G19" s="22" t="s">
@@ -6498,11 +7942,11 @@
       </c>
       <c r="D20" s="28">
         <f t="shared" si="4"/>
-        <v>-127475.57657142864</v>
+        <v>-127775.57657142864</v>
       </c>
       <c r="E20" s="28">
         <f t="shared" si="4"/>
-        <v>-330334.57657142874</v>
+        <v>-330934.57657142874</v>
       </c>
       <c r="F20" s="21"/>
       <c r="G20" s="22"/>
@@ -6554,11 +7998,11 @@
       </c>
       <c r="D23" s="28">
         <f t="shared" si="5"/>
-        <v>-132475.57657142862</v>
+        <v>-132775.57657142862</v>
       </c>
       <c r="E23" s="28">
         <f t="shared" si="5"/>
-        <v>-340334.57657142874</v>
+        <v>-340934.57657142874</v>
       </c>
       <c r="F23" s="21"/>
       <c r="G23" s="22"/>
@@ -6576,11 +8020,11 @@
       </c>
       <c r="D24" s="28">
         <f t="shared" ref="D24:E24" si="6">C24+D23</f>
-        <v>-176095.39800000007</v>
+        <v>-176395.39800000007</v>
       </c>
       <c r="E24" s="28">
         <f t="shared" si="6"/>
-        <v>-516429.97457142884</v>
+        <v>-517329.97457142884</v>
       </c>
       <c r="F24" s="21"/>
       <c r="G24" s="22"/>
@@ -6616,7 +8060,7 @@
       </c>
       <c r="C27" s="17">
         <f>MAX(0,-MIN(C24:E24))</f>
-        <v>516429.97457142884</v>
+        <v>517329.97457142884</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="13" x14ac:dyDescent="0.3">
@@ -6634,9 +8078,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C299EF4-2BFD-4A30-9CB8-0FD18304D49C}">
-  <dimension ref="A1:I27"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="46.6328125" style="1" customWidth="1"/>
@@ -7053,64 +8497,85 @@
         <v>217</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" ht="50" x14ac:dyDescent="0.25">
       <c r="A24" s="19" t="s">
-        <v>218</v>
+        <v>287</v>
       </c>
       <c r="B24" s="19"/>
       <c r="C24" s="19"/>
       <c r="D24" s="19"/>
       <c r="E24" s="19"/>
       <c r="F24" s="26">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="G24" s="26">
-        <v>1000</v>
+        <v>600</v>
       </c>
       <c r="H24" s="21" t="s">
         <v>89</v>
       </c>
       <c r="I24" s="22" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A25" s="19" t="s">
+        <v>218</v>
+      </c>
+      <c r="B25" s="19"/>
+      <c r="C25" s="19"/>
+      <c r="D25" s="19"/>
+      <c r="E25" s="19"/>
+      <c r="F25" s="26">
+        <v>0</v>
+      </c>
+      <c r="G25" s="26">
+        <v>1000</v>
+      </c>
+      <c r="H25" s="21" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="25" spans="1:9" ht="13" x14ac:dyDescent="0.3">
-      <c r="A25" s="2" t="s">
+      <c r="I25" s="22" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" ht="13" x14ac:dyDescent="0.3">
+      <c r="A26" s="2" t="s">
         <v>189</v>
       </c>
-      <c r="B25" s="2"/>
-      <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
-      <c r="E25" s="2"/>
-      <c r="F25" s="17">
-        <f>SUM(F17:F24)</f>
-        <v>24300</v>
-      </c>
-      <c r="G25" s="17">
-        <f>SUM(G17:G24)</f>
-        <v>57800</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9" ht="13" x14ac:dyDescent="0.3">
-      <c r="A27" s="45" t="s">
+      <c r="B26" s="2"/>
+      <c r="C26" s="2"/>
+      <c r="D26" s="2"/>
+      <c r="E26" s="2"/>
+      <c r="F26" s="17">
+        <f>SUM(F17:F25)</f>
+        <v>24600</v>
+      </c>
+      <c r="G26" s="17">
+        <f>SUM(G17:G25)</f>
+        <v>58400</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" ht="13" x14ac:dyDescent="0.3">
+      <c r="A28" s="45" t="s">
         <v>190</v>
       </c>
-      <c r="B27" s="45"/>
-      <c r="C27" s="45"/>
-      <c r="D27" s="45"/>
-      <c r="E27" s="45"/>
-      <c r="F27" s="46">
-        <f>F13+F25</f>
-        <v>56786.148000000001</v>
-      </c>
-      <c r="G27" s="46">
-        <f>G13+G25</f>
-        <v>226006.14799999999</v>
+      <c r="B28" s="45"/>
+      <c r="C28" s="45"/>
+      <c r="D28" s="45"/>
+      <c r="E28" s="45"/>
+      <c r="F28" s="46">
+        <f>F13+F26</f>
+        <v>57086.148000000001</v>
+      </c>
+      <c r="G28" s="46">
+        <f>G13+G26</f>
+        <v>226606.14799999999</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H8:H24" xr:uid="{17BF4D97-1CC3-431D-AE47-E54A12C319AD}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H8:H25" xr:uid="{17BF4D97-1CC3-431D-AE47-E54A12C319AD}">
       <formula1>"F,I,P,H"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Finance : hypothèses de prévision modifiées et note aux Opérations, au Produit et au Marketing (28/10/2026)
- Prévisions : jauges 40 / 35 / 30 / 20, salle pleine, équipe à 15 ou 20 % du CA, sans photographe (modification du responsable Finance)
- Trésorerie et tableau de bord recalculés
- Note listant les modifications, leurs effets et les questions aux trois pôles ; fiche et README mis à jour

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/2 FINANCE/PREVISIONS/2026 1027 Modèle - Budget, plan financier, prix et marges.xlsx
+++ b/2 FINANCE/PREVISIONS/2026 1027 Modèle - Budget, plan financier, prix et marges.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vians\Documents\Claude\Projects\HEC-GEMM-Groupe-7\2 FINANCE\PREVISIONS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F55C2F6-4C18-4A9D-B247-0FED85B16C82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52E9816D-4B05-4B99-BC98-E6881055BFEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{09426CC5-4BCC-48B7-8854-C5C8E2CE30D1}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" activeTab="3" xr2:uid="{09426CC5-4BCC-48B7-8854-C5C8E2CE30D1}"/>
   </bookViews>
   <sheets>
     <sheet name="Mode d'emploi" sheetId="1" r:id="rId1"/>
@@ -1314,7 +1314,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1441,7 +1441,6 @@
     </xf>
     <xf numFmtId="165" fontId="7" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="170" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2015,16 +2014,16 @@
         <v>42</v>
       </c>
       <c r="C7" s="20">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="D7" s="20">
-        <v>24</v>
+        <v>35</v>
       </c>
       <c r="E7" s="20">
+        <v>30</v>
+      </c>
+      <c r="F7" s="20">
         <v>20</v>
-      </c>
-      <c r="F7" s="20">
-        <v>10</v>
       </c>
       <c r="G7" s="21" t="s">
         <v>86</v>
@@ -2044,13 +2043,13 @@
         <v>44</v>
       </c>
       <c r="C8" s="23">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="D8" s="23">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="E8" s="23">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="F8" s="23">
         <v>1</v>
@@ -2074,19 +2073,19 @@
       </c>
       <c r="C9" s="24">
         <f t="shared" ref="C9:F9" si="0">ROUND(C7*C8,0)</f>
-        <v>19</v>
+        <v>40</v>
       </c>
       <c r="D9" s="24">
         <f t="shared" si="0"/>
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="E9" s="24">
         <f t="shared" si="0"/>
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="F9" s="24">
         <f t="shared" si="0"/>
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="G9" s="21"/>
       <c r="H9" s="22"/>
@@ -2300,19 +2299,19 @@
       </c>
       <c r="C17" s="28">
         <f t="shared" ref="C17:F17" si="3">MAX(C9*C13+C14,C15)+C16</f>
-        <v>4919.642857142856</v>
+        <v>10357.142857142855</v>
       </c>
       <c r="D17" s="28">
         <f t="shared" si="3"/>
-        <v>7124.9999999999991</v>
+        <v>13124.999999999998</v>
       </c>
       <c r="E17" s="28">
         <f t="shared" si="3"/>
-        <v>9857.1428571428569</v>
+        <v>18482.142857142855</v>
       </c>
       <c r="F17" s="28">
-        <f t="shared" si="3"/>
-        <v>8035.7142857142853</v>
+        <f>MAX(F9*F13+F14,F15)+F16</f>
+        <v>10714.285714285714</v>
       </c>
       <c r="G17" s="21"/>
       <c r="H17" s="22"/>
@@ -2511,20 +2510,20 @@
         <v>56</v>
       </c>
       <c r="C25" s="28">
-        <f t="shared" ref="C25:F25" si="5">C9*(C23+C24)</f>
-        <v>1615</v>
+        <f>C9*(C23+C24)</f>
+        <v>3400</v>
       </c>
       <c r="D25" s="28">
-        <f t="shared" si="5"/>
-        <v>2128</v>
+        <f t="shared" ref="C25:F25" si="5">D9*(D23+D24)</f>
+        <v>3920</v>
       </c>
       <c r="E25" s="28">
         <f t="shared" si="5"/>
-        <v>2656</v>
+        <v>4980</v>
       </c>
       <c r="F25" s="28">
         <f t="shared" si="5"/>
-        <v>800</v>
+        <v>1600</v>
       </c>
       <c r="G25" s="21"/>
       <c r="H25" s="22"/>
@@ -2538,20 +2537,20 @@
         <v>56</v>
       </c>
       <c r="C26" s="54">
-        <f>Staffing!D39</f>
-        <v>2936</v>
+        <f>0.15*C17</f>
+        <v>1553.5714285714282</v>
       </c>
       <c r="D26" s="54">
-        <f>Staffing!E39</f>
-        <v>2936</v>
+        <f>0.2*D17</f>
+        <v>2625</v>
       </c>
       <c r="E26" s="54">
-        <f>Staffing!F39</f>
-        <v>2621</v>
+        <f>0.2*E17</f>
+        <v>3696.4285714285711</v>
       </c>
       <c r="F26" s="54">
-        <f>Staffing!G39</f>
-        <v>2040</v>
+        <f t="shared" ref="D26:F26" si="6">0.15*F17</f>
+        <v>1607.1428571428571</v>
       </c>
       <c r="G26" s="21" t="s">
         <v>253</v>
@@ -2716,20 +2715,20 @@
         <v>56</v>
       </c>
       <c r="C32" s="28">
-        <f t="shared" ref="C32:F32" si="6">(C30+C31)*C17</f>
-        <v>78.714285714285694</v>
+        <f t="shared" ref="C32:F32" si="7">(C30+C31)*C17</f>
+        <v>165.71428571428569</v>
       </c>
       <c r="D32" s="28">
-        <f t="shared" si="6"/>
-        <v>470.24999999999994</v>
+        <f t="shared" si="7"/>
+        <v>866.24999999999989</v>
       </c>
       <c r="E32" s="28">
-        <f t="shared" si="6"/>
-        <v>1143.4285714285716</v>
+        <f t="shared" si="7"/>
+        <v>2143.9285714285711</v>
       </c>
       <c r="F32" s="28">
-        <f t="shared" si="6"/>
-        <v>803.57142857142856</v>
+        <f t="shared" si="7"/>
+        <v>1071.4285714285713</v>
       </c>
       <c r="G32" s="21"/>
       <c r="H32" s="22"/>
@@ -2743,13 +2742,13 @@
         <v>56</v>
       </c>
       <c r="C33" s="26">
-        <v>260</v>
+        <v>0</v>
       </c>
       <c r="D33" s="26">
-        <v>260</v>
+        <v>0</v>
       </c>
       <c r="E33" s="26">
-        <v>260</v>
+        <v>0</v>
       </c>
       <c r="F33" s="26">
         <v>0</v>
@@ -2772,20 +2771,20 @@
         <v>56</v>
       </c>
       <c r="C34" s="28">
-        <f t="shared" ref="C34:F34" si="7">C19+C22+C25+C26+C27+C28+C29+C32+C33</f>
-        <v>7839.7142857142853</v>
+        <f t="shared" ref="C34:F34" si="8">C19+C22+C25+C26+C27+C28+C29+C32+C33</f>
+        <v>8069.2857142857138</v>
       </c>
       <c r="D34" s="28">
-        <f t="shared" si="7"/>
-        <v>9844.25</v>
+        <f t="shared" si="8"/>
+        <v>11461.25</v>
       </c>
       <c r="E34" s="28">
-        <f t="shared" si="7"/>
-        <v>13480.428571428572</v>
+        <f t="shared" si="8"/>
+        <v>17620.357142857141</v>
       </c>
       <c r="F34" s="28">
-        <f t="shared" si="7"/>
-        <v>7893.5714285714284</v>
+        <f t="shared" si="8"/>
+        <v>8528.5714285714275</v>
       </c>
       <c r="G34" s="21"/>
       <c r="H34" s="22"/>
@@ -2812,20 +2811,20 @@
         <v>56</v>
       </c>
       <c r="C36" s="28">
-        <f t="shared" ref="C36:F36" si="8">C17-C34</f>
-        <v>-2920.0714285714294</v>
+        <f t="shared" ref="C36:F36" si="9">C17-C34</f>
+        <v>2287.8571428571413</v>
       </c>
       <c r="D36" s="28">
-        <f t="shared" si="8"/>
-        <v>-2719.2500000000009</v>
+        <f t="shared" si="9"/>
+        <v>1663.7499999999982</v>
       </c>
       <c r="E36" s="28">
-        <f t="shared" si="8"/>
-        <v>-3623.2857142857156</v>
+        <f t="shared" si="9"/>
+        <v>861.78571428571377</v>
       </c>
       <c r="F36" s="28">
-        <f t="shared" si="8"/>
-        <v>142.14285714285688</v>
+        <f t="shared" si="9"/>
+        <v>2185.7142857142862</v>
       </c>
       <c r="G36" s="21"/>
       <c r="H36" s="22"/>
@@ -2839,20 +2838,20 @@
         <v>64</v>
       </c>
       <c r="C37" s="31">
-        <f t="shared" ref="C37:F37" si="9">IF(C17&gt;0,C36/C17,0)</f>
-        <v>-0.59355353901996399</v>
+        <f t="shared" ref="C37:F37" si="10">IF(C17&gt;0,C36/C17,0)</f>
+        <v>0.22089655172413783</v>
       </c>
       <c r="D37" s="31">
-        <f t="shared" si="9"/>
-        <v>-0.38164912280701774</v>
+        <f t="shared" si="10"/>
+        <v>0.12676190476190463</v>
       </c>
       <c r="E37" s="31">
-        <f t="shared" si="9"/>
-        <v>-0.36757971014492768</v>
+        <f t="shared" si="10"/>
+        <v>4.6628019323671471E-2</v>
       </c>
       <c r="F37" s="31">
-        <f t="shared" si="9"/>
-        <v>1.7688888888888858E-2</v>
+        <f t="shared" si="10"/>
+        <v>0.20400000000000007</v>
       </c>
       <c r="G37" s="21"/>
       <c r="H37" s="22"/>
@@ -2866,20 +2865,20 @@
         <v>54</v>
       </c>
       <c r="C38" s="27">
-        <f t="shared" ref="C38:F38" si="10">IF(C9&gt;0,C36/C9,0)</f>
-        <v>-153.68796992481208</v>
+        <f t="shared" ref="C38:F38" si="11">IF(C9&gt;0,C36/C9,0)</f>
+        <v>57.196428571428534</v>
       </c>
       <c r="D38" s="27">
-        <f t="shared" si="10"/>
-        <v>-143.11842105263162</v>
+        <f t="shared" si="11"/>
+        <v>47.535714285714235</v>
       </c>
       <c r="E38" s="27">
-        <f t="shared" si="10"/>
-        <v>-226.45535714285722</v>
+        <f t="shared" si="11"/>
+        <v>28.72619047619046</v>
       </c>
       <c r="F38" s="27">
-        <f t="shared" si="10"/>
-        <v>14.214285714285689</v>
+        <f t="shared" si="11"/>
+        <v>109.28571428571431</v>
       </c>
       <c r="G38" s="21"/>
       <c r="H38" s="22"/>
@@ -2893,20 +2892,20 @@
         <v>64</v>
       </c>
       <c r="C39" s="31">
-        <f t="shared" ref="C39:F39" si="11">IF(C17&gt;0,C19/C17,0)</f>
-        <v>0.30490018148820336</v>
+        <f t="shared" ref="C39:F39" si="12">IF(C17&gt;0,C19/C17,0)</f>
+        <v>0.14482758620689659</v>
       </c>
       <c r="D39" s="31">
-        <f t="shared" si="11"/>
-        <v>0.2105263157894737</v>
+        <f t="shared" si="12"/>
+        <v>0.1142857142857143</v>
       </c>
       <c r="E39" s="31">
-        <f t="shared" si="11"/>
-        <v>0.25362318840579712</v>
+        <f t="shared" si="12"/>
+        <v>0.13526570048309181</v>
       </c>
       <c r="F39" s="31">
-        <f t="shared" si="11"/>
-        <v>0.24888888888888891</v>
+        <f t="shared" si="12"/>
+        <v>0.18666666666666668</v>
       </c>
       <c r="G39" s="21"/>
       <c r="H39" s="22"/>
@@ -2920,20 +2919,20 @@
         <v>64</v>
       </c>
       <c r="C40" s="31">
-        <f t="shared" ref="C40:F40" si="12">IF(C17&gt;0,C22/C17,0)</f>
-        <v>0.19310344827586212</v>
+        <f t="shared" ref="C40:F40" si="13">IF(C17&gt;0,C22/C17,0)</f>
+        <v>9.1724137931034497E-2</v>
       </c>
       <c r="D40" s="31">
-        <f t="shared" si="12"/>
-        <v>0.28070175438596495</v>
+        <f t="shared" si="13"/>
+        <v>0.15238095238095239</v>
       </c>
       <c r="E40" s="31">
-        <f t="shared" si="12"/>
-        <v>0.37536231884057975</v>
+        <f t="shared" si="13"/>
+        <v>0.20019323671497588</v>
       </c>
       <c r="F40" s="31">
-        <f t="shared" si="12"/>
-        <v>0.224</v>
+        <f t="shared" si="13"/>
+        <v>0.16800000000000001</v>
       </c>
       <c r="G40" s="21"/>
       <c r="H40" s="22"/>
@@ -2947,20 +2946,20 @@
         <v>64</v>
       </c>
       <c r="C41" s="31">
-        <f t="shared" ref="C41:F41" si="13">C37</f>
-        <v>-0.59355353901996399</v>
+        <f t="shared" ref="C41:F41" si="14">C37</f>
+        <v>0.22089655172413783</v>
       </c>
       <c r="D41" s="31">
-        <f t="shared" si="13"/>
-        <v>-0.38164912280701774</v>
+        <f t="shared" si="14"/>
+        <v>0.12676190476190463</v>
       </c>
       <c r="E41" s="31">
-        <f t="shared" si="13"/>
-        <v>-0.36757971014492768</v>
+        <f t="shared" si="14"/>
+        <v>4.6628019323671471E-2</v>
       </c>
       <c r="F41" s="31">
-        <f t="shared" si="13"/>
-        <v>1.7688888888888858E-2</v>
+        <f t="shared" si="14"/>
+        <v>0.20400000000000007</v>
       </c>
       <c r="G41" s="21"/>
       <c r="H41" s="22"/>
@@ -2974,20 +2973,20 @@
         <v>48</v>
       </c>
       <c r="C42" s="27">
-        <f t="shared" ref="C42:F42" si="14">IF(AND(C9&gt;0,1-C21-C30-C31&gt;0),((C19+C20+C26+C27+C28+C29+C33+C9*(C23+C24))/(1-C21-C30-C31)-C14-C16)/C9*(1+C12),0)</f>
-        <v>464.92939666238772</v>
+        <f t="shared" ref="C42:F42" si="15">IF(AND(C9&gt;0,1-C21-C30-C31&gt;0),((C19+C20+C26+C27+C28+C29+C33+C9*(C23+C24))/(1-C21-C30-C31)-C14-C16)/C9*(1+C12),0)</f>
+        <v>224.89837398373987</v>
       </c>
       <c r="D42" s="27">
-        <f t="shared" si="14"/>
-        <v>591.6195198918067</v>
+        <f t="shared" si="15"/>
+        <v>362.99785867237694</v>
       </c>
       <c r="E42" s="27">
-        <f t="shared" si="14"/>
-        <v>976.91176470588243</v>
+        <f t="shared" si="15"/>
+        <v>653.60482654600298</v>
       </c>
       <c r="F42" s="27">
-        <f t="shared" si="14"/>
-        <v>282.31111111111113</v>
+        <f t="shared" si="15"/>
+        <v>163.99999999999997</v>
       </c>
       <c r="G42" s="21"/>
       <c r="H42" s="22"/>
@@ -3001,20 +3000,20 @@
         <v>44</v>
       </c>
       <c r="C43" s="31">
-        <f t="shared" ref="C43:F43" si="15">IF(AND(C7&gt;0,C13*(1-C21-C30-C31)-(C23+C24)&gt;0),MAX(0,(C19+C20+C26+C27+C28+C29+C33-(C14+C16)*(1-C21-C30-C31))/(C13*(1-C21-C30-C31)-(C23+C24)))/C7,0)</f>
-        <v>1.5082737343991026</v>
+        <f t="shared" ref="C43:F43" si="16">IF(AND(C7&gt;0,C13*(1-C21-C30-C31)-(C23+C24)&gt;0),MAX(0,(C19+C20+C26+C27+C28+C29+C33-(C14+C16)*(1-C21-C30-C31))/(C13*(1-C21-C30-C31)-(C23+C24)))/C7,0)</f>
+        <v>0.66312578880942374</v>
       </c>
       <c r="D43" s="31">
-        <f t="shared" si="15"/>
-        <v>1.2672263029031132</v>
+        <f t="shared" si="16"/>
+        <v>0.80047968820266846</v>
       </c>
       <c r="E43" s="31">
-        <f t="shared" si="15"/>
-        <v>1.2785020281105555</v>
+        <f t="shared" si="16"/>
+        <v>0.92412665471810818</v>
       </c>
       <c r="F43" s="31">
-        <f t="shared" si="15"/>
-        <v>0.91175166297117516</v>
+        <f t="shared" si="16"/>
+        <v>0.32150776053215069</v>
       </c>
       <c r="G43" s="21"/>
       <c r="H43" s="22"/>
@@ -4324,7 +4323,7 @@
       </c>
       <c r="B13" s="17">
         <f>SUM(C13:N13)</f>
-        <v>121955.35714285714</v>
+        <v>200892.8571428571</v>
       </c>
       <c r="C13" s="34">
         <f>C7*'Prix et marges'!$C$17+C8*'Prix et marges'!$D$17+C9*'Prix et marges'!$E$17+C10*'Prix et marges'!$F$17</f>
@@ -4336,31 +4335,31 @@
       </c>
       <c r="E13" s="34">
         <f>E7*'Prix et marges'!$C$17+E8*'Prix et marges'!$D$17+E9*'Prix et marges'!$E$17+E10*'Prix et marges'!$F$17</f>
-        <v>4919.642857142856</v>
+        <v>10357.142857142855</v>
       </c>
       <c r="F13" s="34">
         <f>F7*'Prix et marges'!$C$17+F8*'Prix et marges'!$D$17+F9*'Prix et marges'!$E$17+F10*'Prix et marges'!$F$17</f>
-        <v>9857.1428571428569</v>
+        <v>18482.142857142855</v>
       </c>
       <c r="G13" s="34">
         <f>G7*'Prix et marges'!$C$17+G8*'Prix et marges'!$D$17+G9*'Prix et marges'!$E$17+G10*'Prix et marges'!$F$17</f>
-        <v>7124.9999999999991</v>
+        <v>13124.999999999998</v>
       </c>
       <c r="H13" s="34">
         <f>H7*'Prix et marges'!$C$17+H8*'Prix et marges'!$D$17+H9*'Prix et marges'!$E$17+H10*'Prix et marges'!$F$17</f>
-        <v>12955.357142857141</v>
+        <v>21071.428571428569</v>
       </c>
       <c r="I13" s="34">
         <f>I7*'Prix et marges'!$C$17+I8*'Prix et marges'!$D$17+I9*'Prix et marges'!$E$17+I10*'Prix et marges'!$F$17</f>
-        <v>17892.857142857141</v>
+        <v>29196.428571428569</v>
       </c>
       <c r="J13" s="34">
         <f>J7*'Prix et marges'!$C$17+J8*'Prix et marges'!$D$17+J9*'Prix et marges'!$E$17+J10*'Prix et marges'!$F$17</f>
-        <v>15160.714285714284</v>
+        <v>23839.28571428571</v>
       </c>
       <c r="K13" s="34">
         <f>K7*'Prix et marges'!$C$17+K8*'Prix et marges'!$D$17+K9*'Prix et marges'!$E$17+K10*'Prix et marges'!$F$17</f>
-        <v>4919.642857142856</v>
+        <v>10357.142857142855</v>
       </c>
       <c r="L13" s="34">
         <f>L7*'Prix et marges'!$C$17+L8*'Prix et marges'!$D$17+L9*'Prix et marges'!$E$17+L10*'Prix et marges'!$F$17</f>
@@ -4368,11 +4367,11 @@
       </c>
       <c r="M13" s="34">
         <f>M7*'Prix et marges'!$C$17+M8*'Prix et marges'!$D$17+M9*'Prix et marges'!$E$17+M10*'Prix et marges'!$F$17</f>
-        <v>25928.571428571428</v>
+        <v>39910.714285714283</v>
       </c>
       <c r="N13" s="34">
         <f>N7*'Prix et marges'!$C$17+N8*'Prix et marges'!$D$17+N9*'Prix et marges'!$E$17+N10*'Prix et marges'!$F$17</f>
-        <v>23196.428571428569</v>
+        <v>34553.571428571428</v>
       </c>
     </row>
     <row r="14" spans="1:16" ht="13" x14ac:dyDescent="0.3">
@@ -4381,7 +4380,7 @@
       </c>
       <c r="B14" s="17">
         <f>SUM(C14:N14)</f>
-        <v>149903.17857142858</v>
+        <v>172307.67857142858</v>
       </c>
       <c r="C14" s="34">
         <f>C7*'Prix et marges'!$C$34+C8*'Prix et marges'!$D$34+C9*'Prix et marges'!$E$34+C10*'Prix et marges'!$F$34+C40</f>
@@ -4393,31 +4392,31 @@
       </c>
       <c r="E14" s="34">
         <f>E7*'Prix et marges'!$C$34+E8*'Prix et marges'!$D$34+E9*'Prix et marges'!$E$34+E10*'Prix et marges'!$F$34+E40</f>
-        <v>8539.7142857142862</v>
+        <v>8769.2857142857138</v>
       </c>
       <c r="F14" s="34">
         <f>F7*'Prix et marges'!$C$34+F8*'Prix et marges'!$D$34+F9*'Prix et marges'!$E$34+F10*'Prix et marges'!$F$34+F40</f>
-        <v>13935.428571428572</v>
+        <v>18075.357142857141</v>
       </c>
       <c r="G14" s="34">
         <f>G7*'Prix et marges'!$C$34+G8*'Prix et marges'!$D$34+G9*'Prix et marges'!$E$34+G10*'Prix et marges'!$F$34+G40</f>
-        <v>9844.25</v>
+        <v>11461.25</v>
       </c>
       <c r="H14" s="34">
         <f>H7*'Prix et marges'!$C$34+H8*'Prix et marges'!$D$34+H9*'Prix et marges'!$E$34+H10*'Prix et marges'!$F$34+H40</f>
-        <v>15733.285714285714</v>
+        <v>16597.857142857141</v>
       </c>
       <c r="I14" s="34">
         <f>I7*'Prix et marges'!$C$34+I8*'Prix et marges'!$D$34+I9*'Prix et marges'!$E$34+I10*'Prix et marges'!$F$34+I40</f>
-        <v>21374</v>
+        <v>26148.928571428569</v>
       </c>
       <c r="J14" s="34">
         <f>J7*'Prix et marges'!$C$34+J8*'Prix et marges'!$D$34+J9*'Prix et marges'!$E$34+J10*'Prix et marges'!$F$34+J40</f>
-        <v>17737.821428571428</v>
+        <v>19989.821428571428</v>
       </c>
       <c r="K14" s="34">
         <f>K7*'Prix et marges'!$C$34+K8*'Prix et marges'!$D$34+K9*'Prix et marges'!$E$34+K10*'Prix et marges'!$F$34+K40</f>
-        <v>7839.7142857142853</v>
+        <v>8069.2857142857138</v>
       </c>
       <c r="L14" s="34">
         <f>L7*'Prix et marges'!$C$34+L8*'Prix et marges'!$D$34+L9*'Prix et marges'!$E$34+L10*'Prix et marges'!$F$34+L40</f>
@@ -4425,11 +4424,11 @@
       </c>
       <c r="M14" s="34">
         <f>M7*'Prix et marges'!$C$34+M8*'Prix et marges'!$D$34+M9*'Prix et marges'!$E$34+M10*'Prix et marges'!$F$34+M40</f>
-        <v>29267.571428571428</v>
+        <v>34677.5</v>
       </c>
       <c r="N14" s="34">
         <f>N7*'Prix et marges'!$C$34+N8*'Prix et marges'!$D$34+N9*'Prix et marges'!$E$34+N10*'Prix et marges'!$F$34+N40</f>
-        <v>25631.392857142855</v>
+        <v>28518.392857142855</v>
       </c>
     </row>
     <row r="15" spans="1:16" ht="13" x14ac:dyDescent="0.3">
@@ -4438,7 +4437,7 @@
       </c>
       <c r="B15" s="17">
         <f>SUM(C15:N15)</f>
-        <v>-27947.821428571438</v>
+        <v>28585.178571428558</v>
       </c>
       <c r="C15" s="17">
         <f t="shared" ref="C15:N15" si="2">C13-C14</f>
@@ -4450,31 +4449,31 @@
       </c>
       <c r="E15" s="17">
         <f t="shared" si="2"/>
-        <v>-3620.0714285714303</v>
+        <v>1587.8571428571413</v>
       </c>
       <c r="F15" s="17">
         <f t="shared" si="2"/>
-        <v>-4078.2857142857156</v>
+        <v>406.78571428571377</v>
       </c>
       <c r="G15" s="17">
         <f t="shared" si="2"/>
-        <v>-2719.2500000000009</v>
+        <v>1663.7499999999982</v>
       </c>
       <c r="H15" s="17">
         <f t="shared" si="2"/>
-        <v>-2777.9285714285725</v>
+        <v>4473.5714285714275</v>
       </c>
       <c r="I15" s="17">
         <f t="shared" si="2"/>
-        <v>-3481.1428571428587</v>
+        <v>3047.5</v>
       </c>
       <c r="J15" s="17">
         <f t="shared" si="2"/>
-        <v>-2577.1071428571431</v>
+        <v>3849.4642857142826</v>
       </c>
       <c r="K15" s="17">
         <f t="shared" si="2"/>
-        <v>-2920.0714285714294</v>
+        <v>2287.8571428571413</v>
       </c>
       <c r="L15" s="17">
         <f t="shared" si="2"/>
@@ -4482,11 +4481,11 @@
       </c>
       <c r="M15" s="17">
         <f t="shared" si="2"/>
-        <v>-3339</v>
+        <v>5233.2142857142826</v>
       </c>
       <c r="N15" s="17">
         <f t="shared" si="2"/>
-        <v>-2434.9642857142862</v>
+        <v>6035.1785714285725</v>
       </c>
     </row>
     <row r="16" spans="1:16" ht="13" x14ac:dyDescent="0.3">
@@ -5338,7 +5337,7 @@
       </c>
       <c r="B34" s="17">
         <f>SUM(C34:N34)</f>
-        <v>-40619.821428571435</v>
+        <v>15913.17857142856</v>
       </c>
       <c r="C34" s="17">
         <f t="shared" ref="C34:N34" si="7">C15-C32</f>
@@ -5350,31 +5349,31 @@
       </c>
       <c r="E34" s="17">
         <f t="shared" si="7"/>
-        <v>-5430.0714285714303</v>
+        <v>-222.1428571428587</v>
       </c>
       <c r="F34" s="17">
         <f t="shared" si="7"/>
-        <v>-5888.2857142857156</v>
+        <v>-1403.2142857142862</v>
       </c>
       <c r="G34" s="17">
         <f t="shared" si="7"/>
-        <v>-3329.2500000000009</v>
+        <v>1053.7499999999982</v>
       </c>
       <c r="H34" s="17">
         <f t="shared" si="7"/>
-        <v>-3387.9285714285725</v>
+        <v>3863.5714285714275</v>
       </c>
       <c r="I34" s="17">
         <f t="shared" si="7"/>
-        <v>-4091.1428571428587</v>
+        <v>2437.5</v>
       </c>
       <c r="J34" s="17">
         <f t="shared" si="7"/>
-        <v>-3187.1071428571431</v>
+        <v>3239.4642857142826</v>
       </c>
       <c r="K34" s="17">
         <f t="shared" si="7"/>
-        <v>-3530.0714285714294</v>
+        <v>1677.8571428571413</v>
       </c>
       <c r="L34" s="17">
         <f t="shared" si="7"/>
@@ -5382,11 +5381,11 @@
       </c>
       <c r="M34" s="17">
         <f t="shared" si="7"/>
-        <v>-3949</v>
+        <v>4623.2142857142826</v>
       </c>
       <c r="N34" s="17">
         <f t="shared" si="7"/>
-        <v>-3044.9642857142862</v>
+        <v>5425.1785714285725</v>
       </c>
     </row>
     <row r="35" spans="1:16" ht="13" x14ac:dyDescent="0.3">
@@ -5395,7 +5394,7 @@
       </c>
       <c r="B35" s="17">
         <f>N35</f>
-        <v>-40619.821428571435</v>
+        <v>15913.17857142856</v>
       </c>
       <c r="C35" s="17">
         <f>C34</f>
@@ -5407,43 +5406,43 @@
       </c>
       <c r="E35" s="17">
         <f t="shared" si="8"/>
-        <v>-9602.0714285714312</v>
+        <v>-4394.1428571428587</v>
       </c>
       <c r="F35" s="17">
         <f t="shared" si="8"/>
-        <v>-15490.357142857147</v>
+        <v>-5797.3571428571449</v>
       </c>
       <c r="G35" s="17">
         <f t="shared" si="8"/>
-        <v>-18819.607142857149</v>
+        <v>-4743.6071428571468</v>
       </c>
       <c r="H35" s="17">
         <f t="shared" si="8"/>
-        <v>-22207.535714285721</v>
+        <v>-880.03571428571922</v>
       </c>
       <c r="I35" s="17">
         <f t="shared" si="8"/>
-        <v>-26298.67857142858</v>
+        <v>1557.4642857142808</v>
       </c>
       <c r="J35" s="17">
         <f t="shared" si="8"/>
-        <v>-29485.785714285725</v>
+        <v>4796.9285714285634</v>
       </c>
       <c r="K35" s="17">
         <f t="shared" si="8"/>
-        <v>-33015.857142857152</v>
+        <v>6474.7857142857047</v>
       </c>
       <c r="L35" s="17">
         <f t="shared" si="8"/>
-        <v>-33625.857142857152</v>
+        <v>5864.7857142857047</v>
       </c>
       <c r="M35" s="17">
         <f t="shared" si="8"/>
-        <v>-37574.857142857152</v>
+        <v>10487.999999999987</v>
       </c>
       <c r="N35" s="17">
         <f t="shared" si="8"/>
-        <v>-40619.821428571435</v>
+        <v>15913.17857142856</v>
       </c>
     </row>
     <row r="37" spans="1:16" ht="13" x14ac:dyDescent="0.3">
@@ -5688,7 +5687,7 @@
       <c r="D5" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="E5" s="62" t="s">
+      <c r="E5" s="1" t="s">
         <v>296</v>
       </c>
     </row>
@@ -5702,7 +5701,7 @@
       <c r="D6" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="E6" s="62" t="s">
+      <c r="E6" s="1" t="s">
         <v>299</v>
       </c>
     </row>
@@ -5716,11 +5715,11 @@
       <c r="D7" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="E7" s="62" t="s">
+      <c r="E7" s="1" t="s">
         <v>302</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="39" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" ht="26" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>303</v>
       </c>
@@ -5750,7 +5749,7 @@
       <c r="D10" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="E10" s="62" t="s">
+      <c r="E10" s="1" t="s">
         <v>307</v>
       </c>
     </row>
@@ -5767,7 +5766,7 @@
       <c r="D11" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="E11" s="62" t="s">
+      <c r="E11" s="1" t="s">
         <v>309</v>
       </c>
     </row>
@@ -5784,7 +5783,7 @@
       <c r="D12" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="E12" s="62" t="s">
+      <c r="E12" s="1" t="s">
         <v>312</v>
       </c>
     </row>
@@ -5801,7 +5800,7 @@
       <c r="D13" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="E13" s="62" t="s">
+      <c r="E13" s="1" t="s">
         <v>315</v>
       </c>
     </row>
@@ -5818,7 +5817,7 @@
       <c r="D14" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="E14" s="62" t="s">
+      <c r="E14" s="1" t="s">
         <v>318</v>
       </c>
     </row>
@@ -5835,7 +5834,7 @@
       <c r="D15" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="E15" s="62" t="s">
+      <c r="E15" s="1" t="s">
         <v>89</v>
       </c>
     </row>
@@ -5852,7 +5851,7 @@
       <c r="D16" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="E16" s="62" t="s">
+      <c r="E16" s="1" t="s">
         <v>320</v>
       </c>
     </row>
@@ -5869,7 +5868,7 @@
       <c r="D17" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="E17" s="62" t="s">
+      <c r="E17" s="1" t="s">
         <v>89</v>
       </c>
     </row>
@@ -5886,7 +5885,7 @@
       <c r="D18" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="E18" s="62" t="s">
+      <c r="E18" s="1" t="s">
         <v>323</v>
       </c>
     </row>
@@ -5903,7 +5902,7 @@
       <c r="D19" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="E19" s="62" t="s">
+      <c r="E19" s="1" t="s">
         <v>89</v>
       </c>
     </row>
@@ -5920,7 +5919,7 @@
       <c r="D20" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="E20" s="62" t="s">
+      <c r="E20" s="1" t="s">
         <v>327</v>
       </c>
     </row>
@@ -5948,19 +5947,19 @@
       </c>
       <c r="C23" s="16">
         <f>'Prix et marges'!C17</f>
-        <v>4919.642857142856</v>
+        <v>10357.142857142855</v>
       </c>
       <c r="D23" s="16">
         <f>'Prix et marges'!D17</f>
-        <v>7124.9999999999991</v>
+        <v>13124.999999999998</v>
       </c>
       <c r="E23" s="16">
         <f>'Prix et marges'!E17</f>
-        <v>9857.1428571428569</v>
+        <v>18482.142857142855</v>
       </c>
       <c r="F23" s="16">
         <f>'Prix et marges'!F17</f>
-        <v>8035.7142857142853</v>
+        <v>10714.285714285714</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
@@ -5990,19 +5989,19 @@
       </c>
       <c r="C25" s="16">
         <f>C23*C24</f>
-        <v>590.35714285714266</v>
+        <v>1242.8571428571427</v>
       </c>
       <c r="D25" s="16">
         <f>D23*D24</f>
-        <v>854.99999999999989</v>
+        <v>1574.9999999999998</v>
       </c>
       <c r="E25" s="16">
         <f>E23*E24</f>
-        <v>1182.8571428571429</v>
+        <v>2217.8571428571427</v>
       </c>
       <c r="F25" s="16">
         <f>F23*F24</f>
-        <v>964.28571428571422</v>
+        <v>1285.7142857142856</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
@@ -6011,19 +6010,19 @@
       </c>
       <c r="C26" s="16">
         <f>'Prix et marges'!C19*$C$10+'Prix et marges'!C22*$C$11+'Prix et marges'!C9*'Prix et marges'!C23*$C$12+'Prix et marges'!C9*'Prix et marges'!C24*$C$13+'Prix et marges'!C26*$C$14+'Prix et marges'!C27*$C$15+'Prix et marges'!C28*$C$16+'Prix et marges'!C29*$C$17+'Prix et marges'!C30*'Prix et marges'!C17*$C$18+'Prix et marges'!C31*'Prix et marges'!C17*$C$19+'Prix et marges'!C33*$C$20</f>
-        <v>1180.6750000000002</v>
+        <v>1041.7142857142858</v>
       </c>
       <c r="D26" s="16">
         <f>'Prix et marges'!D19*$C$10+'Prix et marges'!D22*$C$11+'Prix et marges'!D9*'Prix et marges'!D23*$C$12+'Prix et marges'!D9*'Prix et marges'!D24*$C$13+'Prix et marges'!D26*$C$14+'Prix et marges'!D27*$C$15+'Prix et marges'!D28*$C$16+'Prix et marges'!D29*$C$17+'Prix et marges'!D30*'Prix et marges'!D17*$C$18+'Prix et marges'!D31*'Prix et marges'!D17*$C$19+'Prix et marges'!D33*$C$20</f>
-        <v>1323.2</v>
+        <v>1465</v>
       </c>
       <c r="E26" s="16">
         <f>'Prix et marges'!E19*$C$10+'Prix et marges'!E22*$C$11+'Prix et marges'!E9*'Prix et marges'!E23*$C$12+'Prix et marges'!E9*'Prix et marges'!E24*$C$13+'Prix et marges'!E26*$C$14+'Prix et marges'!E27*$C$15+'Prix et marges'!E28*$C$16+'Prix et marges'!E29*$C$17+'Prix et marges'!E30*'Prix et marges'!E17*$C$18+'Prix et marges'!E31*'Prix et marges'!E17*$C$19+'Prix et marges'!E33*$C$20</f>
-        <v>1662.5428571428572</v>
+        <v>2259.9285714285716</v>
       </c>
       <c r="F26" s="16">
         <f>'Prix et marges'!F19*$C$10+'Prix et marges'!F22*$C$11+'Prix et marges'!F9*'Prix et marges'!F23*$C$12+'Prix et marges'!F9*'Prix et marges'!F24*$C$13+'Prix et marges'!F26*$C$14+'Prix et marges'!F27*$C$15+'Prix et marges'!F28*$C$16+'Prix et marges'!F29*$C$17+'Prix et marges'!F30*'Prix et marges'!F17*$C$18+'Prix et marges'!F31*'Prix et marges'!F17*$C$19+'Prix et marges'!F33*$C$20</f>
-        <v>1116.2142857142858</v>
+        <v>1170.7142857142858</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
@@ -6032,22 +6031,22 @@
       </c>
       <c r="C27" s="16">
         <f>C25-C26</f>
-        <v>-590.31785714285752</v>
+        <v>201.14285714285688</v>
       </c>
       <c r="D27" s="16">
         <f>D25-D26</f>
-        <v>-468.20000000000016</v>
+        <v>109.99999999999977</v>
       </c>
       <c r="E27" s="16">
         <f>E25-E26</f>
-        <v>-479.68571428571431</v>
+        <v>-42.071428571428896</v>
       </c>
       <c r="F27" s="16">
         <f>F25-F26</f>
-        <v>-151.92857142857156</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" ht="65" x14ac:dyDescent="0.25">
+        <v>114.99999999999977</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="26" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
         <v>335</v>
       </c>
@@ -6077,7 +6076,7 @@
       <c r="D30" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="E30" s="62" t="s">
+      <c r="E30" s="1" t="s">
         <v>89</v>
       </c>
     </row>
@@ -6094,7 +6093,7 @@
       <c r="D31" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="E31" s="62" t="s">
+      <c r="E31" s="1" t="s">
         <v>89</v>
       </c>
     </row>
@@ -6111,7 +6110,7 @@
       <c r="D32" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="E32" s="62" t="s">
+      <c r="E32" s="1" t="s">
         <v>339</v>
       </c>
     </row>
@@ -6128,7 +6127,7 @@
       <c r="D33" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="E33" s="62" t="s">
+      <c r="E33" s="1" t="s">
         <v>341</v>
       </c>
     </row>
@@ -6145,7 +6144,7 @@
       <c r="D34" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="E34" s="62" t="s">
+      <c r="E34" s="1" t="s">
         <v>89</v>
       </c>
     </row>
@@ -6162,7 +6161,7 @@
       <c r="D35" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="E35" s="62" t="s">
+      <c r="E35" s="1" t="s">
         <v>343</v>
       </c>
     </row>
@@ -6179,7 +6178,7 @@
       <c r="D36" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="E36" s="62" t="s">
+      <c r="E36" s="1" t="s">
         <v>344</v>
       </c>
     </row>
@@ -6196,7 +6195,7 @@
       <c r="D37" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="E37" s="62" t="s">
+      <c r="E37" s="1" t="s">
         <v>345</v>
       </c>
     </row>
@@ -6213,7 +6212,7 @@
       <c r="D38" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="E38" s="62" t="s">
+      <c r="E38" s="1" t="s">
         <v>89</v>
       </c>
     </row>
@@ -6222,7 +6221,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="41" spans="1:14" ht="26" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:14" ht="13" x14ac:dyDescent="0.3">
       <c r="A41" s="6" t="s">
         <v>31</v>
       </c>
@@ -6284,7 +6283,7 @@
       </c>
       <c r="B42" s="16">
         <f>SUM(C42:N42)</f>
-        <v>14634.642857142855</v>
+        <v>24107.142857142855</v>
       </c>
       <c r="C42" s="16">
         <f>'Budget mensuel'!C7*$C$25+'Budget mensuel'!C8*$D$25+'Budget mensuel'!C9*$E$25+'Budget mensuel'!C10*$F$25</f>
@@ -6296,31 +6295,31 @@
       </c>
       <c r="E42" s="16">
         <f>'Budget mensuel'!E7*$C$25+'Budget mensuel'!E8*$D$25+'Budget mensuel'!E9*$E$25+'Budget mensuel'!E10*$F$25</f>
-        <v>590.35714285714266</v>
+        <v>1242.8571428571427</v>
       </c>
       <c r="F42" s="16">
         <f>'Budget mensuel'!F7*$C$25+'Budget mensuel'!F8*$D$25+'Budget mensuel'!F9*$E$25+'Budget mensuel'!F10*$F$25</f>
-        <v>1182.8571428571429</v>
+        <v>2217.8571428571427</v>
       </c>
       <c r="G42" s="16">
         <f>'Budget mensuel'!G7*$C$25+'Budget mensuel'!G8*$D$25+'Budget mensuel'!G9*$E$25+'Budget mensuel'!G10*$F$25</f>
-        <v>854.99999999999989</v>
+        <v>1574.9999999999998</v>
       </c>
       <c r="H42" s="16">
         <f>'Budget mensuel'!H7*$C$25+'Budget mensuel'!H8*$D$25+'Budget mensuel'!H9*$E$25+'Budget mensuel'!H10*$F$25</f>
-        <v>1554.6428571428569</v>
+        <v>2528.5714285714284</v>
       </c>
       <c r="I42" s="16">
         <f>'Budget mensuel'!I7*$C$25+'Budget mensuel'!I8*$D$25+'Budget mensuel'!I9*$E$25+'Budget mensuel'!I10*$F$25</f>
-        <v>2147.1428571428569</v>
+        <v>3503.5714285714284</v>
       </c>
       <c r="J42" s="16">
         <f>'Budget mensuel'!J7*$C$25+'Budget mensuel'!J8*$D$25+'Budget mensuel'!J9*$E$25+'Budget mensuel'!J10*$F$25</f>
-        <v>1819.2857142857142</v>
+        <v>2860.7142857142853</v>
       </c>
       <c r="K42" s="16">
         <f>'Budget mensuel'!K7*$C$25+'Budget mensuel'!K8*$D$25+'Budget mensuel'!K9*$E$25+'Budget mensuel'!K10*$F$25</f>
-        <v>590.35714285714266</v>
+        <v>1242.8571428571427</v>
       </c>
       <c r="L42" s="16">
         <f>'Budget mensuel'!L7*$C$25+'Budget mensuel'!L8*$D$25+'Budget mensuel'!L9*$E$25+'Budget mensuel'!L10*$F$25</f>
@@ -6328,11 +6327,11 @@
       </c>
       <c r="M42" s="16">
         <f>'Budget mensuel'!M7*$C$25+'Budget mensuel'!M8*$D$25+'Budget mensuel'!M9*$E$25+'Budget mensuel'!M10*$F$25</f>
-        <v>3111.4285714285716</v>
+        <v>4789.2857142857138</v>
       </c>
       <c r="N42" s="16">
         <f>'Budget mensuel'!N7*$C$25+'Budget mensuel'!N8*$D$25+'Budget mensuel'!N9*$E$25+'Budget mensuel'!N10*$F$25</f>
-        <v>2783.5714285714284</v>
+        <v>4146.4285714285706</v>
       </c>
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.25">
@@ -6341,7 +6340,7 @@
       </c>
       <c r="B43" s="16">
         <f>SUM(C43:N43)</f>
-        <v>20543.75357142857</v>
+        <v>22725.928571428572</v>
       </c>
       <c r="C43" s="16">
         <f>'Budget mensuel'!C7*$C$26+'Budget mensuel'!C8*$D$26+'Budget mensuel'!C9*$E$26+'Budget mensuel'!C10*$F$26+'Budget mensuel'!C40*$C$14</f>
@@ -6353,31 +6352,31 @@
       </c>
       <c r="E43" s="16">
         <f>'Budget mensuel'!E7*$C$26+'Budget mensuel'!E8*$D$26+'Budget mensuel'!E9*$E$26+'Budget mensuel'!E10*$F$26+'Budget mensuel'!E40*$C$14</f>
-        <v>1320.6750000000002</v>
+        <v>1181.7142857142858</v>
       </c>
       <c r="F43" s="16">
         <f>'Budget mensuel'!F7*$C$26+'Budget mensuel'!F8*$D$26+'Budget mensuel'!F9*$E$26+'Budget mensuel'!F10*$F$26+'Budget mensuel'!F40*$C$14</f>
-        <v>1753.5428571428572</v>
+        <v>2350.9285714285716</v>
       </c>
       <c r="G43" s="16">
         <f>'Budget mensuel'!G7*$C$26+'Budget mensuel'!G8*$D$26+'Budget mensuel'!G9*$E$26+'Budget mensuel'!G10*$F$26+'Budget mensuel'!G40*$C$14</f>
-        <v>1323.2</v>
+        <v>1465</v>
       </c>
       <c r="H43" s="16">
         <f>'Budget mensuel'!H7*$C$26+'Budget mensuel'!H8*$D$26+'Budget mensuel'!H9*$E$26+'Budget mensuel'!H10*$F$26+'Budget mensuel'!H40*$C$14</f>
-        <v>2296.889285714286</v>
+        <v>2212.4285714285716</v>
       </c>
       <c r="I43" s="16">
         <f>'Budget mensuel'!I7*$C$26+'Budget mensuel'!I8*$D$26+'Budget mensuel'!I9*$E$26+'Budget mensuel'!I10*$F$26+'Budget mensuel'!I40*$C$14</f>
-        <v>2778.7571428571428</v>
+        <v>3430.6428571428573</v>
       </c>
       <c r="J43" s="16">
         <f>'Budget mensuel'!J7*$C$26+'Budget mensuel'!J8*$D$26+'Budget mensuel'!J9*$E$26+'Budget mensuel'!J10*$F$26+'Budget mensuel'!J40*$C$14</f>
-        <v>2439.4142857142861</v>
+        <v>2635.7142857142858</v>
       </c>
       <c r="K43" s="16">
         <f>'Budget mensuel'!K7*$C$26+'Budget mensuel'!K8*$D$26+'Budget mensuel'!K9*$E$26+'Budget mensuel'!K10*$F$26+'Budget mensuel'!K40*$C$14</f>
-        <v>1180.6750000000002</v>
+        <v>1041.7142857142858</v>
       </c>
       <c r="L43" s="16">
         <f>'Budget mensuel'!L7*$C$26+'Budget mensuel'!L8*$D$26+'Budget mensuel'!L9*$E$26+'Budget mensuel'!L10*$F$26+'Budget mensuel'!L40*$C$14</f>
@@ -6385,11 +6384,11 @@
       </c>
       <c r="M43" s="16">
         <f>'Budget mensuel'!M7*$C$26+'Budget mensuel'!M8*$D$26+'Budget mensuel'!M9*$E$26+'Budget mensuel'!M10*$F$26+'Budget mensuel'!M40*$C$14</f>
-        <v>3894.971428571429</v>
+        <v>4601.3571428571431</v>
       </c>
       <c r="N43" s="16">
         <f>'Budget mensuel'!N7*$C$26+'Budget mensuel'!N8*$D$26+'Budget mensuel'!N9*$E$26+'Budget mensuel'!N10*$F$26+'Budget mensuel'!N40*$C$14</f>
-        <v>3555.6285714285714</v>
+        <v>3806.4285714285716</v>
       </c>
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.25">
@@ -6501,55 +6500,55 @@
       </c>
       <c r="B46" s="17">
         <f>SUM(C46:N46)</f>
-        <v>-8741.1107142857163</v>
+        <v>-1450.7857142857183</v>
       </c>
       <c r="C46" s="17">
-        <f>C42-C43-C44-C45</f>
+        <f t="shared" ref="C46:N46" si="0">C42-C43-C44-C45</f>
         <v>-1001</v>
       </c>
       <c r="D46" s="17">
-        <f>D42-D43-D44-D45</f>
+        <f t="shared" si="0"/>
         <v>-341</v>
       </c>
       <c r="E46" s="17">
-        <f>E42-E43-E44-E45</f>
-        <v>-1071.3178571428575</v>
+        <f t="shared" si="0"/>
+        <v>-279.85714285714312</v>
       </c>
       <c r="F46" s="17">
-        <f>F42-F43-F44-F45</f>
-        <v>-911.68571428571431</v>
+        <f t="shared" si="0"/>
+        <v>-474.0714285714289</v>
       </c>
       <c r="G46" s="17">
-        <f>G42-G43-G44-G45</f>
-        <v>-569.20000000000016</v>
+        <f t="shared" si="0"/>
+        <v>8.9999999999997726</v>
       </c>
       <c r="H46" s="17">
-        <f>H42-H43-H44-H45</f>
-        <v>-843.24642857142908</v>
+        <f t="shared" si="0"/>
+        <v>215.14285714285688</v>
       </c>
       <c r="I46" s="17">
-        <f>I42-I43-I44-I45</f>
-        <v>-732.61428571428587</v>
+        <f t="shared" si="0"/>
+        <v>-28.071428571428896</v>
       </c>
       <c r="J46" s="17">
-        <f>J42-J43-J44-J45</f>
-        <v>-721.12857142857183</v>
+        <f t="shared" si="0"/>
+        <v>123.99999999999955</v>
       </c>
       <c r="K46" s="17">
-        <f>K42-K43-K44-K45</f>
-        <v>-691.31785714285752</v>
+        <f t="shared" si="0"/>
+        <v>100.14285714285688</v>
       </c>
       <c r="L46" s="17">
-        <f>L42-L43-L44-L45</f>
+        <f t="shared" si="0"/>
         <v>-101</v>
       </c>
       <c r="M46" s="17">
-        <f>M42-M43-M44-M45</f>
-        <v>-884.54285714285743</v>
+        <f t="shared" si="0"/>
+        <v>86.928571428570649</v>
       </c>
       <c r="N46" s="17">
-        <f>N42-N43-N44-N45</f>
-        <v>-873.05714285714294</v>
+        <f t="shared" si="0"/>
+        <v>238.99999999999909</v>
       </c>
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.25">
@@ -6564,48 +6563,48 @@
         <v>0</v>
       </c>
       <c r="D47" s="16">
-        <f>C49</f>
+        <f t="shared" ref="D47:N47" si="1">C49</f>
         <v>1001</v>
       </c>
       <c r="E47" s="16">
-        <f>D49</f>
+        <f t="shared" si="1"/>
         <v>1342</v>
       </c>
       <c r="F47" s="16">
-        <f>E49</f>
-        <v>2413.3178571428575</v>
+        <f t="shared" si="1"/>
+        <v>1621.8571428571431</v>
       </c>
       <c r="G47" s="16">
-        <f>F49</f>
-        <v>3325.0035714285718</v>
+        <f t="shared" si="1"/>
+        <v>2095.928571428572</v>
       </c>
       <c r="H47" s="16">
-        <f>G49</f>
-        <v>3894.2035714285721</v>
+        <f t="shared" si="1"/>
+        <v>2086.9285714285725</v>
       </c>
       <c r="I47" s="16">
-        <f>H49</f>
-        <v>4737.4500000000007</v>
+        <f t="shared" si="1"/>
+        <v>1871.7857142857156</v>
       </c>
       <c r="J47" s="16">
-        <f>I49</f>
-        <v>5470.0642857142866</v>
+        <f t="shared" si="1"/>
+        <v>1899.8571428571445</v>
       </c>
       <c r="K47" s="16">
-        <f>J49</f>
-        <v>6191.192857142858</v>
+        <f t="shared" si="1"/>
+        <v>1775.8571428571449</v>
       </c>
       <c r="L47" s="16">
-        <f>K49</f>
-        <v>6882.5107142857159</v>
+        <f t="shared" si="1"/>
+        <v>1675.7142857142881</v>
       </c>
       <c r="M47" s="16">
-        <f>L49</f>
-        <v>6983.5107142857159</v>
+        <f t="shared" si="1"/>
+        <v>1776.7142857142881</v>
       </c>
       <c r="N47" s="16">
-        <f>M49</f>
-        <v>7868.0535714285734</v>
+        <f t="shared" si="1"/>
+        <v>1689.7857142857174</v>
       </c>
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.25">
@@ -6617,51 +6616,51 @@
         <v>0</v>
       </c>
       <c r="C48" s="16">
-        <f>MAX(0,C46-C47)</f>
+        <f t="shared" ref="C48:N48" si="2">MAX(0,C46-C47)</f>
         <v>0</v>
       </c>
       <c r="D48" s="16">
-        <f>MAX(0,D46-D47)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="E48" s="16">
-        <f>MAX(0,E46-E47)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="F48" s="16">
-        <f>MAX(0,F46-F47)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="G48" s="16">
-        <f>MAX(0,G46-G47)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="H48" s="16">
-        <f>MAX(0,H46-H47)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="I48" s="16">
-        <f>MAX(0,I46-I47)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="J48" s="16">
-        <f>MAX(0,J46-J47)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="K48" s="16">
-        <f>MAX(0,K46-K47)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="L48" s="16">
-        <f>MAX(0,L46-L47)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="M48" s="16">
-        <f>MAX(0,M46-M47)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="N48" s="16">
-        <f>MAX(0,N46-N47)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -6671,55 +6670,55 @@
       </c>
       <c r="B49" s="16">
         <f>N49</f>
-        <v>8741.1107142857163</v>
+        <v>1450.7857142857183</v>
       </c>
       <c r="C49" s="16">
-        <f>MAX(0,C47-C46)</f>
+        <f t="shared" ref="C49:N49" si="3">MAX(0,C47-C46)</f>
         <v>1001</v>
       </c>
       <c r="D49" s="16">
-        <f>MAX(0,D47-D46)</f>
+        <f t="shared" si="3"/>
         <v>1342</v>
       </c>
       <c r="E49" s="16">
-        <f>MAX(0,E47-E46)</f>
-        <v>2413.3178571428575</v>
+        <f t="shared" si="3"/>
+        <v>1621.8571428571431</v>
       </c>
       <c r="F49" s="16">
-        <f>MAX(0,F47-F46)</f>
-        <v>3325.0035714285718</v>
+        <f t="shared" si="3"/>
+        <v>2095.928571428572</v>
       </c>
       <c r="G49" s="16">
-        <f>MAX(0,G47-G46)</f>
-        <v>3894.2035714285721</v>
+        <f t="shared" si="3"/>
+        <v>2086.9285714285725</v>
       </c>
       <c r="H49" s="16">
-        <f>MAX(0,H47-H46)</f>
-        <v>4737.4500000000007</v>
+        <f t="shared" si="3"/>
+        <v>1871.7857142857156</v>
       </c>
       <c r="I49" s="16">
-        <f>MAX(0,I47-I46)</f>
-        <v>5470.0642857142866</v>
+        <f t="shared" si="3"/>
+        <v>1899.8571428571445</v>
       </c>
       <c r="J49" s="16">
-        <f>MAX(0,J47-J46)</f>
-        <v>6191.192857142858</v>
+        <f t="shared" si="3"/>
+        <v>1775.8571428571449</v>
       </c>
       <c r="K49" s="16">
-        <f>MAX(0,K47-K46)</f>
-        <v>6882.5107142857159</v>
+        <f t="shared" si="3"/>
+        <v>1675.7142857142881</v>
       </c>
       <c r="L49" s="16">
-        <f>MAX(0,L47-L46)</f>
-        <v>6983.5107142857159</v>
+        <f t="shared" si="3"/>
+        <v>1776.7142857142881</v>
       </c>
       <c r="M49" s="16">
-        <f>MAX(0,M47-M46)</f>
-        <v>7868.0535714285734</v>
+        <f t="shared" si="3"/>
+        <v>1689.7857142857174</v>
       </c>
       <c r="N49" s="16">
-        <f>MAX(0,N47-N46)</f>
-        <v>8741.1107142857163</v>
+        <f t="shared" si="3"/>
+        <v>1450.7857142857183</v>
       </c>
     </row>
     <row r="50" spans="1:14" x14ac:dyDescent="0.25">
@@ -6734,47 +6733,47 @@
         <v>0</v>
       </c>
       <c r="D50" s="16">
-        <f>C48</f>
+        <f t="shared" ref="D50:N50" si="4">C48</f>
         <v>0</v>
       </c>
       <c r="E50" s="16">
-        <f>D48</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="F50" s="16">
-        <f>E48</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="G50" s="16">
-        <f>F48</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="H50" s="16">
-        <f>G48</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="I50" s="16">
-        <f>H48</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="J50" s="16">
-        <f>I48</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="K50" s="16">
-        <f>J48</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="L50" s="16">
-        <f>K48</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="M50" s="16">
-        <f>L48</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="N50" s="16">
-        <f>M48</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -6784,55 +6783,55 @@
       </c>
       <c r="B51" s="46">
         <f>SUM(C51:N51)</f>
-        <v>-8741.1107142857163</v>
+        <v>-1450.7857142857183</v>
       </c>
       <c r="C51" s="46">
-        <f>C42-C43-C44-C45-C50</f>
+        <f t="shared" ref="C51:N51" si="5">C42-C43-C44-C45-C50</f>
         <v>-1001</v>
       </c>
       <c r="D51" s="46">
-        <f>D42-D43-D44-D45-D50</f>
+        <f t="shared" si="5"/>
         <v>-341</v>
       </c>
       <c r="E51" s="46">
-        <f>E42-E43-E44-E45-E50</f>
-        <v>-1071.3178571428575</v>
+        <f t="shared" si="5"/>
+        <v>-279.85714285714312</v>
       </c>
       <c r="F51" s="46">
-        <f>F42-F43-F44-F45-F50</f>
-        <v>-911.68571428571431</v>
+        <f t="shared" si="5"/>
+        <v>-474.0714285714289</v>
       </c>
       <c r="G51" s="46">
-        <f>G42-G43-G44-G45-G50</f>
-        <v>-569.20000000000016</v>
+        <f t="shared" si="5"/>
+        <v>8.9999999999997726</v>
       </c>
       <c r="H51" s="46">
-        <f>H42-H43-H44-H45-H50</f>
-        <v>-843.24642857142908</v>
+        <f t="shared" si="5"/>
+        <v>215.14285714285688</v>
       </c>
       <c r="I51" s="46">
-        <f>I42-I43-I44-I45-I50</f>
-        <v>-732.61428571428587</v>
+        <f t="shared" si="5"/>
+        <v>-28.071428571428896</v>
       </c>
       <c r="J51" s="46">
-        <f>J42-J43-J44-J45-J50</f>
-        <v>-721.12857142857183</v>
+        <f t="shared" si="5"/>
+        <v>123.99999999999955</v>
       </c>
       <c r="K51" s="46">
-        <f>K42-K43-K44-K45-K50</f>
-        <v>-691.31785714285752</v>
+        <f t="shared" si="5"/>
+        <v>100.14285714285688</v>
       </c>
       <c r="L51" s="46">
-        <f>L42-L43-L44-L45-L50</f>
+        <f t="shared" si="5"/>
         <v>-101</v>
       </c>
       <c r="M51" s="46">
-        <f>M42-M43-M44-M45-M50</f>
-        <v>-884.54285714285743</v>
+        <f t="shared" si="5"/>
+        <v>86.928571428570649</v>
       </c>
       <c r="N51" s="46">
-        <f>N42-N43-N44-N45-N50</f>
-        <v>-873.05714285714294</v>
+        <f t="shared" si="5"/>
+        <v>238.99999999999909</v>
       </c>
     </row>
     <row r="53" spans="1:14" ht="13" x14ac:dyDescent="0.3">
@@ -7104,7 +7103,7 @@
       </c>
       <c r="B12" s="16">
         <f>SUM(C12:N12)</f>
-        <v>121955.35714285714</v>
+        <v>200892.8571428571</v>
       </c>
       <c r="C12" s="36">
         <f>'Budget mensuel'!C13</f>
@@ -7116,31 +7115,31 @@
       </c>
       <c r="E12" s="36">
         <f>'Budget mensuel'!E13</f>
-        <v>4919.642857142856</v>
+        <v>10357.142857142855</v>
       </c>
       <c r="F12" s="36">
         <f>'Budget mensuel'!F13</f>
-        <v>9857.1428571428569</v>
+        <v>18482.142857142855</v>
       </c>
       <c r="G12" s="36">
         <f>'Budget mensuel'!G13</f>
-        <v>7124.9999999999991</v>
+        <v>13124.999999999998</v>
       </c>
       <c r="H12" s="36">
         <f>'Budget mensuel'!H13</f>
-        <v>12955.357142857141</v>
+        <v>21071.428571428569</v>
       </c>
       <c r="I12" s="36">
         <f>'Budget mensuel'!I13</f>
-        <v>17892.857142857141</v>
+        <v>29196.428571428569</v>
       </c>
       <c r="J12" s="36">
         <f>'Budget mensuel'!J13</f>
-        <v>15160.714285714284</v>
+        <v>23839.28571428571</v>
       </c>
       <c r="K12" s="36">
         <f>'Budget mensuel'!K13</f>
-        <v>4919.642857142856</v>
+        <v>10357.142857142855</v>
       </c>
       <c r="L12" s="36">
         <f>'Budget mensuel'!L13</f>
@@ -7148,11 +7147,11 @@
       </c>
       <c r="M12" s="36">
         <f>'Budget mensuel'!M13</f>
-        <v>25928.571428571428</v>
+        <v>39910.714285714283</v>
       </c>
       <c r="N12" s="36">
         <f>'Budget mensuel'!N13</f>
-        <v>23196.428571428569</v>
+        <v>34553.571428571428</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
@@ -7410,7 +7409,7 @@
       </c>
       <c r="B22" s="16">
         <f>SUM(C22:N22)</f>
-        <v>-40619.821428571435</v>
+        <v>15913.17857142856</v>
       </c>
       <c r="C22" s="36">
         <f>'Budget mensuel'!C34</f>
@@ -7422,31 +7421,31 @@
       </c>
       <c r="E22" s="36">
         <f>'Budget mensuel'!E34</f>
-        <v>-5430.0714285714303</v>
+        <v>-222.1428571428587</v>
       </c>
       <c r="F22" s="36">
         <f>'Budget mensuel'!F34</f>
-        <v>-5888.2857142857156</v>
+        <v>-1403.2142857142862</v>
       </c>
       <c r="G22" s="36">
         <f>'Budget mensuel'!G34</f>
-        <v>-3329.2500000000009</v>
+        <v>1053.7499999999982</v>
       </c>
       <c r="H22" s="36">
         <f>'Budget mensuel'!H34</f>
-        <v>-3387.9285714285725</v>
+        <v>3863.5714285714275</v>
       </c>
       <c r="I22" s="36">
         <f>'Budget mensuel'!I34</f>
-        <v>-4091.1428571428587</v>
+        <v>2437.5</v>
       </c>
       <c r="J22" s="36">
         <f>'Budget mensuel'!J34</f>
-        <v>-3187.1071428571431</v>
+        <v>3239.4642857142826</v>
       </c>
       <c r="K22" s="36">
         <f>'Budget mensuel'!K34</f>
-        <v>-3530.0714285714294</v>
+        <v>1677.8571428571413</v>
       </c>
       <c r="L22" s="36">
         <f>'Budget mensuel'!L34</f>
@@ -7454,11 +7453,11 @@
       </c>
       <c r="M22" s="36">
         <f>'Budget mensuel'!M34</f>
-        <v>-3949</v>
+        <v>4623.2142857142826</v>
       </c>
       <c r="N22" s="36">
         <f>'Budget mensuel'!N34</f>
-        <v>-3044.9642857142862</v>
+        <v>5425.1785714285725</v>
       </c>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.25">
@@ -7774,15 +7773,15 @@
       </c>
       <c r="C13" s="38">
         <f>C7*'Prix et marges'!$C$17+C8*'Prix et marges'!$D$17+C9*'Prix et marges'!$E$17+C10*'Prix et marges'!$F$17</f>
-        <v>121955.35714285713</v>
+        <v>200892.8571428571</v>
       </c>
       <c r="D13" s="38">
         <f>D7*'Prix et marges'!$C$17+D8*'Prix et marges'!$D$17+D9*'Prix et marges'!$E$17+D10*'Prix et marges'!$F$17</f>
-        <v>368071.42857142852</v>
+        <v>592857.14285714284</v>
       </c>
       <c r="E13" s="38">
         <f>E7*'Prix et marges'!$C$17+E8*'Prix et marges'!$D$17+E9*'Prix et marges'!$E$17+E10*'Prix et marges'!$F$17</f>
-        <v>648535.7142857142</v>
+        <v>1017857.1428571427</v>
       </c>
       <c r="F13" s="21"/>
       <c r="G13" s="22"/>
@@ -7796,15 +7795,15 @@
       </c>
       <c r="C14" s="38">
         <f>C7*'Prix et marges'!$C$34+C8*'Prix et marges'!$D$34+C9*'Prix et marges'!$E$34+C10*'Prix et marges'!$F$34+'Budget mensuel'!$B$40</f>
-        <v>149903.17857142858</v>
+        <v>172307.67857142855</v>
       </c>
       <c r="D14" s="38">
         <f>D7*'Prix et marges'!$C$34+D8*'Prix et marges'!$D$34+D9*'Prix et marges'!$E$34+D10*'Prix et marges'!$F$34</f>
-        <v>438760.85714285716</v>
+        <v>501892.8571428571</v>
       </c>
       <c r="E14" s="38">
         <f>E7*'Prix et marges'!$C$34+E8*'Prix et marges'!$D$34+E9*'Prix et marges'!$E$34+E10*'Prix et marges'!$F$34</f>
-        <v>752864.14285714296</v>
+        <v>855182.14285714272</v>
       </c>
       <c r="F14" s="21"/>
       <c r="G14" s="22"/>
@@ -7818,15 +7817,15 @@
       </c>
       <c r="C15" s="28">
         <f t="shared" ref="C15:E15" si="1">C13-C14</f>
-        <v>-27947.821428571449</v>
+        <v>28585.178571428551</v>
       </c>
       <c r="D15" s="28">
         <f t="shared" si="1"/>
-        <v>-70689.428571428638</v>
+        <v>90964.285714285739</v>
       </c>
       <c r="E15" s="28">
         <f t="shared" si="1"/>
-        <v>-104328.42857142875</v>
+        <v>162675</v>
       </c>
       <c r="F15" s="21"/>
       <c r="G15" s="22"/>
@@ -7840,15 +7839,15 @@
       </c>
       <c r="C16" s="31">
         <f t="shared" ref="C16:E16" si="2">IF(C13&gt;0,C15/C13,0)</f>
-        <v>-0.22916436049491198</v>
+        <v>0.14229066666666659</v>
       </c>
       <c r="D16" s="31">
         <f t="shared" si="2"/>
-        <v>-0.1920535610324085</v>
+        <v>0.15343373493975909</v>
       </c>
       <c r="E16" s="31">
         <f t="shared" si="2"/>
-        <v>-0.16086766892450055</v>
+        <v>0.15982105263157897</v>
       </c>
       <c r="F16" s="21"/>
       <c r="G16" s="22"/>
@@ -7938,15 +7937,15 @@
       </c>
       <c r="C20" s="28">
         <f t="shared" ref="C20:E20" si="4">C15-C19</f>
-        <v>-40619.821428571449</v>
+        <v>15913.178571428551</v>
       </c>
       <c r="D20" s="28">
         <f t="shared" si="4"/>
-        <v>-127775.57657142864</v>
+        <v>33878.137714285738</v>
       </c>
       <c r="E20" s="28">
         <f t="shared" si="4"/>
-        <v>-330934.57657142874</v>
+        <v>-63931.147999999986</v>
       </c>
       <c r="F20" s="21"/>
       <c r="G20" s="22"/>
@@ -7994,15 +7993,15 @@
       </c>
       <c r="C23" s="28">
         <f t="shared" ref="C23:E23" si="5">C20-C22</f>
-        <v>-43619.821428571449</v>
+        <v>12913.178571428551</v>
       </c>
       <c r="D23" s="28">
         <f t="shared" si="5"/>
-        <v>-132775.57657142862</v>
+        <v>28878.137714285738</v>
       </c>
       <c r="E23" s="28">
         <f t="shared" si="5"/>
-        <v>-340934.57657142874</v>
+        <v>-73931.147999999986</v>
       </c>
       <c r="F23" s="21"/>
       <c r="G23" s="22"/>
@@ -8016,15 +8015,15 @@
       </c>
       <c r="C24" s="28">
         <f>C23</f>
-        <v>-43619.821428571449</v>
+        <v>12913.178571428551</v>
       </c>
       <c r="D24" s="28">
         <f t="shared" ref="D24:E24" si="6">C24+D23</f>
-        <v>-176395.39800000007</v>
+        <v>41791.316285714289</v>
       </c>
       <c r="E24" s="28">
         <f t="shared" si="6"/>
-        <v>-517329.97457142884</v>
+        <v>-32139.831714285698</v>
       </c>
       <c r="F24" s="21"/>
       <c r="G24" s="22"/>
@@ -8038,15 +8037,15 @@
       </c>
       <c r="C25" s="39">
         <f t="shared" ref="C25:E25" si="7">IF(C11&gt;0,IF(C15&gt;0,C19/(C15/C11),0),0)</f>
-        <v>0</v>
+        <v>7.0929065387282426</v>
       </c>
       <c r="D25" s="39">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>30.123197060070662</v>
       </c>
       <c r="E25" s="39">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>117.01193442139234</v>
       </c>
       <c r="F25" s="21"/>
       <c r="G25" s="22"/>
@@ -8060,7 +8059,7 @@
       </c>
       <c r="C27" s="17">
         <f>MAX(0,-MIN(C24:E24))</f>
-        <v>517329.97457142884</v>
+        <v>32139.831714285698</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="13" x14ac:dyDescent="0.3">

</xml_diff>